<commit_message>
Komisyon karşılaştırma güncellendi (13.08.2026 16:28)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -632,9 +632,9 @@
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr"/>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>39.87TL / 797.68TL</t>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>39.87TL</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr"/>
@@ -642,11 +642,7 @@
       <c r="F4" s="12" t="inlineStr"/>
       <c r="G4" s="12" t="inlineStr"/>
       <c r="H4" s="12" t="inlineStr"/>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="I4" s="12" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
@@ -654,13 +650,13 @@
           <t>Düzenli EFT - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr"/>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>7,97TL</t>
         </is>
@@ -677,19 +673,19 @@
           <t>Düzenli EFT - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>199.41TL</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>199,41TL</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr"/>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>199,41 TL</t>
         </is>
@@ -736,7 +732,7 @@
           <t>199.41TL</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>797.68TL</t>
         </is>
@@ -752,7 +748,7 @@
           <t>398,83 TL</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>797,68 TL</t>
         </is>
@@ -823,13 +819,13 @@
           <t>Düzenli Havale - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>3.99TL</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr"/>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>3,99TL</t>
         </is>
@@ -846,19 +842,19 @@
           <t>Düzenli Havale - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>99.71TL</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr"/>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>99,71TL</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr"/>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>99,71 TL</t>
         </is>
@@ -882,7 +878,7 @@
           <t>3.99TL</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>19.94TL</t>
         </is>
@@ -895,8 +891,16 @@
       <c r="E15" s="12" t="inlineStr"/>
       <c r="F15" s="12" t="inlineStr"/>
       <c r="G15" s="12" t="inlineStr"/>
-      <c r="H15" s="12" t="inlineStr"/>
-      <c r="I15" s="12" t="inlineStr"/>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>13,92 TL / -</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>19,94 TL / -</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
@@ -922,20 +926,24 @@
       <c r="E16" s="12" t="inlineStr"/>
       <c r="F16" s="13" t="inlineStr">
         <is>
+          <t>199,42</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
           <t>398,84 TL</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>398,84 TL</t>
-        </is>
-      </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
           <t>27,62 TL / -</t>
         </is>
       </c>
-      <c r="I16" s="12" t="inlineStr"/>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>398,84 TL / -</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
@@ -945,17 +953,17 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>1900.00TL / 0.70% / 2950.00TL</t>
+          <t>1900.00TL / 0.70%</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>3676.20TL / 0.70% / 13457.15TL</t>
+          <t>3676.20TL / 0.70%</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>150TL / 245TL</t>
+          <t>150TL</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -970,7 +978,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>19,94 TL</t>
+          <t>39,88 TL</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
@@ -1018,7 +1026,7 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>380.95TL / 0.48% / 1523.81TL</t>
+          <t>380.95TL / 0.48%</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr"/>
@@ -1028,7 +1036,7 @@
       <c r="G21" s="12" t="inlineStr"/>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>200 TL / 0,4 / 1.200 TL</t>
+          <t>200 TL / 0,4</t>
         </is>
       </c>
       <c r="I21" s="12" t="inlineStr"/>
@@ -1039,7 +1047,7 @@
           <t>FAST - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
@@ -1049,7 +1057,11 @@
       <c r="E22" s="12" t="inlineStr"/>
       <c r="F22" s="12" t="inlineStr"/>
       <c r="G22" s="12" t="inlineStr"/>
-      <c r="H22" s="12" t="inlineStr"/>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>7,97 TL / -</t>
+        </is>
+      </c>
       <c r="I22" s="12" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
@@ -1058,7 +1070,7 @@
           <t>FAST - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
@@ -1068,7 +1080,11 @@
       <c r="E23" s="12" t="inlineStr"/>
       <c r="F23" s="12" t="inlineStr"/>
       <c r="G23" s="12" t="inlineStr"/>
-      <c r="H23" s="12" t="inlineStr"/>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>15,96 TL / -</t>
+        </is>
+      </c>
       <c r="I23" s="12" t="inlineStr"/>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -1096,13 +1112,13 @@
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr"/>
-      <c r="F26" s="13" t="inlineStr">
-        <is>
-          <t>26.990,48 TL</t>
-        </is>
-      </c>
+      <c r="F26" s="12" t="inlineStr"/>
       <c r="G26" s="12" t="inlineStr"/>
-      <c r="H26" s="12" t="inlineStr"/>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
       <c r="I26" s="12" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -1123,13 +1139,13 @@
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr"/>
-      <c r="F27" s="13" t="inlineStr">
-        <is>
-          <t>16.190,48 TL</t>
-        </is>
-      </c>
+      <c r="F27" s="12" t="inlineStr"/>
       <c r="G27" s="12" t="inlineStr"/>
-      <c r="H27" s="12" t="inlineStr"/>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
       <c r="I27" s="12" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
@@ -1150,13 +1166,13 @@
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr"/>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>21.595,24 TL</t>
-        </is>
-      </c>
+      <c r="F28" s="12" t="inlineStr"/>
       <c r="G28" s="12" t="inlineStr"/>
-      <c r="H28" s="12" t="inlineStr"/>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
       <c r="I28" s="12" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
@@ -1165,7 +1181,7 @@
           <t>Kasa Depozito - büyük</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>28570.00TL</t>
         </is>
@@ -1175,7 +1191,11 @@
       <c r="E29" s="12" t="inlineStr"/>
       <c r="F29" s="12" t="inlineStr"/>
       <c r="G29" s="12" t="inlineStr"/>
-      <c r="H29" s="12" t="inlineStr"/>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
       <c r="I29" s="12" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
@@ -1184,7 +1204,7 @@
           <t>Kasa Depozito - orta</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>23805.00TL</t>
         </is>
@@ -1194,7 +1214,11 @@
       <c r="E30" s="12" t="inlineStr"/>
       <c r="F30" s="12" t="inlineStr"/>
       <c r="G30" s="12" t="inlineStr"/>
-      <c r="H30" s="12" t="inlineStr"/>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
       <c r="I30" s="12" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
@@ -1203,7 +1227,7 @@
           <t>Kasa Depozito - küçük</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>20950.00TL</t>
         </is>
@@ -1213,7 +1237,11 @@
       <c r="E31" s="12" t="inlineStr"/>
       <c r="F31" s="12" t="inlineStr"/>
       <c r="G31" s="12" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr"/>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
       <c r="I31" s="12" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
@@ -1222,7 +1250,7 @@
           <t>Yıllık Kasa Ücreti - genel</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>1469.52TL</t>
         </is>
@@ -1232,11 +1260,7 @@
       <c r="E32" s="12" t="inlineStr"/>
       <c r="F32" s="12" t="inlineStr"/>
       <c r="G32" s="12" t="inlineStr"/>
-      <c r="H32" s="13" t="inlineStr">
-        <is>
-          <t>- / - / 28.333,33 TL</t>
-        </is>
-      </c>
+      <c r="H32" s="12" t="inlineStr"/>
       <c r="I32" s="12" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
@@ -1247,7 +1271,7 @@
       </c>
       <c r="B33" s="12" t="inlineStr"/>
       <c r="C33" s="12" t="inlineStr"/>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>9420TL</t>
         </is>
@@ -1255,11 +1279,7 @@
       <c r="E33" s="12" t="inlineStr"/>
       <c r="F33" s="12" t="inlineStr"/>
       <c r="G33" s="12" t="inlineStr"/>
-      <c r="H33" s="13" t="inlineStr">
-        <is>
-          <t>- / - / 28.333,33 TL</t>
-        </is>
-      </c>
+      <c r="H33" s="12" t="inlineStr"/>
       <c r="I33" s="12" t="inlineStr"/>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -1272,18 +1292,26 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 0-100</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>50.00TL</t>
+          <t>Altın Transfer</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>100.00TL</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr"/>
-      <c r="D36" s="12" t="inlineStr"/>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>415TL</t>
+        </is>
+      </c>
       <c r="E36" s="12" t="inlineStr"/>
-      <c r="F36" s="12" t="inlineStr"/>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>0.00018</t>
+        </is>
+      </c>
       <c r="G36" s="12" t="inlineStr"/>
       <c r="H36" s="12" t="inlineStr"/>
       <c r="I36" s="12" t="inlineStr"/>
@@ -1291,767 +1319,719 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>637.00TL</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
+          <t>Altın Transfer - 1-10gr</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr"/>
+      <c r="C37" s="12" t="inlineStr"/>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>415TL</t>
+          <t>57,5TL</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr"/>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>60 TL</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr"/>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>- / 10</t>
-        </is>
-      </c>
+      <c r="H37" s="12" t="inlineStr"/>
       <c r="I37" s="12" t="inlineStr"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 1-10gr</t>
+          <t>Altın Transfer - 11-100gr</t>
         </is>
       </c>
       <c r="B38" s="12" t="inlineStr"/>
       <c r="C38" s="12" t="inlineStr"/>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>57,5TL</t>
+          <t>115TL</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr"/>
       <c r="F38" s="13" t="inlineStr">
         <is>
-          <t>60 TL</t>
+          <t>120 TL</t>
         </is>
       </c>
       <c r="G38" s="12" t="inlineStr"/>
       <c r="H38" s="12" t="inlineStr"/>
       <c r="I38" s="12" t="inlineStr"/>
     </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>Altın Transfer - 11-100gr</t>
-        </is>
-      </c>
-      <c r="B39" s="12" t="inlineStr"/>
-      <c r="C39" s="12" t="inlineStr"/>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>115TL</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="inlineStr"/>
-      <c r="F39" s="13" t="inlineStr">
-        <is>
-          <t>120 TL</t>
-        </is>
-      </c>
-      <c r="G39" s="12" t="inlineStr"/>
-      <c r="H39" s="12" t="inlineStr"/>
-      <c r="I39" s="12" t="inlineStr"/>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>95TL</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr"/>
-      <c r="F42" s="13" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr"/>
+      <c r="F41" s="13" t="inlineStr">
         <is>
           <t>65 TL</t>
         </is>
       </c>
-      <c r="G42" s="13" t="inlineStr">
+      <c r="G41" s="12" t="inlineStr">
         <is>
           <t>95,24 TL</t>
         </is>
       </c>
-      <c r="H42" s="13" t="inlineStr">
-        <is>
-          <t>94,29 TL / -</t>
-        </is>
-      </c>
-      <c r="I42" s="12" t="inlineStr"/>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>339 TL / -</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri - Kart</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="11" t="inlineStr">
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>5.00TL / 3.50%</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>0.00TL / 50.00TL</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>0TL / 2,86TL</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr"/>
-      <c r="F45" s="13" t="inlineStr">
-        <is>
-          <t>0.5 TL / 55 TL</t>
-        </is>
-      </c>
-      <c r="G45" s="13" t="inlineStr">
-        <is>
-          <t>0.5 TL / 55 TL</t>
-        </is>
-      </c>
-      <c r="H45" s="13" t="inlineStr">
-        <is>
-          <t>0,63 TL / - / 45 TL</t>
-        </is>
-      </c>
-      <c r="I45" s="12" t="inlineStr"/>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>0.00TL</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>0TL</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr"/>
+      <c r="F44" s="13" t="inlineStr">
+        <is>
+          <t>0.5 TL</t>
+        </is>
+      </c>
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t>0.5 TL</t>
+        </is>
+      </c>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>0,63 TL / -</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="11" t="inlineStr">
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>3.50TL / 3.50%</t>
         </is>
       </c>
-      <c r="C48" s="12" t="inlineStr"/>
-      <c r="D48" s="13" t="inlineStr">
-        <is>
-          <t>0TL / 3,1%</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr"/>
-      <c r="F48" s="13" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr"/>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>0TL</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr"/>
+      <c r="F47" s="13" t="inlineStr">
         <is>
           <t>2 TL / 3,5%</t>
         </is>
       </c>
-      <c r="G48" s="12" t="inlineStr"/>
-      <c r="H48" s="12" t="inlineStr"/>
-      <c r="I48" s="12" t="inlineStr">
-        <is>
-          <t>3 TL / - / 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="G47" s="12" t="inlineStr"/>
+      <c r="H47" s="12" t="inlineStr"/>
+      <c r="I47" s="12" t="inlineStr">
+        <is>
+          <t>3 TL / -</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="10" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B50" s="13" t="inlineStr">
         <is>
           <t>275.00TL</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr"/>
-      <c r="D51" s="13" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr"/>
+      <c r="D50" s="13" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="E51" s="12" t="inlineStr"/>
-      <c r="F51" s="13" t="inlineStr">
+      <c r="E50" s="12" t="inlineStr"/>
+      <c r="F50" s="13" t="inlineStr">
         <is>
           <t>275 TL</t>
         </is>
       </c>
-      <c r="G51" s="12" t="inlineStr"/>
-      <c r="H51" s="13" t="inlineStr">
-        <is>
-          <t>275 TL / -</t>
-        </is>
-      </c>
-      <c r="I51" s="12" t="inlineStr"/>
-    </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="G50" s="12" t="inlineStr"/>
+      <c r="H50" s="12" t="inlineStr"/>
+      <c r="I50" s="12" t="inlineStr"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
-      <c r="B54" s="12" t="inlineStr"/>
-      <c r="C54" s="12" t="inlineStr"/>
-      <c r="D54" s="13" t="inlineStr">
-        <is>
-          <t>26TL / 30TL</t>
-        </is>
-      </c>
-      <c r="E54" s="12" t="inlineStr"/>
-      <c r="F54" s="13" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr"/>
+      <c r="C53" s="12" t="inlineStr"/>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>26TL</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="inlineStr"/>
+      <c r="F53" s="13" t="inlineStr">
         <is>
           <t>38,10 TL</t>
         </is>
       </c>
-      <c r="G54" s="12" t="inlineStr"/>
-      <c r="H54" s="12" t="inlineStr"/>
-      <c r="I54" s="12" t="inlineStr"/>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="10" t="inlineStr">
+      <c r="G53" s="12" t="inlineStr"/>
+      <c r="H53" s="12" t="inlineStr"/>
+      <c r="I53" s="12" t="inlineStr"/>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="11" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr"/>
-      <c r="C57" s="12" t="inlineStr"/>
-      <c r="D57" s="12" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr"/>
+      <c r="C56" s="12" t="inlineStr"/>
+      <c r="D56" s="12" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E57" s="12" t="inlineStr"/>
-      <c r="F57" s="12" t="inlineStr"/>
-      <c r="G57" s="12" t="inlineStr"/>
-      <c r="H57" s="12" t="inlineStr"/>
-      <c r="I57" s="12" t="inlineStr"/>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
+      <c r="E56" s="12" t="inlineStr"/>
+      <c r="F56" s="12" t="inlineStr"/>
+      <c r="G56" s="12" t="inlineStr"/>
+      <c r="H56" s="12" t="inlineStr"/>
+      <c r="I56" s="12" t="inlineStr"/>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t>Telefon Ödemeleri Aracılık</t>
         </is>
       </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>Telefon Ödemeleri</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="inlineStr"/>
+      <c r="C59" s="12" t="inlineStr"/>
+      <c r="D59" s="12" t="inlineStr"/>
+      <c r="E59" s="12" t="inlineStr"/>
+      <c r="F59" s="12" t="inlineStr">
+        <is>
+          <t>1 %</t>
+        </is>
+      </c>
+      <c r="G59" s="12" t="inlineStr"/>
+      <c r="H59" s="12" t="inlineStr"/>
+      <c r="I59" s="12" t="inlineStr"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>Telefon Ödemeleri</t>
+          <t>Telefon - 399000+ TRY</t>
         </is>
       </c>
       <c r="B60" s="12" t="inlineStr"/>
       <c r="C60" s="12" t="inlineStr"/>
       <c r="D60" s="12" t="inlineStr"/>
       <c r="E60" s="12" t="inlineStr"/>
-      <c r="F60" s="13" t="inlineStr">
-        <is>
-          <t>1 %</t>
+      <c r="F60" s="12" t="inlineStr">
+        <is>
+          <t>99,71 TL</t>
         </is>
       </c>
       <c r="G60" s="12" t="inlineStr"/>
-      <c r="H60" s="13" t="inlineStr">
-        <is>
-          <t>- / - / 50 USD</t>
-        </is>
-      </c>
+      <c r="H60" s="12" t="inlineStr"/>
       <c r="I60" s="12" t="inlineStr"/>
     </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="11" t="inlineStr">
-        <is>
-          <t>Telefon - 399000+ TRY</t>
-        </is>
-      </c>
-      <c r="B61" s="12" t="inlineStr"/>
-      <c r="C61" s="12" t="inlineStr"/>
-      <c r="D61" s="12" t="inlineStr"/>
-      <c r="E61" s="12" t="inlineStr"/>
-      <c r="F61" s="12" t="inlineStr">
-        <is>
-          <t>99,71 TL</t>
-        </is>
-      </c>
-      <c r="G61" s="12" t="inlineStr"/>
-      <c r="H61" s="12" t="inlineStr"/>
-      <c r="I61" s="12" t="inlineStr"/>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="10" t="inlineStr">
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="10" t="inlineStr">
         <is>
           <t>Vergi Tahsilat Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="11" t="inlineStr">
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>Vergi Tahsilat</t>
         </is>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>0.00TL / 0.00%</t>
-        </is>
-      </c>
-      <c r="C64" s="12" t="inlineStr"/>
-      <c r="D64" s="12" t="inlineStr"/>
-      <c r="E64" s="12" t="inlineStr"/>
-      <c r="F64" s="12" t="inlineStr"/>
-      <c r="G64" s="12" t="inlineStr"/>
-      <c r="H64" s="13" t="inlineStr">
-        <is>
-          <t>- / - / 100 TL</t>
-        </is>
-      </c>
-      <c r="I64" s="12" t="inlineStr"/>
-    </row>
-    <row r="66" ht="16" customHeight="1">
-      <c r="A66" s="10" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr"/>
+      <c r="C63" s="12" t="inlineStr"/>
+      <c r="D63" s="12" t="inlineStr"/>
+      <c r="E63" s="12" t="inlineStr"/>
+      <c r="F63" s="12" t="inlineStr"/>
+      <c r="G63" s="12" t="inlineStr"/>
+      <c r="H63" s="12" t="inlineStr"/>
+      <c r="I63" s="12" t="inlineStr"/>
+    </row>
+    <row r="65" ht="16" customHeight="1">
+      <c r="A65" s="10" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="11" t="inlineStr">
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
         </is>
       </c>
-      <c r="B67" s="13" t="inlineStr">
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>287.62TL</t>
         </is>
       </c>
-      <c r="C67" s="12" t="inlineStr"/>
-      <c r="D67" s="12" t="inlineStr"/>
-      <c r="E67" s="12" t="inlineStr"/>
-      <c r="F67" s="12" t="inlineStr"/>
-      <c r="G67" s="12" t="inlineStr"/>
-      <c r="H67" s="13" t="inlineStr">
-        <is>
-          <t>- / - / 18,9 TL</t>
-        </is>
-      </c>
-      <c r="I67" s="12" t="inlineStr"/>
-    </row>
-    <row r="69" ht="16" customHeight="1">
-      <c r="A69" s="10" t="inlineStr">
+      <c r="C66" s="12" t="inlineStr"/>
+      <c r="D66" s="12" t="inlineStr"/>
+      <c r="E66" s="12" t="inlineStr"/>
+      <c r="F66" s="12" t="inlineStr"/>
+      <c r="G66" s="12" t="inlineStr"/>
+      <c r="H66" s="12" t="inlineStr"/>
+      <c r="I66" s="12" t="inlineStr"/>
+    </row>
+    <row r="68" ht="16" customHeight="1">
+      <c r="A68" s="10" t="inlineStr">
         <is>
           <t>Mevduat Araştırma</t>
         </is>
       </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>Referans Mektubu -</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>4000.00TL</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="inlineStr"/>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>770TL</t>
+        </is>
+      </c>
+      <c r="E69" s="12" t="inlineStr"/>
+      <c r="F69" s="12" t="inlineStr"/>
+      <c r="G69" s="12" t="inlineStr"/>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>50 TL / -</t>
+        </is>
+      </c>
+      <c r="I69" s="12" t="inlineStr"/>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>Referans Mektubu -</t>
-        </is>
-      </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>2.00%</t>
-        </is>
-      </c>
+          <t>Hesap Özeti Verilmesi -</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr"/>
       <c r="C70" s="12" t="inlineStr"/>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>770TL / 0.1%</t>
+          <t>190TL</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr"/>
       <c r="F70" s="13" t="inlineStr">
         <is>
-          <t>5000 TL</t>
+          <t>12 TL</t>
         </is>
       </c>
       <c r="G70" s="12" t="inlineStr"/>
-      <c r="H70" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H70" s="12" t="inlineStr"/>
       <c r="I70" s="12" t="inlineStr"/>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="11" t="inlineStr">
         <is>
-          <t>Hesap Özeti Verilmesi -</t>
+          <t>Borcu Yoktur Yazısı</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr"/>
       <c r="C71" s="12" t="inlineStr"/>
-      <c r="D71" s="13" t="inlineStr">
-        <is>
-          <t>190TL</t>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>390TL</t>
         </is>
       </c>
       <c r="E71" s="12" t="inlineStr"/>
-      <c r="F71" s="13" t="inlineStr">
-        <is>
-          <t>12 TL</t>
-        </is>
-      </c>
+      <c r="F71" s="12" t="inlineStr"/>
       <c r="G71" s="12" t="inlineStr"/>
-      <c r="H71" s="13" t="inlineStr">
-        <is>
-          <t>- / - / 45 TL</t>
-        </is>
-      </c>
+      <c r="H71" s="12" t="inlineStr"/>
       <c r="I71" s="12" t="inlineStr"/>
     </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="11" t="inlineStr">
-        <is>
-          <t>Borcu Yoktur Yazısı</t>
-        </is>
-      </c>
-      <c r="B72" s="12" t="inlineStr"/>
-      <c r="C72" s="12" t="inlineStr"/>
-      <c r="D72" s="12" t="inlineStr">
-        <is>
-          <t>390TL</t>
-        </is>
-      </c>
-      <c r="E72" s="12" t="inlineStr"/>
-      <c r="F72" s="12" t="inlineStr"/>
-      <c r="G72" s="12" t="inlineStr"/>
-      <c r="H72" s="12" t="inlineStr"/>
-      <c r="I72" s="12" t="inlineStr"/>
-    </row>
-    <row r="74" ht="16" customHeight="1">
-      <c r="A74" s="10" t="inlineStr">
+    <row r="73" ht="16" customHeight="1">
+      <c r="A73" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="11" t="inlineStr">
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="11" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr"/>
-      <c r="C75" s="12" t="inlineStr"/>
-      <c r="D75" s="12" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr"/>
+      <c r="C74" s="12" t="inlineStr"/>
+      <c r="D74" s="13" t="inlineStr">
         <is>
           <t>0.41TL</t>
         </is>
       </c>
-      <c r="E75" s="12" t="inlineStr"/>
-      <c r="F75" s="12" t="inlineStr"/>
-      <c r="G75" s="12" t="inlineStr"/>
-      <c r="H75" s="12" t="inlineStr"/>
-      <c r="I75" s="12" t="inlineStr"/>
-    </row>
-    <row r="77" ht="16" customHeight="1">
-      <c r="A77" s="10" t="inlineStr">
+      <c r="E74" s="12" t="inlineStr"/>
+      <c r="F74" s="12" t="inlineStr"/>
+      <c r="G74" s="12" t="inlineStr"/>
+      <c r="H74" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
+      <c r="I74" s="12" t="inlineStr"/>
+    </row>
+    <row r="76" ht="16" customHeight="1">
+      <c r="A76" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="11" t="inlineStr">
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="11" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
-      <c r="B78" s="12" t="inlineStr"/>
-      <c r="C78" s="12" t="inlineStr"/>
-      <c r="D78" s="13" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr"/>
+      <c r="C77" s="12" t="inlineStr"/>
+      <c r="D77" s="13" t="inlineStr">
         <is>
           <t>0.45EUR</t>
         </is>
       </c>
-      <c r="E78" s="12" t="inlineStr"/>
-      <c r="F78" s="13" t="inlineStr">
+      <c r="E77" s="12" t="inlineStr"/>
+      <c r="F77" s="13" t="inlineStr">
         <is>
           <t>0.27 TL</t>
         </is>
       </c>
-      <c r="G78" s="12" t="inlineStr"/>
-      <c r="H78" s="13" t="inlineStr">
-        <is>
-          <t>- / - / 0,27 TL</t>
-        </is>
-      </c>
-      <c r="I78" s="12" t="inlineStr"/>
-    </row>
-    <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="10" t="inlineStr">
+      <c r="G77" s="12" t="inlineStr"/>
+      <c r="H77" s="12" t="inlineStr"/>
+      <c r="I77" s="12" t="inlineStr"/>
+    </row>
+    <row r="79" ht="16" customHeight="1">
+      <c r="A79" s="10" t="inlineStr">
         <is>
           <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
         </is>
       </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>Çek Düzenleme -</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>9.52TL / 0.10%</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr"/>
+      <c r="D80" s="13" t="inlineStr">
+        <is>
+          <t>290TL / 1.10%</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="inlineStr"/>
+      <c r="F80" s="13" t="inlineStr">
+        <is>
+          <t>761,90 TL</t>
+        </is>
+      </c>
+      <c r="G80" s="12" t="inlineStr"/>
+      <c r="H80" s="13" t="inlineStr">
+        <is>
+          <t>104,76 TL / -</t>
+        </is>
+      </c>
+      <c r="I80" s="12" t="inlineStr"/>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="11" t="inlineStr">
         <is>
-          <t>Çek Düzenleme -</t>
-        </is>
-      </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>9.52TL / 0.10% / 9523.81TL</t>
-        </is>
-      </c>
+          <t>Çek Defteri (Yaprak Başı) -</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="inlineStr"/>
       <c r="C81" s="12" t="inlineStr"/>
-      <c r="D81" s="13" t="inlineStr">
-        <is>
-          <t>290TL / 1.10%</t>
-        </is>
-      </c>
+      <c r="D81" s="12" t="inlineStr"/>
       <c r="E81" s="12" t="inlineStr"/>
-      <c r="F81" s="13" t="inlineStr">
-        <is>
-          <t>761,90 TL / 7.619,05 TL / 0.5 %</t>
+      <c r="F81" s="12" t="inlineStr">
+        <is>
+          <t>2.380,95 TL</t>
         </is>
       </c>
       <c r="G81" s="12" t="inlineStr"/>
-      <c r="H81" s="13" t="inlineStr">
-        <is>
-          <t>104,76 TL / -</t>
-        </is>
-      </c>
+      <c r="H81" s="12" t="inlineStr"/>
       <c r="I81" s="12" t="inlineStr"/>
     </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>Çek Defteri (Yaprak Başı) -</t>
-        </is>
-      </c>
-      <c r="B82" s="12" t="inlineStr"/>
-      <c r="C82" s="12" t="inlineStr"/>
-      <c r="D82" s="12" t="inlineStr"/>
-      <c r="E82" s="12" t="inlineStr"/>
-      <c r="F82" s="12" t="inlineStr">
-        <is>
-          <t>2.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G82" s="12" t="inlineStr"/>
-      <c r="H82" s="12" t="inlineStr"/>
-      <c r="I82" s="12" t="inlineStr"/>
-    </row>
-    <row r="84" ht="16" customHeight="1">
-      <c r="A84" s="10" t="inlineStr">
+    <row r="83" ht="16" customHeight="1">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>Çek İade Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="11" t="inlineStr">
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="11" t="inlineStr">
         <is>
           <t>Çek İade Ücreti</t>
         </is>
       </c>
-      <c r="B85" s="13" t="inlineStr">
+      <c r="B84" s="13" t="inlineStr">
         <is>
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="C85" s="12" t="inlineStr"/>
-      <c r="D85" s="13" t="inlineStr">
+      <c r="C84" s="12" t="inlineStr"/>
+      <c r="D84" s="13" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E85" s="12" t="inlineStr"/>
-      <c r="F85" s="13" t="inlineStr">
+      <c r="E84" s="12" t="inlineStr"/>
+      <c r="F84" s="13" t="inlineStr">
         <is>
           <t>380,95 TL</t>
         </is>
       </c>
-      <c r="G85" s="12" t="inlineStr"/>
-      <c r="H85" s="13" t="inlineStr">
+      <c r="G84" s="12" t="inlineStr"/>
+      <c r="H84" s="13" t="inlineStr">
         <is>
           <t>123,81 TL / -</t>
         </is>
       </c>
-      <c r="I85" s="12" t="inlineStr"/>
-    </row>
-    <row r="87" ht="16" customHeight="1">
-      <c r="A87" s="10" t="inlineStr">
+      <c r="I84" s="12" t="inlineStr"/>
+    </row>
+    <row r="86" ht="16" customHeight="1">
+      <c r="A86" s="10" t="inlineStr">
         <is>
           <t>Çek Tahsilat Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="11" t="inlineStr">
+        <is>
+          <t>Çek Tahsilat</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>45USD</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>590.48TL / 0.77%</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr"/>
+      <c r="E87" s="13" t="inlineStr">
+        <is>
+          <t>1.70%</t>
+        </is>
+      </c>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>714,29 TL</t>
+        </is>
+      </c>
+      <c r="G87" s="12" t="inlineStr"/>
+      <c r="H87" s="13" t="inlineStr">
+        <is>
+          <t>260 TL / -</t>
+        </is>
+      </c>
+      <c r="I87" s="13" t="inlineStr">
+        <is>
+          <t>- / -</t>
         </is>
       </c>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>Çek Tahsilat</t>
+          <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>45USD / 0.15%</t>
-        </is>
-      </c>
-      <c r="C88" s="13" t="inlineStr">
-        <is>
-          <t>590.48TL / 0.77% / 3904.77TL</t>
-        </is>
-      </c>
-      <c r="D88" s="12" t="inlineStr"/>
+          <t>257.15TL</t>
+        </is>
+      </c>
+      <c r="C88" s="12" t="inlineStr"/>
+      <c r="D88" s="13" t="inlineStr">
+        <is>
+          <t>2940TL / 1%</t>
+        </is>
+      </c>
       <c r="E88" s="13" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>390TL / 0.2%</t>
         </is>
       </c>
       <c r="F88" s="13" t="inlineStr">
         <is>
-          <t>714,29 TL</t>
-        </is>
-      </c>
-      <c r="G88" s="12" t="inlineStr"/>
-      <c r="H88" s="13" t="inlineStr">
-        <is>
-          <t>25.000 TL / -</t>
-        </is>
-      </c>
-      <c r="I88" s="13" t="inlineStr">
-        <is>
-          <t>576,19 TL / 0,6 / 3.930,48 TL / -</t>
-        </is>
-      </c>
+          <t>1.666,67 TL</t>
+        </is>
+      </c>
+      <c r="G88" s="13" t="inlineStr">
+        <is>
+          <t>585,71 TL</t>
+        </is>
+      </c>
+      <c r="H88" s="12" t="inlineStr"/>
+      <c r="I88" s="12" t="inlineStr"/>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="11" t="inlineStr">
         <is>
-          <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
+          <t>Diğer Banka Çeki -</t>
         </is>
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>257.15TL</t>
+          <t>390.48TL</t>
         </is>
       </c>
       <c r="C89" s="12" t="inlineStr"/>
       <c r="D89" s="13" t="inlineStr">
         <is>
-          <t>2940TL / 1% / 29450TL</t>
-        </is>
-      </c>
-      <c r="E89" s="13" t="inlineStr">
-        <is>
-          <t>390TL / 0.2% / 1950TL</t>
-        </is>
-      </c>
-      <c r="F89" s="13" t="inlineStr">
-        <is>
-          <t>1.666,67 TL / 9.904,77 TL / 0.5 %</t>
-        </is>
-      </c>
-      <c r="G89" s="13" t="inlineStr">
-        <is>
-          <t>585,71 TL / 4.000 TL / 0.8 %</t>
-        </is>
-      </c>
-      <c r="H89" s="13" t="inlineStr">
-        <is>
-          <t>260 TL / -</t>
-        </is>
-      </c>
-      <c r="I89" s="13" t="inlineStr">
-        <is>
-          <t>576,19 TL / 0,6 / 3.930,48 TL / -</t>
+          <t>350TL</t>
+        </is>
+      </c>
+      <c r="E89" s="12" t="inlineStr"/>
+      <c r="F89" s="12" t="inlineStr"/>
+      <c r="G89" s="12" t="inlineStr"/>
+      <c r="H89" s="12" t="inlineStr"/>
+      <c r="I89" s="12" t="inlineStr">
+        <is>
+          <t>576,19 TL / 0,6</t>
         </is>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>Diğer Banka Çeki -</t>
-        </is>
-      </c>
-      <c r="B90" s="13" t="inlineStr">
-        <is>
-          <t>390.48TL</t>
-        </is>
-      </c>
+          <t>Aynı Banka Çeki -</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr"/>
       <c r="C90" s="12" t="inlineStr"/>
-      <c r="D90" s="13" t="inlineStr">
-        <is>
-          <t>350TL</t>
-        </is>
-      </c>
+      <c r="D90" s="12" t="inlineStr"/>
       <c r="E90" s="12" t="inlineStr"/>
       <c r="F90" s="12" t="inlineStr"/>
       <c r="G90" s="12" t="inlineStr"/>
       <c r="H90" s="12" t="inlineStr"/>
-      <c r="I90" s="12" t="inlineStr"/>
+      <c r="I90" s="12" t="inlineStr">
+        <is>
+          <t>427,62 TL / -</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="10" t="inlineStr">
@@ -2220,81 +2200,96 @@
       </c>
       <c r="I103" s="12" t="inlineStr"/>
     </row>
-    <row r="105" ht="16" customHeight="1">
-      <c r="A105" s="10" t="inlineStr">
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="11" t="inlineStr">
+        <is>
+          <t>Aynı Banka Senet Tahsili -</t>
+        </is>
+      </c>
+      <c r="B104" s="12" t="inlineStr"/>
+      <c r="C104" s="12" t="inlineStr"/>
+      <c r="D104" s="12" t="inlineStr"/>
+      <c r="E104" s="12" t="inlineStr"/>
+      <c r="F104" s="12" t="inlineStr"/>
+      <c r="G104" s="12" t="inlineStr"/>
+      <c r="H104" s="12" t="inlineStr">
+        <is>
+          <t>600 TL / -</t>
+        </is>
+      </c>
+      <c r="I104" s="12" t="inlineStr"/>
+    </row>
+    <row r="106" ht="16" customHeight="1">
+      <c r="A106" s="10" t="inlineStr">
         <is>
           <t>HGS</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="20" customHeight="1">
-      <c r="A106" s="11" t="inlineStr">
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="11" t="inlineStr">
         <is>
           <t>HGS Kart Ücreti</t>
         </is>
       </c>
-      <c r="B106" s="13" t="inlineStr">
+      <c r="B107" s="13" t="inlineStr">
         <is>
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="C106" s="12" t="inlineStr"/>
-      <c r="D106" s="13" t="inlineStr">
+      <c r="C107" s="12" t="inlineStr"/>
+      <c r="D107" s="13" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="E106" s="12" t="inlineStr"/>
-      <c r="F106" s="13" t="inlineStr">
+      <c r="E107" s="12" t="inlineStr"/>
+      <c r="F107" s="13" t="inlineStr">
         <is>
           <t>500 TL</t>
         </is>
       </c>
-      <c r="G106" s="12" t="inlineStr"/>
-      <c r="H106" s="13" t="inlineStr">
-        <is>
-          <t>550 TL / -</t>
-        </is>
-      </c>
-      <c r="I106" s="12" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="14" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 13.08.2026 16:12</t>
+      <c r="G107" s="12" t="inlineStr"/>
+      <c r="H107" s="12" t="inlineStr"/>
+      <c r="I107" s="12" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 13.08.2026 16:28</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A65:I65"/>
     <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A84:I84"/>
-    <mergeCell ref="A66:I66"/>
+    <mergeCell ref="A46:I46"/>
     <mergeCell ref="H1:I1"/>
-    <mergeCell ref="A80:I80"/>
-    <mergeCell ref="A56:I56"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A74:I74"/>
-    <mergeCell ref="A105:I105"/>
-    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A55:I55"/>
     <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A86:I86"/>
     <mergeCell ref="A95:I95"/>
-    <mergeCell ref="A47:I47"/>
-    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A76:I76"/>
+    <mergeCell ref="A106:I106"/>
     <mergeCell ref="A35:I35"/>
     <mergeCell ref="B1:C1"/>
+    <mergeCell ref="A62:I62"/>
     <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A63:I63"/>
-    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A68:I68"/>
     <mergeCell ref="A102:I102"/>
-    <mergeCell ref="A77:I77"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A58:I58"/>
+    <mergeCell ref="A83:I83"/>
     <mergeCell ref="A92:I92"/>
-    <mergeCell ref="A59:I59"/>
     <mergeCell ref="A98:I98"/>
-    <mergeCell ref="A69:I69"/>
-    <mergeCell ref="A87:I87"/>
+    <mergeCell ref="A73:I73"/>
+    <mergeCell ref="A49:I49"/>
+    <mergeCell ref="A79:I79"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (13.08.2026 16:50)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -1505,19 +1505,19 @@
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>275.00TL</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr"/>
-      <c r="D50" s="13" t="inlineStr">
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr"/>
-      <c r="F50" s="13" t="inlineStr">
+      <c r="F50" s="12" t="inlineStr">
         <is>
           <t>275 TL</t>
         </is>
@@ -2256,7 +2256,7 @@
     <row r="109">
       <c r="A109" s="14" t="inlineStr">
         <is>
-          <t>Son güncelleme: 13.08.2026 16:28</t>
+          <t>Son güncelleme: 13.08.2026 16:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (13.08.2026 17:05)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -62,7 +62,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -97,12 +97,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00003087"/>
         <bgColor rgb="00003087"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,7 +164,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -878,7 +872,7 @@
           <t>3.99TL</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>19.94TL</t>
         </is>
@@ -893,12 +887,12 @@
       <c r="G15" s="12" t="inlineStr"/>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>13,92 TL / -</t>
-        </is>
-      </c>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>19,94 TL / -</t>
+          <t>13,92 TL</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>19,94 TL</t>
         </is>
       </c>
     </row>
@@ -913,7 +907,7 @@
           <t>99.71TL</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>398.84TL</t>
         </is>
@@ -929,19 +923,19 @@
           <t>199,42</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>398,84 TL</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>27,62 TL / -</t>
-        </is>
-      </c>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>398,84 TL / -</t>
+          <t>27,62 TL</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>398,84 TL</t>
         </is>
       </c>
     </row>
@@ -983,7 +977,7 @@
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>13,33 TL / -</t>
+          <t>13,33 TL</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr"/>
@@ -1047,7 +1041,7 @@
           <t>FAST - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
@@ -1057,9 +1051,9 @@
       <c r="E22" s="12" t="inlineStr"/>
       <c r="F22" s="12" t="inlineStr"/>
       <c r="G22" s="12" t="inlineStr"/>
-      <c r="H22" s="13" t="inlineStr">
-        <is>
-          <t>7,97 TL / -</t>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>7,97 TL</t>
         </is>
       </c>
       <c r="I22" s="12" t="inlineStr"/>
@@ -1070,7 +1064,7 @@
           <t>FAST - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
@@ -1080,9 +1074,9 @@
       <c r="E23" s="12" t="inlineStr"/>
       <c r="F23" s="12" t="inlineStr"/>
       <c r="G23" s="12" t="inlineStr"/>
-      <c r="H23" s="13" t="inlineStr">
-        <is>
-          <t>15,96 TL / -</t>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>15,96 TL</t>
         </is>
       </c>
       <c r="I23" s="12" t="inlineStr"/>
@@ -1114,11 +1108,7 @@
       <c r="E26" s="12" t="inlineStr"/>
       <c r="F26" s="12" t="inlineStr"/>
       <c r="G26" s="12" t="inlineStr"/>
-      <c r="H26" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H26" s="12" t="inlineStr"/>
       <c r="I26" s="12" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -1141,11 +1131,7 @@
       <c r="E27" s="12" t="inlineStr"/>
       <c r="F27" s="12" t="inlineStr"/>
       <c r="G27" s="12" t="inlineStr"/>
-      <c r="H27" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H27" s="12" t="inlineStr"/>
       <c r="I27" s="12" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
@@ -1168,11 +1154,7 @@
       <c r="E28" s="12" t="inlineStr"/>
       <c r="F28" s="12" t="inlineStr"/>
       <c r="G28" s="12" t="inlineStr"/>
-      <c r="H28" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H28" s="12" t="inlineStr"/>
       <c r="I28" s="12" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
@@ -1181,7 +1163,7 @@
           <t>Kasa Depozito - büyük</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>28570.00TL</t>
         </is>
@@ -1191,11 +1173,7 @@
       <c r="E29" s="12" t="inlineStr"/>
       <c r="F29" s="12" t="inlineStr"/>
       <c r="G29" s="12" t="inlineStr"/>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H29" s="12" t="inlineStr"/>
       <c r="I29" s="12" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
@@ -1204,7 +1182,7 @@
           <t>Kasa Depozito - orta</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>23805.00TL</t>
         </is>
@@ -1214,11 +1192,7 @@
       <c r="E30" s="12" t="inlineStr"/>
       <c r="F30" s="12" t="inlineStr"/>
       <c r="G30" s="12" t="inlineStr"/>
-      <c r="H30" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H30" s="12" t="inlineStr"/>
       <c r="I30" s="12" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
@@ -1227,7 +1201,7 @@
           <t>Kasa Depozito - küçük</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>20950.00TL</t>
         </is>
@@ -1237,11 +1211,7 @@
       <c r="E31" s="12" t="inlineStr"/>
       <c r="F31" s="12" t="inlineStr"/>
       <c r="G31" s="12" t="inlineStr"/>
-      <c r="H31" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H31" s="12" t="inlineStr"/>
       <c r="I31" s="12" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
@@ -1403,7 +1373,7 @@
       </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
-          <t>339 TL / -</t>
+          <t>339 TL</t>
         </is>
       </c>
       <c r="I41" s="12" t="inlineStr"/>
@@ -1449,7 +1419,7 @@
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>0,63 TL / -</t>
+          <t>0,63 TL</t>
         </is>
       </c>
       <c r="I44" s="12" t="inlineStr"/>
@@ -1488,7 +1458,7 @@
       <c r="H47" s="12" t="inlineStr"/>
       <c r="I47" s="12" t="inlineStr">
         <is>
-          <t>3 TL / -</t>
+          <t>3 TL</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1674,7 @@
       <c r="G69" s="12" t="inlineStr"/>
       <c r="H69" s="13" t="inlineStr">
         <is>
-          <t>50 TL / -</t>
+          <t>50 TL</t>
         </is>
       </c>
       <c r="I69" s="12" t="inlineStr"/>
@@ -1766,7 +1736,7 @@
       </c>
       <c r="B74" s="12" t="inlineStr"/>
       <c r="C74" s="12" t="inlineStr"/>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="D74" s="12" t="inlineStr">
         <is>
           <t>0.41TL</t>
         </is>
@@ -1774,11 +1744,7 @@
       <c r="E74" s="12" t="inlineStr"/>
       <c r="F74" s="12" t="inlineStr"/>
       <c r="G74" s="12" t="inlineStr"/>
-      <c r="H74" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+      <c r="H74" s="12" t="inlineStr"/>
       <c r="I74" s="12" t="inlineStr"/>
     </row>
     <row r="76" ht="16" customHeight="1">
@@ -1844,7 +1810,7 @@
       <c r="G80" s="12" t="inlineStr"/>
       <c r="H80" s="13" t="inlineStr">
         <is>
-          <t>104,76 TL / -</t>
+          <t>104,76 TL</t>
         </is>
       </c>
       <c r="I80" s="12" t="inlineStr"/>
@@ -1901,7 +1867,7 @@
       <c r="G84" s="12" t="inlineStr"/>
       <c r="H84" s="13" t="inlineStr">
         <is>
-          <t>123,81 TL / -</t>
+          <t>123,81 TL</t>
         </is>
       </c>
       <c r="I84" s="12" t="inlineStr"/>
@@ -1943,14 +1909,10 @@
       <c r="G87" s="12" t="inlineStr"/>
       <c r="H87" s="13" t="inlineStr">
         <is>
-          <t>260 TL / -</t>
-        </is>
-      </c>
-      <c r="I87" s="13" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
+          <t>260 TL</t>
+        </is>
+      </c>
+      <c r="I87" s="12" t="inlineStr"/>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
@@ -2029,7 +1991,7 @@
       <c r="H90" s="12" t="inlineStr"/>
       <c r="I90" s="12" t="inlineStr">
         <is>
-          <t>427,62 TL / -</t>
+          <t>427,62 TL</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2016,7 @@
       <c r="G93" s="12" t="inlineStr"/>
       <c r="H93" s="12" t="inlineStr">
         <is>
-          <t>371,43 TL / -</t>
+          <t>371,43 TL</t>
         </is>
       </c>
       <c r="I93" s="12" t="inlineStr"/>
@@ -2092,7 +2054,7 @@
       <c r="G96" s="12" t="inlineStr"/>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t>600 TL / -</t>
+          <t>600 TL</t>
         </is>
       </c>
       <c r="I96" s="12" t="inlineStr"/>
@@ -2130,7 +2092,7 @@
       <c r="G99" s="12" t="inlineStr"/>
       <c r="H99" s="13" t="inlineStr">
         <is>
-          <t>551,43 TL / -</t>
+          <t>551,43 TL</t>
         </is>
       </c>
       <c r="I99" s="12" t="inlineStr"/>
@@ -2161,7 +2123,7 @@
       <c r="G100" s="12" t="inlineStr"/>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>600 TL / -</t>
+          <t>600 TL</t>
         </is>
       </c>
       <c r="I100" s="12" t="inlineStr"/>
@@ -2195,7 +2157,7 @@
       <c r="G103" s="12" t="inlineStr"/>
       <c r="H103" s="13" t="inlineStr">
         <is>
-          <t>600 TL / -</t>
+          <t>600 TL</t>
         </is>
       </c>
       <c r="I103" s="12" t="inlineStr"/>
@@ -2214,7 +2176,7 @@
       <c r="G104" s="12" t="inlineStr"/>
       <c r="H104" s="12" t="inlineStr">
         <is>
-          <t>600 TL / -</t>
+          <t>600 TL</t>
         </is>
       </c>
       <c r="I104" s="12" t="inlineStr"/>
@@ -2256,7 +2218,7 @@
     <row r="109">
       <c r="A109" s="14" t="inlineStr">
         <is>
-          <t>Son güncelleme: 13.08.2026 16:50</t>
+          <t>Son güncelleme: 13.08.2026 17:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 10:46)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,7 @@
     </font>
     <font>
       <b val="1"/>
+      <i val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
@@ -42,14 +43,27 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFD700"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="0000B050"/>
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="0000B050"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000070C0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000070C0"/>
       <sz val="10"/>
     </font>
     <font>
@@ -58,11 +72,29 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="00FF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <color rgb="00888888"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -83,8 +115,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00012169"/>
         <bgColor rgb="00012169"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+        <bgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -95,8 +139,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F4B183"/>
+        <bgColor rgb="00F4B183"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00003087"/>
         <bgColor rgb="00003087"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008EA9C1"/>
+        <bgColor rgb="008EA9C1"/>
       </patternFill>
     </fill>
     <fill>
@@ -132,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -140,40 +196,64 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -539,18 +619,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -618,7 +699,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
           <t>EFT Gönderimi</t>
@@ -631,18 +712,51 @@
           <t>EFT İsme Gelen</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr"/>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>39.87TL</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="12" t="inlineStr"/>
-      <c r="F4" s="12" t="inlineStr"/>
-      <c r="G4" s="12" t="inlineStr"/>
-      <c r="H4" s="12" t="inlineStr"/>
-      <c r="I4" s="12" t="inlineStr"/>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>Para çekmeyi, para yatırmayı eklemedim</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
@@ -655,17 +769,46 @@
           <t>7.97TL</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr"/>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>7,97TL</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr"/>
-      <c r="F5" s="12" t="inlineStr"/>
-      <c r="G5" s="12" t="inlineStr"/>
-      <c r="H5" s="12" t="inlineStr"/>
-      <c r="I5" s="12" t="inlineStr"/>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L5" s="20" t="inlineStr">
+        <is>
+          <t>Akbank'ta bireysel kotalar var havale/EFT için</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
@@ -678,21 +821,46 @@
           <t>199.41TL</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr"/>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>199,41TL</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr"/>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>199,41 TL</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr"/>
-      <c r="H6" s="12" t="inlineStr"/>
-      <c r="I6" s="12" t="inlineStr"/>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>Kredi Risk Raporumuz zamanlanabilir</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
@@ -700,26 +868,51 @@
           <t>EFT - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>39.87TL</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>27,84TL</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr"/>
-      <c r="F7" s="12" t="inlineStr"/>
-      <c r="G7" s="12" t="inlineStr"/>
-      <c r="H7" s="12" t="inlineStr"/>
-      <c r="I7" s="12" t="inlineStr"/>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L7" s="20" t="inlineStr">
+        <is>
+          <t>Şubeden kıymetli maden teslimi %10'a kadar</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
@@ -727,34 +920,46 @@
           <t>EFT - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>199.41TL</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>797.68TL</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>398,83TL</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr"/>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>398,83 TL</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>797,68 TL</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr"/>
-      <c r="I8" s="12" t="inlineStr"/>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
@@ -762,26 +967,46 @@
           <t>EFT Gönderimi</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>85.72TL</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr"/>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="12" t="inlineStr"/>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>619.047,62 TL</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>39,87 TL</t>
         </is>
       </c>
-      <c r="H9" s="12" t="inlineStr"/>
-      <c r="I9" s="12" t="inlineStr"/>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
@@ -789,24 +1014,48 @@
           <t>Düzenli EFT</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>1.00TL / 1.00%</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr"/>
-      <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="12" t="inlineStr"/>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
         <is>
           <t>7,97 TL</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr"/>
-      <c r="H10" s="12" t="inlineStr"/>
-      <c r="I10" s="12" t="inlineStr"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Havale Gönderimi</t>
@@ -824,17 +1073,41 @@
           <t>3.99TL</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr"/>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>3,99TL</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr"/>
-      <c r="F13" s="12" t="inlineStr"/>
-      <c r="G13" s="12" t="inlineStr"/>
-      <c r="H13" s="12" t="inlineStr"/>
-      <c r="I13" s="12" t="inlineStr"/>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
@@ -847,25 +1120,41 @@
           <t>99.71TL</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr"/>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>99,71TL</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr"/>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>99,71 TL</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>99,71 TL</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr"/>
-      <c r="I14" s="12" t="inlineStr"/>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
@@ -873,30 +1162,42 @@
           <t>Havale - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>3.99TL</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>19.94TL</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>3,99TL</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr"/>
-      <c r="F15" s="12" t="inlineStr"/>
-      <c r="G15" s="12" t="inlineStr"/>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>13,92 TL / -</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr">
+      <c r="I15" s="21" t="inlineStr">
         <is>
           <t>19,94 TL / -</t>
         </is>
@@ -908,38 +1209,42 @@
           <t>Havale - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>99.71TL</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>398.84TL</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>99,71TL</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr"/>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
         <is>
           <t>199,42</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>398,84 TL</t>
         </is>
       </c>
-      <c r="H16" s="13" t="inlineStr">
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>27,62 TL / -</t>
         </is>
       </c>
-      <c r="I16" s="13" t="inlineStr">
+      <c r="I16" s="21" t="inlineStr">
         <is>
           <t>398,84 TL / -</t>
         </is>
@@ -951,42 +1256,46 @@
           <t>Havale Gönderimi</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>1900.00TL / 0.70%</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>3676.20TL / 0.70%</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>150TL</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>125TL</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="F17" s="21" t="inlineStr">
         <is>
           <t>309.523,81 TL</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>39,88 TL</t>
         </is>
       </c>
-      <c r="H17" s="13" t="inlineStr">
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>13,33 TL / -</t>
         </is>
       </c>
-      <c r="I17" s="12" t="inlineStr"/>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
@@ -994,24 +1303,48 @@
           <t>Düzenli Havale</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr"/>
-      <c r="C18" s="12" t="inlineStr"/>
-      <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="12" t="inlineStr"/>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>3,99 TL</t>
         </is>
       </c>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>3,99 TL</t>
         </is>
       </c>
-      <c r="H18" s="12" t="inlineStr"/>
-      <c r="I18" s="12" t="inlineStr"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>FAST</t>
@@ -1024,22 +1357,46 @@
           <t>FAST</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>380.95TL / 0.48%</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr"/>
-      <c r="D21" s="12" t="inlineStr"/>
-      <c r="E21" s="12" t="inlineStr"/>
-      <c r="F21" s="12" t="inlineStr"/>
-      <c r="G21" s="12" t="inlineStr"/>
-      <c r="H21" s="13" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
         <is>
           <t>200 TL / 0,4</t>
         </is>
       </c>
-      <c r="I21" s="12" t="inlineStr"/>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
@@ -1047,22 +1404,46 @@
           <t>FAST - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr"/>
-      <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="12" t="inlineStr"/>
-      <c r="F22" s="12" t="inlineStr"/>
-      <c r="G22" s="12" t="inlineStr"/>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
         <is>
           <t>7,97 TL / -</t>
         </is>
       </c>
-      <c r="I22" s="12" t="inlineStr"/>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
@@ -1070,24 +1451,48 @@
           <t>FAST - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr"/>
-      <c r="D23" s="12" t="inlineStr"/>
-      <c r="E23" s="12" t="inlineStr"/>
-      <c r="F23" s="12" t="inlineStr"/>
-      <c r="G23" s="12" t="inlineStr"/>
-      <c r="H23" s="13" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
         <is>
           <t>15,96 TL / -</t>
         </is>
       </c>
-      <c r="I23" s="12" t="inlineStr"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Kiralık Kasa</t>
@@ -1100,26 +1505,46 @@
           <t>Yıllık Kasa Ücreti - büyük</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>30000.00TL</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr"/>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>4140TL</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr"/>
-      <c r="F26" s="12" t="inlineStr"/>
-      <c r="G26" s="12" t="inlineStr"/>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H26" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I26" s="12" t="inlineStr"/>
+      <c r="I26" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
@@ -1127,26 +1552,46 @@
           <t>Yıllık Kasa Ücreti - küçük</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>22000.00TL</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr"/>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>2610TL</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr"/>
-      <c r="F27" s="12" t="inlineStr"/>
-      <c r="G27" s="12" t="inlineStr"/>
-      <c r="H27" s="13" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I27" s="12" t="inlineStr"/>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
@@ -1154,26 +1599,46 @@
           <t>Yıllık Kasa Ücreti - orta</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>25000.00TL</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr"/>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>3390TL</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr"/>
-      <c r="F28" s="12" t="inlineStr"/>
-      <c r="G28" s="12" t="inlineStr"/>
-      <c r="H28" s="13" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H28" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I28" s="12" t="inlineStr"/>
+      <c r="I28" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
@@ -1181,22 +1646,46 @@
           <t>Kasa Depozito - büyük</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>28570.00TL</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr"/>
-      <c r="D29" s="12" t="inlineStr"/>
-      <c r="E29" s="12" t="inlineStr"/>
-      <c r="F29" s="12" t="inlineStr"/>
-      <c r="G29" s="12" t="inlineStr"/>
-      <c r="H29" s="13" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I29" s="12" t="inlineStr"/>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
@@ -1204,22 +1693,46 @@
           <t>Kasa Depozito - orta</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>23805.00TL</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr"/>
-      <c r="D30" s="12" t="inlineStr"/>
-      <c r="E30" s="12" t="inlineStr"/>
-      <c r="F30" s="12" t="inlineStr"/>
-      <c r="G30" s="12" t="inlineStr"/>
-      <c r="H30" s="13" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H30" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I30" s="12" t="inlineStr"/>
+      <c r="I30" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
@@ -1227,22 +1740,46 @@
           <t>Kasa Depozito - küçük</t>
         </is>
       </c>
-      <c r="B31" s="13" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>20950.00TL</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr"/>
-      <c r="D31" s="12" t="inlineStr"/>
-      <c r="E31" s="12" t="inlineStr"/>
-      <c r="F31" s="12" t="inlineStr"/>
-      <c r="G31" s="12" t="inlineStr"/>
-      <c r="H31" s="13" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G31" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H31" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I31" s="12" t="inlineStr"/>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
@@ -1255,13 +1792,41 @@
           <t>1469.52TL</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr"/>
-      <c r="D32" s="12" t="inlineStr"/>
-      <c r="E32" s="12" t="inlineStr"/>
-      <c r="F32" s="12" t="inlineStr"/>
-      <c r="G32" s="12" t="inlineStr"/>
-      <c r="H32" s="12" t="inlineStr"/>
-      <c r="I32" s="12" t="inlineStr"/>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H32" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I32" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
@@ -1269,20 +1834,48 @@
           <t>Kasa Depozito - genel</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr"/>
-      <c r="C33" s="12" t="inlineStr"/>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>9420TL</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr"/>
-      <c r="F33" s="12" t="inlineStr"/>
-      <c r="G33" s="12" t="inlineStr"/>
-      <c r="H33" s="12" t="inlineStr"/>
-      <c r="I33" s="12" t="inlineStr"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H33" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Kıymetli Maden</t>
@@ -1295,26 +1888,46 @@
           <t>Altın Transfer</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>100.00TL</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr"/>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
         <is>
           <t>415TL</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr"/>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F36" s="21" t="inlineStr">
         <is>
           <t>0.00018</t>
         </is>
       </c>
-      <c r="G36" s="12" t="inlineStr"/>
-      <c r="H36" s="12" t="inlineStr"/>
-      <c r="I36" s="12" t="inlineStr"/>
+      <c r="G36" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I36" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
@@ -1322,22 +1935,46 @@
           <t>Altın Transfer - 1-10gr</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr"/>
-      <c r="C37" s="12" t="inlineStr"/>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>57,5TL</t>
         </is>
       </c>
-      <c r="E37" s="12" t="inlineStr"/>
-      <c r="F37" s="13" t="inlineStr">
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F37" s="21" t="inlineStr">
         <is>
           <t>60 TL</t>
         </is>
       </c>
-      <c r="G37" s="12" t="inlineStr"/>
-      <c r="H37" s="12" t="inlineStr"/>
-      <c r="I37" s="12" t="inlineStr"/>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H37" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
@@ -1345,24 +1982,48 @@
           <t>Altın Transfer - 11-100gr</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr"/>
-      <c r="C38" s="12" t="inlineStr"/>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>115TL</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr"/>
-      <c r="F38" s="13" t="inlineStr">
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F38" s="21" t="inlineStr">
         <is>
           <t>120 TL</t>
         </is>
       </c>
-      <c r="G38" s="12" t="inlineStr"/>
-      <c r="H38" s="12" t="inlineStr"/>
-      <c r="I38" s="12" t="inlineStr"/>
-    </row>
-    <row r="40" ht="16" customHeight="1">
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H38" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I38" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
@@ -1375,40 +2036,48 @@
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="D41" s="13" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>95TL</t>
         </is>
       </c>
-      <c r="E41" s="12" t="inlineStr"/>
-      <c r="F41" s="13" t="inlineStr">
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="inlineStr">
         <is>
           <t>65 TL</t>
         </is>
       </c>
-      <c r="G41" s="12" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
         <is>
           <t>95,24 TL</t>
         </is>
       </c>
-      <c r="H41" s="13" t="inlineStr">
+      <c r="H41" s="21" t="inlineStr">
         <is>
           <t>339 TL / -</t>
         </is>
       </c>
-      <c r="I41" s="12" t="inlineStr"/>
-    </row>
-    <row r="43" ht="16" customHeight="1">
+      <c r="I41" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri - Kart</t>
@@ -1421,43 +2090,68 @@
           <t>Fatura Ödemeleri</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
+      <c r="B44" s="21" t="inlineStr">
         <is>
           <t>5.00TL / 3.50%</t>
         </is>
       </c>
-      <c r="C44" s="13" t="inlineStr">
+      <c r="C44" s="21" t="inlineStr">
         <is>
           <t>0.00TL</t>
         </is>
       </c>
-      <c r="D44" s="13" t="inlineStr">
+      <c r="D44" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr"/>
-      <c r="F44" s="13" t="inlineStr">
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F44" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="G44" s="13" t="inlineStr">
+      <c r="G44" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="H44" s="13" t="inlineStr">
+      <c r="H44" s="21" t="inlineStr">
         <is>
           <t>0,63 TL / -</t>
         </is>
       </c>
-      <c r="I44" s="12" t="inlineStr"/>
-    </row>
-    <row r="46" ht="16" customHeight="1">
+      <c r="I44" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L44" s="20" t="inlineStr">
+        <is>
+          <t>Fatura ödemeleri üst tier için %3,5'a çıkabiliyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="L45" s="20" t="inlineStr">
+        <is>
+          <t>Borcu Yoktur Yazısı almak için ücret alınabiliyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
+        </is>
+      </c>
+      <c r="L46" s="20" t="inlineStr">
+        <is>
+          <t>Mevduat Araştırma Ücretleri zamlanabilir</t>
         </is>
       </c>
     </row>
@@ -1467,32 +2161,53 @@
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B47" s="21" t="inlineStr">
         <is>
           <t>3.50TL / 3.50%</t>
         </is>
       </c>
-      <c r="C47" s="12" t="inlineStr"/>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D47" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E47" s="12" t="inlineStr"/>
-      <c r="F47" s="13" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="inlineStr">
         <is>
           <t>2 TL / 3,5%</t>
         </is>
       </c>
-      <c r="G47" s="12" t="inlineStr"/>
-      <c r="H47" s="12" t="inlineStr"/>
-      <c r="I47" s="12" t="inlineStr">
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H47" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="inlineStr">
         <is>
           <t>3 TL / -</t>
         </is>
       </c>
-    </row>
-    <row r="49" ht="16" customHeight="1">
+      <c r="L47" s="20" t="inlineStr">
+        <is>
+          <t>Güvenli Araç Alım Satım YKB 97,53 TRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
@@ -1510,23 +2225,43 @@
           <t>275.00TL</t>
         </is>
       </c>
-      <c r="C50" s="12" t="inlineStr"/>
-      <c r="D50" s="12" t="inlineStr">
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr"/>
-      <c r="F50" s="12" t="inlineStr">
+      <c r="E50" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
         <is>
           <t>275 TL</t>
         </is>
       </c>
-      <c r="G50" s="12" t="inlineStr"/>
-      <c r="H50" s="12" t="inlineStr"/>
-      <c r="I50" s="12" t="inlineStr"/>
-    </row>
-    <row r="52" ht="16" customHeight="1">
+      <c r="G50" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H50" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I50" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
@@ -1539,24 +2274,48 @@
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr"/>
-      <c r="C53" s="12" t="inlineStr"/>
-      <c r="D53" s="13" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
         <is>
           <t>26TL</t>
         </is>
       </c>
-      <c r="E53" s="12" t="inlineStr"/>
-      <c r="F53" s="13" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F53" s="21" t="inlineStr">
         <is>
           <t>38,10 TL</t>
         </is>
       </c>
-      <c r="G53" s="12" t="inlineStr"/>
-      <c r="H53" s="12" t="inlineStr"/>
-      <c r="I53" s="12" t="inlineStr"/>
-    </row>
-    <row r="55" ht="16" customHeight="1">
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I53" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
       <c r="A55" s="10" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
@@ -1569,20 +2328,48 @@
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr"/>
-      <c r="C56" s="12" t="inlineStr"/>
-      <c r="D56" s="12" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E56" s="12" t="inlineStr"/>
-      <c r="F56" s="12" t="inlineStr"/>
-      <c r="G56" s="12" t="inlineStr"/>
-      <c r="H56" s="12" t="inlineStr"/>
-      <c r="I56" s="12" t="inlineStr"/>
-    </row>
-    <row r="58" ht="16" customHeight="1">
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H56" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I56" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
           <t>Telefon Ödemeleri Aracılık</t>
@@ -1595,18 +2382,46 @@
           <t>Telefon Ödemeleri</t>
         </is>
       </c>
-      <c r="B59" s="12" t="inlineStr"/>
-      <c r="C59" s="12" t="inlineStr"/>
-      <c r="D59" s="12" t="inlineStr"/>
-      <c r="E59" s="12" t="inlineStr"/>
-      <c r="F59" s="12" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="inlineStr">
         <is>
           <t>1 %</t>
         </is>
       </c>
-      <c r="G59" s="12" t="inlineStr"/>
-      <c r="H59" s="12" t="inlineStr"/>
-      <c r="I59" s="12" t="inlineStr"/>
+      <c r="G59" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="11" t="inlineStr">
@@ -1614,20 +2429,48 @@
           <t>Telefon - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr"/>
-      <c r="C60" s="12" t="inlineStr"/>
-      <c r="D60" s="12" t="inlineStr"/>
-      <c r="E60" s="12" t="inlineStr"/>
-      <c r="F60" s="12" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E60" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
         <is>
           <t>99,71 TL</t>
         </is>
       </c>
-      <c r="G60" s="12" t="inlineStr"/>
-      <c r="H60" s="12" t="inlineStr"/>
-      <c r="I60" s="12" t="inlineStr"/>
-    </row>
-    <row r="62" ht="16" customHeight="1">
+      <c r="G60" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I60" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="10" t="inlineStr">
         <is>
           <t>Vergi Tahsilat Aracılık</t>
@@ -1641,15 +2484,15 @@
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr"/>
-      <c r="C63" s="12" t="inlineStr"/>
-      <c r="D63" s="12" t="inlineStr"/>
-      <c r="E63" s="12" t="inlineStr"/>
-      <c r="F63" s="12" t="inlineStr"/>
-      <c r="G63" s="12" t="inlineStr"/>
-      <c r="H63" s="12" t="inlineStr"/>
-      <c r="I63" s="12" t="inlineStr"/>
-    </row>
-    <row r="65" ht="16" customHeight="1">
+      <c r="C63" s="13" t="inlineStr"/>
+      <c r="D63" s="14" t="inlineStr"/>
+      <c r="E63" s="15" t="inlineStr"/>
+      <c r="F63" s="16" t="inlineStr"/>
+      <c r="G63" s="17" t="inlineStr"/>
+      <c r="H63" s="18" t="inlineStr"/>
+      <c r="I63" s="19" t="inlineStr"/>
+    </row>
+    <row r="65" ht="18" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
@@ -1667,15 +2510,43 @@
           <t>287.62TL</t>
         </is>
       </c>
-      <c r="C66" s="12" t="inlineStr"/>
-      <c r="D66" s="12" t="inlineStr"/>
-      <c r="E66" s="12" t="inlineStr"/>
-      <c r="F66" s="12" t="inlineStr"/>
-      <c r="G66" s="12" t="inlineStr"/>
-      <c r="H66" s="12" t="inlineStr"/>
-      <c r="I66" s="12" t="inlineStr"/>
-    </row>
-    <row r="68" ht="16" customHeight="1">
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G66" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I66" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="10" t="inlineStr">
         <is>
           <t>Mevduat Araştırma</t>
@@ -1688,26 +2559,46 @@
           <t>Referans Mektubu -</t>
         </is>
       </c>
-      <c r="B69" s="13" t="inlineStr">
+      <c r="B69" s="21" t="inlineStr">
         <is>
           <t>4000.00TL</t>
         </is>
       </c>
-      <c r="C69" s="12" t="inlineStr"/>
-      <c r="D69" s="13" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D69" s="21" t="inlineStr">
         <is>
           <t>770TL</t>
         </is>
       </c>
-      <c r="E69" s="12" t="inlineStr"/>
-      <c r="F69" s="12" t="inlineStr"/>
-      <c r="G69" s="12" t="inlineStr"/>
-      <c r="H69" s="13" t="inlineStr">
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G69" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H69" s="21" t="inlineStr">
         <is>
           <t>50 TL / -</t>
         </is>
       </c>
-      <c r="I69" s="12" t="inlineStr"/>
+      <c r="I69" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="11" t="inlineStr">
@@ -1715,22 +2606,46 @@
           <t>Hesap Özeti Verilmesi -</t>
         </is>
       </c>
-      <c r="B70" s="12" t="inlineStr"/>
-      <c r="C70" s="12" t="inlineStr"/>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
         <is>
           <t>190TL</t>
         </is>
       </c>
-      <c r="E70" s="12" t="inlineStr"/>
-      <c r="F70" s="13" t="inlineStr">
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F70" s="21" t="inlineStr">
         <is>
           <t>12 TL</t>
         </is>
       </c>
-      <c r="G70" s="12" t="inlineStr"/>
-      <c r="H70" s="12" t="inlineStr"/>
-      <c r="I70" s="12" t="inlineStr"/>
+      <c r="G70" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H70" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I70" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="11" t="inlineStr">
@@ -1738,20 +2653,48 @@
           <t>Borcu Yoktur Yazısı</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr"/>
-      <c r="C71" s="12" t="inlineStr"/>
-      <c r="D71" s="12" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E71" s="12" t="inlineStr"/>
-      <c r="F71" s="12" t="inlineStr"/>
-      <c r="G71" s="12" t="inlineStr"/>
-      <c r="H71" s="12" t="inlineStr"/>
-      <c r="I71" s="12" t="inlineStr"/>
-    </row>
-    <row r="73" ht="16" customHeight="1">
+      <c r="E71" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G71" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H71" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I71" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
@@ -1764,24 +2707,48 @@
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
-      <c r="B74" s="12" t="inlineStr"/>
-      <c r="C74" s="12" t="inlineStr"/>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D74" s="21" t="inlineStr">
         <is>
           <t>0.41TL</t>
         </is>
       </c>
-      <c r="E74" s="12" t="inlineStr"/>
-      <c r="F74" s="12" t="inlineStr"/>
-      <c r="G74" s="12" t="inlineStr"/>
-      <c r="H74" s="13" t="inlineStr">
+      <c r="E74" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F74" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G74" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H74" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I74" s="12" t="inlineStr"/>
-    </row>
-    <row r="76" ht="16" customHeight="1">
+      <c r="I74" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
       <c r="A76" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
@@ -1794,24 +2761,48 @@
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
-      <c r="B77" s="12" t="inlineStr"/>
-      <c r="C77" s="12" t="inlineStr"/>
-      <c r="D77" s="13" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D77" s="21" t="inlineStr">
         <is>
           <t>0.45EUR</t>
         </is>
       </c>
-      <c r="E77" s="12" t="inlineStr"/>
-      <c r="F77" s="13" t="inlineStr">
+      <c r="E77" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F77" s="21" t="inlineStr">
         <is>
           <t>0.27 TL</t>
         </is>
       </c>
-      <c r="G77" s="12" t="inlineStr"/>
-      <c r="H77" s="12" t="inlineStr"/>
-      <c r="I77" s="12" t="inlineStr"/>
-    </row>
-    <row r="79" ht="16" customHeight="1">
+      <c r="G77" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H77" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I77" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
       <c r="A79" s="10" t="inlineStr">
         <is>
           <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
@@ -1824,30 +2815,46 @@
           <t>Çek Düzenleme -</t>
         </is>
       </c>
-      <c r="B80" s="13" t="inlineStr">
+      <c r="B80" s="21" t="inlineStr">
         <is>
           <t>9.52TL / 0.10%</t>
         </is>
       </c>
-      <c r="C80" s="12" t="inlineStr"/>
-      <c r="D80" s="13" t="inlineStr">
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D80" s="21" t="inlineStr">
         <is>
           <t>290TL / 1.10%</t>
         </is>
       </c>
-      <c r="E80" s="12" t="inlineStr"/>
-      <c r="F80" s="13" t="inlineStr">
+      <c r="E80" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F80" s="21" t="inlineStr">
         <is>
           <t>761,90 TL</t>
         </is>
       </c>
-      <c r="G80" s="12" t="inlineStr"/>
-      <c r="H80" s="13" t="inlineStr">
+      <c r="G80" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H80" s="21" t="inlineStr">
         <is>
           <t>104,76 TL / -</t>
         </is>
       </c>
-      <c r="I80" s="12" t="inlineStr"/>
+      <c r="I80" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="11" t="inlineStr">
@@ -1855,20 +2862,48 @@
           <t>Çek Defteri (Yaprak Başı) -</t>
         </is>
       </c>
-      <c r="B81" s="12" t="inlineStr"/>
-      <c r="C81" s="12" t="inlineStr"/>
-      <c r="D81" s="12" t="inlineStr"/>
-      <c r="E81" s="12" t="inlineStr"/>
-      <c r="F81" s="12" t="inlineStr">
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E81" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
         <is>
           <t>2.380,95 TL</t>
         </is>
       </c>
-      <c r="G81" s="12" t="inlineStr"/>
-      <c r="H81" s="12" t="inlineStr"/>
-      <c r="I81" s="12" t="inlineStr"/>
-    </row>
-    <row r="83" ht="16" customHeight="1">
+      <c r="G81" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I81" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
       <c r="A83" s="10" t="inlineStr">
         <is>
           <t>Çek İade Ücreti</t>
@@ -1881,32 +2916,48 @@
           <t>Çek İade Ücreti</t>
         </is>
       </c>
-      <c r="B84" s="13" t="inlineStr">
+      <c r="B84" s="21" t="inlineStr">
         <is>
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="C84" s="12" t="inlineStr"/>
-      <c r="D84" s="13" t="inlineStr">
+      <c r="C84" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D84" s="21" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E84" s="12" t="inlineStr"/>
-      <c r="F84" s="13" t="inlineStr">
+      <c r="E84" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F84" s="21" t="inlineStr">
         <is>
           <t>380,95 TL</t>
         </is>
       </c>
-      <c r="G84" s="12" t="inlineStr"/>
-      <c r="H84" s="13" t="inlineStr">
+      <c r="G84" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H84" s="21" t="inlineStr">
         <is>
           <t>123,81 TL / -</t>
         </is>
       </c>
-      <c r="I84" s="12" t="inlineStr"/>
-    </row>
-    <row r="86" ht="16" customHeight="1">
+      <c r="I84" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
       <c r="A86" s="10" t="inlineStr">
         <is>
           <t>Çek Tahsilat Ücreti</t>
@@ -1919,34 +2970,42 @@
           <t>Çek Tahsilat</t>
         </is>
       </c>
-      <c r="B87" s="13" t="inlineStr">
+      <c r="B87" s="21" t="inlineStr">
         <is>
           <t>45USD</t>
         </is>
       </c>
-      <c r="C87" s="13" t="inlineStr">
+      <c r="C87" s="21" t="inlineStr">
         <is>
           <t>590.48TL / 0.77%</t>
         </is>
       </c>
-      <c r="D87" s="12" t="inlineStr"/>
-      <c r="E87" s="13" t="inlineStr">
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E87" s="21" t="inlineStr">
         <is>
           <t>1.70%</t>
         </is>
       </c>
-      <c r="F87" s="13" t="inlineStr">
+      <c r="F87" s="21" t="inlineStr">
         <is>
           <t>714,29 TL</t>
         </is>
       </c>
-      <c r="G87" s="12" t="inlineStr"/>
-      <c r="H87" s="13" t="inlineStr">
+      <c r="G87" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H87" s="21" t="inlineStr">
         <is>
           <t>260 TL / -</t>
         </is>
       </c>
-      <c r="I87" s="13" t="inlineStr">
+      <c r="I87" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
@@ -1958,34 +3017,46 @@
           <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
         </is>
       </c>
-      <c r="B88" s="13" t="inlineStr">
+      <c r="B88" s="21" t="inlineStr">
         <is>
           <t>257.15TL</t>
         </is>
       </c>
-      <c r="C88" s="12" t="inlineStr"/>
-      <c r="D88" s="13" t="inlineStr">
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D88" s="21" t="inlineStr">
         <is>
           <t>2940TL / 1%</t>
         </is>
       </c>
-      <c r="E88" s="13" t="inlineStr">
+      <c r="E88" s="21" t="inlineStr">
         <is>
           <t>390TL / 0.2%</t>
         </is>
       </c>
-      <c r="F88" s="13" t="inlineStr">
+      <c r="F88" s="21" t="inlineStr">
         <is>
           <t>1.666,67 TL</t>
         </is>
       </c>
-      <c r="G88" s="13" t="inlineStr">
+      <c r="G88" s="21" t="inlineStr">
         <is>
           <t>585,71 TL</t>
         </is>
       </c>
-      <c r="H88" s="12" t="inlineStr"/>
-      <c r="I88" s="12" t="inlineStr"/>
+      <c r="H88" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I88" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="11" t="inlineStr">
@@ -1993,22 +3064,42 @@
           <t>Diğer Banka Çeki -</t>
         </is>
       </c>
-      <c r="B89" s="13" t="inlineStr">
+      <c r="B89" s="21" t="inlineStr">
         <is>
           <t>390.48TL</t>
         </is>
       </c>
-      <c r="C89" s="12" t="inlineStr"/>
-      <c r="D89" s="13" t="inlineStr">
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D89" s="21" t="inlineStr">
         <is>
           <t>350TL</t>
         </is>
       </c>
-      <c r="E89" s="12" t="inlineStr"/>
-      <c r="F89" s="12" t="inlineStr"/>
-      <c r="G89" s="12" t="inlineStr"/>
-      <c r="H89" s="12" t="inlineStr"/>
-      <c r="I89" s="12" t="inlineStr">
+      <c r="E89" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F89" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G89" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H89" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I89" s="19" t="inlineStr">
         <is>
           <t>576,19 TL / 0,6</t>
         </is>
@@ -2020,20 +3111,48 @@
           <t>Aynı Banka Çeki -</t>
         </is>
       </c>
-      <c r="B90" s="12" t="inlineStr"/>
-      <c r="C90" s="12" t="inlineStr"/>
-      <c r="D90" s="12" t="inlineStr"/>
-      <c r="E90" s="12" t="inlineStr"/>
-      <c r="F90" s="12" t="inlineStr"/>
-      <c r="G90" s="12" t="inlineStr"/>
-      <c r="H90" s="12" t="inlineStr"/>
-      <c r="I90" s="12" t="inlineStr">
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E90" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G90" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I90" s="19" t="inlineStr">
         <is>
           <t>427,62 TL / -</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="16" customHeight="1">
+    <row r="92" ht="18" customHeight="1">
       <c r="A92" s="10" t="inlineStr">
         <is>
           <t>Çek Belgelendirme ve Düzeltme Ücreti</t>
@@ -2046,20 +3165,48 @@
           <t>Karşılıksız Çek Belgelendirme -</t>
         </is>
       </c>
-      <c r="B93" s="12" t="inlineStr"/>
-      <c r="C93" s="12" t="inlineStr"/>
-      <c r="D93" s="12" t="inlineStr"/>
-      <c r="E93" s="12" t="inlineStr"/>
-      <c r="F93" s="12" t="inlineStr"/>
-      <c r="G93" s="12" t="inlineStr"/>
-      <c r="H93" s="12" t="inlineStr">
+      <c r="B93" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E93" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F93" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G93" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H93" s="18" t="inlineStr">
         <is>
           <t>371,43 TL / -</t>
         </is>
       </c>
-      <c r="I93" s="12" t="inlineStr"/>
-    </row>
-    <row r="95" ht="16" customHeight="1">
+      <c r="I93" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
       <c r="A95" s="10" t="inlineStr">
         <is>
           <t>Senet İade Ücreti</t>
@@ -2072,32 +3219,48 @@
           <t>Senet İade Ücreti</t>
         </is>
       </c>
-      <c r="B96" s="13" t="inlineStr">
+      <c r="B96" s="21" t="inlineStr">
         <is>
           <t>495.24TL</t>
         </is>
       </c>
-      <c r="C96" s="12" t="inlineStr"/>
-      <c r="D96" s="13" t="inlineStr">
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D96" s="21" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
-      <c r="E96" s="12" t="inlineStr"/>
-      <c r="F96" s="13" t="inlineStr">
+      <c r="E96" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F96" s="21" t="inlineStr">
         <is>
           <t>571,43 TL</t>
         </is>
       </c>
-      <c r="G96" s="12" t="inlineStr"/>
-      <c r="H96" s="13" t="inlineStr">
+      <c r="G96" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H96" s="21" t="inlineStr">
         <is>
           <t>600 TL / -</t>
         </is>
       </c>
-      <c r="I96" s="12" t="inlineStr"/>
-    </row>
-    <row r="98" ht="16" customHeight="1">
+      <c r="I96" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="18" customHeight="1">
       <c r="A98" s="10" t="inlineStr">
         <is>
           <t>Senet Protesto İşlemleri Ücreti</t>
@@ -2110,30 +3273,46 @@
           <t>Senet Protesto Kaldırma -</t>
         </is>
       </c>
-      <c r="B99" s="13" t="inlineStr">
+      <c r="B99" s="21" t="inlineStr">
         <is>
           <t>533.34TL</t>
         </is>
       </c>
-      <c r="C99" s="12" t="inlineStr"/>
-      <c r="D99" s="13" t="inlineStr">
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D99" s="21" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
-      <c r="E99" s="12" t="inlineStr"/>
-      <c r="F99" s="13" t="inlineStr">
+      <c r="E99" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F99" s="21" t="inlineStr">
         <is>
           <t>619,05 TL</t>
         </is>
       </c>
-      <c r="G99" s="12" t="inlineStr"/>
-      <c r="H99" s="13" t="inlineStr">
+      <c r="G99" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H99" s="21" t="inlineStr">
         <is>
           <t>551,43 TL / -</t>
         </is>
       </c>
-      <c r="I99" s="12" t="inlineStr"/>
+      <c r="I99" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="11" t="inlineStr">
@@ -2141,32 +3320,48 @@
           <t>Senet Protesto -</t>
         </is>
       </c>
-      <c r="B100" s="13" t="inlineStr">
+      <c r="B100" s="21" t="inlineStr">
         <is>
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="C100" s="12" t="inlineStr"/>
-      <c r="D100" s="13" t="inlineStr">
+      <c r="C100" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D100" s="21" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
-      <c r="E100" s="12" t="inlineStr"/>
-      <c r="F100" s="13" t="inlineStr">
+      <c r="E100" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F100" s="21" t="inlineStr">
         <is>
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="G100" s="12" t="inlineStr"/>
-      <c r="H100" s="13" t="inlineStr">
+      <c r="G100" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H100" s="21" t="inlineStr">
         <is>
           <t>600 TL / -</t>
         </is>
       </c>
-      <c r="I100" s="12" t="inlineStr"/>
-    </row>
-    <row r="102" ht="16" customHeight="1">
+      <c r="I100" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="18" customHeight="1">
       <c r="A102" s="10" t="inlineStr">
         <is>
           <t>Senet Tahsile Alma Ücreti</t>
@@ -2179,26 +3374,46 @@
           <t>Muhabir Banka Senet Tahsili -</t>
         </is>
       </c>
-      <c r="B103" s="12" t="inlineStr"/>
-      <c r="C103" s="12" t="inlineStr">
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C103" s="13" t="inlineStr">
         <is>
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="D103" s="12" t="inlineStr"/>
-      <c r="E103" s="12" t="inlineStr"/>
-      <c r="F103" s="13" t="inlineStr">
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E103" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F103" s="21" t="inlineStr">
         <is>
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="G103" s="12" t="inlineStr"/>
-      <c r="H103" s="13" t="inlineStr">
+      <c r="G103" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H103" s="21" t="inlineStr">
         <is>
           <t>600 TL / -</t>
         </is>
       </c>
-      <c r="I103" s="12" t="inlineStr"/>
+      <c r="I103" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="11" t="inlineStr">
@@ -2206,20 +3421,48 @@
           <t>Aynı Banka Senet Tahsili -</t>
         </is>
       </c>
-      <c r="B104" s="12" t="inlineStr"/>
-      <c r="C104" s="12" t="inlineStr"/>
-      <c r="D104" s="12" t="inlineStr"/>
-      <c r="E104" s="12" t="inlineStr"/>
-      <c r="F104" s="12" t="inlineStr"/>
-      <c r="G104" s="12" t="inlineStr"/>
-      <c r="H104" s="12" t="inlineStr">
+      <c r="B104" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C104" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E104" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F104" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G104" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
         <is>
           <t>600 TL / -</t>
         </is>
       </c>
-      <c r="I104" s="12" t="inlineStr"/>
-    </row>
-    <row r="106" ht="16" customHeight="1">
+      <c r="I104" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="18" customHeight="1">
       <c r="A106" s="10" t="inlineStr">
         <is>
           <t>HGS</t>
@@ -2232,64 +3475,59 @@
           <t>HGS Kart Ücreti</t>
         </is>
       </c>
-      <c r="B107" s="13" t="inlineStr">
+      <c r="B107" s="21" t="inlineStr">
         <is>
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="C107" s="12" t="inlineStr"/>
-      <c r="D107" s="13" t="inlineStr">
+      <c r="C107" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D107" s="21" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="E107" s="12" t="inlineStr"/>
-      <c r="F107" s="13" t="inlineStr">
+      <c r="E107" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F107" s="21" t="inlineStr">
         <is>
           <t>500 TL</t>
         </is>
       </c>
-      <c r="G107" s="12" t="inlineStr"/>
-      <c r="H107" s="12" t="inlineStr"/>
-      <c r="I107" s="12" t="inlineStr"/>
+      <c r="G107" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H107" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I107" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="14" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 14.08.2026 10:30</t>
+      <c r="A109" s="22" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 14.08.2026 10:46</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A65:I65"/>
+  <mergeCells count="5">
     <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A46:I46"/>
     <mergeCell ref="H1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A55:I55"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A86:I86"/>
-    <mergeCell ref="A95:I95"/>
-    <mergeCell ref="A76:I76"/>
-    <mergeCell ref="A106:I106"/>
-    <mergeCell ref="A35:I35"/>
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="A62:I62"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A52:I52"/>
-    <mergeCell ref="A43:I43"/>
-    <mergeCell ref="A68:I68"/>
-    <mergeCell ref="A102:I102"/>
-    <mergeCell ref="A40:I40"/>
-    <mergeCell ref="A58:I58"/>
-    <mergeCell ref="A83:I83"/>
-    <mergeCell ref="A92:I92"/>
-    <mergeCell ref="A98:I98"/>
-    <mergeCell ref="A73:I73"/>
-    <mergeCell ref="A49:I49"/>
-    <mergeCell ref="A79:I79"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 11:28)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -786,7 +786,7 @@
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>7,97 TL</t>
         </is>
       </c>
       <c r="G5" s="17" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>15,96 TL</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
@@ -940,14 +940,14 @@
           <t>39,87TL</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>309.523,82 TL</t>
         </is>
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>39,87 TL</t>
         </is>
       </c>
       <c r="H8" s="18" t="inlineStr">
@@ -987,14 +987,14 @@
           <t>79,76TL</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>619.047,62 TL</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>79,76 TL</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
@@ -1083,12 +1083,12 @@
       </c>
       <c r="F11" s="21" t="inlineStr">
         <is>
-          <t>619.047,62 TL</t>
+          <t>4.25 %</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>39,87 TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
@@ -1108,7 +1108,7 @@
           <t>Düzenli EFT</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>1.00TL / 1.00%</t>
         </is>
@@ -1128,9 +1128,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F12" s="21" t="inlineStr">
-        <is>
-          <t>7,97 TL</t>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr">
@@ -1184,12 +1184,12 @@
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3,99 TL</t>
         </is>
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3,99 TL</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>7,98 TL</t>
         </is>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>7,98 TL</t>
         </is>
       </c>
       <c r="H16" s="18" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>3.99TL</t>
+          <t>1050.00TL</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>19.94TL</t>
+          <t>2485.72TL</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -1323,19 +1323,19 @@
           <t>19,94TL</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>152.380,96 TL</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>19,94 TL</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>13,92 TL / -</t>
+          <t>13,33 TL / -</t>
         </is>
       </c>
       <c r="I18" s="21" t="inlineStr">
@@ -1350,44 +1350,44 @@
           <t>Havale - 8300-399000 TRY</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>7.98TL</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>39.88TL</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>1500.00TL</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>2923.81TL</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>7,98TL</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>39,88TL</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H19" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>309.523,81 TL</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="inlineStr">
+        <is>
+          <t>39,88 TL</t>
+        </is>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>27,62 TL / -</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="inlineStr">
+        <is>
+          <t>39,88 TL / -</t>
         </is>
       </c>
     </row>
@@ -1399,12 +1399,12 @@
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>99.71TL</t>
+          <t>1900.00TL / 0.70%</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>398.84TL</t>
+          <t>3676.20TL / 0.70%</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="H20" s="21" t="inlineStr">
         <is>
-          <t>27,62 TL / -</t>
+          <t>199,05 TL / -</t>
         </is>
       </c>
       <c r="I20" s="21" t="inlineStr">
@@ -1444,14 +1444,14 @@
           <t>Havale Gönderimi</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
-        <is>
-          <t>1900.00TL / 0.70%</t>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>3676.20TL / 0.70%</t>
+          <t>1038.10TL / 0.58%</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
@@ -1466,17 +1466,17 @@
       </c>
       <c r="F21" s="21" t="inlineStr">
         <is>
-          <t>309.523,81 TL</t>
-        </is>
-      </c>
-      <c r="G21" s="21" t="inlineStr">
-        <is>
-          <t>39,88 TL</t>
-        </is>
-      </c>
-      <c r="H21" s="21" t="inlineStr">
-        <is>
-          <t>13,33 TL / -</t>
+          <t>1.300 TL / 0,6 %</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I21" s="19" t="inlineStr">
@@ -1485,67 +1485,67 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Düzenli Havale</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>3,99 TL</t>
-        </is>
-      </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>3,99 TL</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I22" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>FAST</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>FAST - 0-8300 TRY</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>7.97TL</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>7,97 TL / -</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>FAST</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="inlineStr">
+          <t>FAST - 399000+ TRY</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>380.95TL / 0.48%</t>
         </is>
@@ -1575,9 +1575,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H25" s="21" t="inlineStr">
-        <is>
-          <t>200 TL / 0,4</t>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
@@ -1589,12 +1589,12 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>FAST - 0-8300 TRY</t>
+          <t>FAST - 8300-399000 TRY</t>
         </is>
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>7.97TL</t>
+          <t>15.96TL</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="H26" s="21" t="inlineStr">
         <is>
-          <t>7,97 TL / -</t>
+          <t>15,96 TL / -</t>
         </is>
       </c>
       <c r="I26" s="19" t="inlineStr">
@@ -1636,12 +1636,12 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>FAST - 8300-399000 TRY</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>15.96TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>200 TL / 0,4</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
@@ -1680,69 +1680,69 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>FAST - 399000+ TRY</t>
-        </is>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E28" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F28" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H28" s="18" t="inlineStr">
-        <is>
-          <t>15,96 TL / -</t>
-        </is>
-      </c>
-      <c r="I28" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Kiralık Kasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Yıllık Kasa Ücreti - büyük</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>30000.00TL</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>4140TL</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H30" s="21" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
+      <c r="I30" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - büyük</t>
+          <t>Yıllık Kasa Ücreti - küçük</t>
         </is>
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>30000.00TL</t>
+          <t>22000.00TL</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
-          <t>4140TL</t>
+          <t>2610TL</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -1784,12 +1784,12 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - küçük</t>
+          <t>Yıllık Kasa Ücreti - orta</t>
         </is>
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>22000.00TL</t>
+          <t>25000.00TL</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
-          <t>2610TL</t>
+          <t>3390TL</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -1831,12 +1831,12 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - orta</t>
+          <t>Kasa Depozito - büyük</t>
         </is>
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>25000.00TL</t>
+          <t>28570.00TL</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1844,9 +1844,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
-        <is>
-          <t>3390TL</t>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
@@ -1878,12 +1878,12 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - büyük</t>
+          <t>Kasa Depozito - orta</t>
         </is>
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>28570.00TL</t>
+          <t>23805.00TL</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1925,12 +1925,12 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - orta</t>
+          <t>Kasa Depozito - küçük</t>
         </is>
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>23805.00TL</t>
+          <t>20950.00TL</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1972,12 +1972,12 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - küçük</t>
-        </is>
-      </c>
-      <c r="B36" s="21" t="inlineStr">
-        <is>
-          <t>20950.00TL</t>
+          <t>Yıllık Kasa Ücreti - genel</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>1469.52TL</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -2005,9 +2005,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H36" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I36" s="19" t="inlineStr">
@@ -2019,12 +2019,12 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - genel</t>
+          <t>Kasa Depozito - genel</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>1469.52TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>9420TL</t>
         </is>
       </c>
       <c r="E37" s="15" t="inlineStr">
@@ -2063,64 +2063,64 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>Kasa Depozito - genel</t>
-        </is>
-      </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
-        <is>
-          <t>9420TL</t>
-        </is>
-      </c>
-      <c r="E38" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F38" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G38" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H38" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I38" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Kıymetli Maden</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Altın Transfer - 0-8300</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>50.00TL</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>3.25%</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H40" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I40" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer</t>
+          <t>Altın Transfer - 8300-399000</t>
         </is>
       </c>
       <c r="B41" s="21" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="D41" s="21" t="inlineStr">
         <is>
-          <t>415TL</t>
+          <t>170TL</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr">
@@ -2143,9 +2143,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F41" s="21" t="inlineStr">
-        <is>
-          <t>0.00018</t>
+      <c r="F41" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G41" s="17" t="inlineStr">
@@ -2167,7 +2167,7 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 1-10gr</t>
+          <t>Altın Transfer</t>
         </is>
       </c>
       <c r="B42" s="12" t="inlineStr">
@@ -2182,17 +2182,17 @@
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr">
         <is>
-          <t>57,5TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>60 TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G42" s="17" t="inlineStr">
@@ -2214,636 +2214,723 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
+          <t>Altın Transfer - 1-10gr</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>57,5TL</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>60 TL</t>
+        </is>
+      </c>
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H43" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I43" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
           <t>Altın Transfer - 11-100gr</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D43" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E43" s="15" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
         <is>
           <t>115TL</t>
         </is>
       </c>
-      <c r="F43" s="16" t="inlineStr">
+      <c r="F44" s="16" t="inlineStr">
         <is>
           <t>120 TL</t>
         </is>
       </c>
-      <c r="G43" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H43" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I43" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="G44" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H44" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I44" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Altın Transfer - 399000+</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D45" s="21" t="inlineStr">
+        <is>
+          <t>415TL</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F45" s="21" t="inlineStr">
+        <is>
+          <t>0.00018</t>
+        </is>
+      </c>
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H45" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I45" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
-      <c r="B46" s="21" t="inlineStr">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="D46" s="21" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>95TL</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F46" s="21" t="inlineStr">
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F48" s="21" t="inlineStr">
         <is>
           <t>65 TL</t>
         </is>
       </c>
-      <c r="G46" s="17" t="inlineStr">
+      <c r="G48" s="17" t="inlineStr">
         <is>
           <t>95,24 TL</t>
         </is>
       </c>
-      <c r="H46" s="21" t="inlineStr">
+      <c r="H48" s="21" t="inlineStr">
         <is>
           <t>339 TL / -</t>
         </is>
       </c>
-      <c r="I46" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="10" t="inlineStr">
+      <c r="I48" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri - Kart</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri</t>
         </is>
       </c>
-      <c r="B49" s="21" t="inlineStr">
+      <c r="B51" s="21" t="inlineStr">
         <is>
           <t>5.00TL / 3.50%</t>
         </is>
       </c>
-      <c r="C49" s="21" t="inlineStr">
+      <c r="C51" s="21" t="inlineStr">
         <is>
           <t>0.00TL</t>
         </is>
       </c>
-      <c r="D49" s="21" t="inlineStr">
+      <c r="D51" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E49" s="21" t="inlineStr">
+      <c r="E51" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="F49" s="21" t="inlineStr">
+      <c r="F51" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="G49" s="21" t="inlineStr">
+      <c r="G51" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="H49" s="21" t="inlineStr">
+      <c r="H51" s="21" t="inlineStr">
         <is>
           <t>0,63 TL / -</t>
         </is>
       </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L49" s="20" t="inlineStr">
+      <c r="I51" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L51" s="20" t="inlineStr">
         <is>
           <t>Fatura ödemeleri üst tier için %3,5'a çıkabiliyor</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="L50" s="20" t="inlineStr">
+    <row r="52">
+      <c r="L52" s="20" t="inlineStr">
         <is>
           <t>Borcu Yoktur Yazısı almak için ücret alınabiliyor</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
-      <c r="L51" s="20" t="inlineStr">
+      <c r="L53" s="20" t="inlineStr">
         <is>
           <t>Mevduat Araştırma Ücretleri zamlanabilir</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
-      <c r="B52" s="21" t="inlineStr">
+      <c r="B54" s="21" t="inlineStr">
         <is>
           <t>3.50TL / 3.50%</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D52" s="21" t="inlineStr">
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E52" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F52" s="21" t="inlineStr">
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F54" s="21" t="inlineStr">
         <is>
           <t>2 TL / 3,5%</t>
         </is>
       </c>
-      <c r="G52" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H52" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I52" s="19" t="inlineStr">
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I54" s="19" t="inlineStr">
         <is>
           <t>3 TL / -</t>
         </is>
       </c>
-      <c r="L52" s="20" t="inlineStr">
+      <c r="L54" s="20" t="inlineStr">
         <is>
           <t>Güvenli Araç Alım Satım YKB 97,53 TRY</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="10" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>275.00TL</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="E55" s="15" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="F55" s="16" t="inlineStr">
+      <c r="F57" s="16" t="inlineStr">
         <is>
           <t>275 TL</t>
         </is>
       </c>
-      <c r="G55" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H55" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="10" t="inlineStr">
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="10" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C58" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D58" s="21" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
         <is>
           <t>26TL</t>
         </is>
       </c>
-      <c r="E58" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F58" s="21" t="inlineStr">
+      <c r="E60" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F60" s="21" t="inlineStr">
         <is>
           <t>38,10 TL</t>
         </is>
       </c>
-      <c r="G58" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H58" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I58" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="G60" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I60" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="10" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="11" t="inlineStr">
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D61" s="14" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E61" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G61" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H61" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="10" t="inlineStr">
         <is>
           <t>Telefon Ödemeleri Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="11" t="inlineStr">
-        <is>
-          <t>Telefon Ödemeleri</t>
-        </is>
-      </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D64" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E64" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F64" s="16" t="inlineStr">
-        <is>
-          <t>1 %</t>
-        </is>
-      </c>
-      <c r="G64" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H64" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I64" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>Telefon - 399000+ TRY</t>
-        </is>
-      </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C65" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D65" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E65" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F65" s="16" t="inlineStr">
-        <is>
-          <t>99,71 TL</t>
-        </is>
-      </c>
-      <c r="G65" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H65" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I65" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="10" t="inlineStr">
-        <is>
-          <t>Vergi Tahsilat Aracılık</t>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>Telefon - 0-8300 TRY</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>3,99 TL</t>
+        </is>
+      </c>
+      <c r="G66" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I66" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>Telefon - 8300-399000 TRY</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>7,98 TL</t>
+        </is>
+      </c>
+      <c r="G67" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H67" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I67" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="11" t="inlineStr">
         <is>
+          <t>Telefon - 399000+ TRY</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>99,71 TL</t>
+        </is>
+      </c>
+      <c r="G68" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H68" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I68" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>Telefon Ödemeleri</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>1 %</t>
+        </is>
+      </c>
+      <c r="G69" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H69" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I69" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Vergi Tahsilat Aracılık</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
           <t>Vergi Tahsilat</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr"/>
-      <c r="C68" s="13" t="inlineStr"/>
-      <c r="D68" s="14" t="inlineStr"/>
-      <c r="E68" s="15" t="inlineStr"/>
-      <c r="F68" s="16" t="inlineStr"/>
-      <c r="G68" s="17" t="inlineStr"/>
-      <c r="H68" s="18" t="inlineStr"/>
-      <c r="I68" s="19" t="inlineStr"/>
-    </row>
-    <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="10" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr"/>
+      <c r="C72" s="13" t="inlineStr"/>
+      <c r="D72" s="14" t="inlineStr"/>
+      <c r="E72" s="15" t="inlineStr"/>
+      <c r="F72" s="16" t="inlineStr"/>
+      <c r="G72" s="17" t="inlineStr"/>
+      <c r="H72" s="18" t="inlineStr"/>
+      <c r="I72" s="19" t="inlineStr"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="10" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="A71" s="11" t="inlineStr">
-        <is>
-          <t>Arşiv Araştırma Ücreti</t>
-        </is>
-      </c>
-      <c r="B71" s="12" t="inlineStr">
-        <is>
-          <t>287.62TL</t>
-        </is>
-      </c>
-      <c r="C71" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D71" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E71" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F71" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G71" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H71" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I71" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="10" t="inlineStr">
-        <is>
-          <t>Mevduat Araştırma</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
-        <is>
-          <t>Referans Mektubu -</t>
-        </is>
-      </c>
-      <c r="B74" s="21" t="inlineStr">
-        <is>
-          <t>4000.00TL</t>
-        </is>
-      </c>
-      <c r="C74" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D74" s="21" t="inlineStr">
-        <is>
-          <t>770TL</t>
-        </is>
-      </c>
-      <c r="E74" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F74" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G74" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H74" s="21" t="inlineStr">
-        <is>
-          <t>50 TL / -</t>
-        </is>
-      </c>
-      <c r="I74" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="11" t="inlineStr">
         <is>
-          <t>Hesap Özeti Verilmesi -</t>
+          <t>Arşiv Araştırma Ücreti</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>287.62TL</t>
         </is>
       </c>
       <c r="C75" s="13" t="inlineStr">
@@ -2851,9 +2938,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D75" s="21" t="inlineStr">
-        <is>
-          <t>190TL</t>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E75" s="15" t="inlineStr">
@@ -2861,9 +2948,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F75" s="21" t="inlineStr">
-        <is>
-          <t>12 TL</t>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G75" s="17" t="inlineStr">
@@ -2882,219 +2969,219 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="11" t="inlineStr">
-        <is>
-          <t>Borcu Yoktur Yazısı</t>
-        </is>
-      </c>
-      <c r="B76" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C76" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D76" s="14" t="inlineStr">
-        <is>
-          <t>390TL</t>
-        </is>
-      </c>
-      <c r="E76" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F76" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G76" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H76" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I76" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="10" t="inlineStr">
-        <is>
-          <t>Bakiye Sorma - Yurtiçi - ATM</t>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Mevduat Araştırma</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>Referans Mektubu -</t>
+        </is>
+      </c>
+      <c r="B78" s="21" t="inlineStr">
+        <is>
+          <t>4000.00TL</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D78" s="21" t="inlineStr">
+        <is>
+          <t>770TL</t>
+        </is>
+      </c>
+      <c r="E78" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G78" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H78" s="21" t="inlineStr">
+        <is>
+          <t>50 TL / -</t>
+        </is>
+      </c>
+      <c r="I78" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="11" t="inlineStr">
         <is>
+          <t>Hesap Özeti Verilmesi -</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D79" s="21" t="inlineStr">
+        <is>
+          <t>190TL</t>
+        </is>
+      </c>
+      <c r="E79" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F79" s="21" t="inlineStr">
+        <is>
+          <t>12 TL</t>
+        </is>
+      </c>
+      <c r="G79" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H79" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I79" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>Borcu Yoktur Yazısı</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>390TL</t>
+        </is>
+      </c>
+      <c r="E80" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G80" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I80" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
-      <c r="B79" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D79" s="21" t="inlineStr">
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>Bakiye Sorma - Yurtiçi - ATM</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C83" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D83" s="21" t="inlineStr">
         <is>
           <t>0.41TL</t>
         </is>
       </c>
-      <c r="E79" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F79" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G79" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H79" s="21" t="inlineStr">
+      <c r="E83" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F83" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G83" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H83" s="21" t="inlineStr">
         <is>
           <t>- / -</t>
         </is>
       </c>
-      <c r="I79" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="10" t="inlineStr">
+      <c r="I83" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>Bakiye Sorma - Yurtdışı - ATM</t>
-        </is>
-      </c>
-      <c r="B82" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C82" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D82" s="21" t="inlineStr">
-        <is>
-          <t>0.45EUR</t>
-        </is>
-      </c>
-      <c r="E82" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F82" s="21" t="inlineStr">
-        <is>
-          <t>0.27 TL</t>
-        </is>
-      </c>
-      <c r="G82" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H82" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I82" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="A84" s="10" t="inlineStr">
-        <is>
-          <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="11" t="inlineStr">
-        <is>
-          <t>Çek Düzenleme -</t>
-        </is>
-      </c>
-      <c r="B85" s="21" t="inlineStr">
-        <is>
-          <t>9.52TL / 0.10%</t>
-        </is>
-      </c>
-      <c r="C85" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D85" s="21" t="inlineStr">
-        <is>
-          <t>290TL / 1.10%</t>
-        </is>
-      </c>
-      <c r="E85" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F85" s="21" t="inlineStr">
-        <is>
-          <t>761,90 TL</t>
-        </is>
-      </c>
-      <c r="G85" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H85" s="21" t="inlineStr">
-        <is>
-          <t>104,76 TL / -</t>
-        </is>
-      </c>
-      <c r="I85" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>Çek Defteri (Yaprak Başı) -</t>
+          <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -3107,9 +3194,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D86" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D86" s="21" t="inlineStr">
+        <is>
+          <t>0.45EUR</t>
         </is>
       </c>
       <c r="E86" s="15" t="inlineStr">
@@ -3117,9 +3204,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F86" s="16" t="inlineStr">
-        <is>
-          <t>2.380,95 TL</t>
+      <c r="F86" s="21" t="inlineStr">
+        <is>
+          <t>0.27 TL</t>
         </is>
       </c>
       <c r="G86" s="17" t="inlineStr">
@@ -3141,423 +3228,423 @@
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>Çek İade Ücreti</t>
+          <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
         </is>
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="11" t="inlineStr">
         <is>
+          <t>Çek Düzenleme -</t>
+        </is>
+      </c>
+      <c r="B89" s="21" t="inlineStr">
+        <is>
+          <t>9.52TL / 0.10%</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D89" s="21" t="inlineStr">
+        <is>
+          <t>290TL / 1.10%</t>
+        </is>
+      </c>
+      <c r="E89" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F89" s="21" t="inlineStr">
+        <is>
+          <t>761,90 TL</t>
+        </is>
+      </c>
+      <c r="G89" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H89" s="21" t="inlineStr">
+        <is>
+          <t>104,76 TL / -</t>
+        </is>
+      </c>
+      <c r="I89" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>Çek Defteri (Yaprak Başı) -</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E90" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>2.380,95 TL</t>
+        </is>
+      </c>
+      <c r="G90" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I90" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
           <t>Çek İade Ücreti</t>
-        </is>
-      </c>
-      <c r="B89" s="21" t="inlineStr">
-        <is>
-          <t>171.43TL</t>
-        </is>
-      </c>
-      <c r="C89" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D89" s="21" t="inlineStr">
-        <is>
-          <t>390TL</t>
-        </is>
-      </c>
-      <c r="E89" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F89" s="21" t="inlineStr">
-        <is>
-          <t>380,95 TL</t>
-        </is>
-      </c>
-      <c r="G89" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H89" s="21" t="inlineStr">
-        <is>
-          <t>123,81 TL / -</t>
-        </is>
-      </c>
-      <c r="I89" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="10" t="inlineStr">
-        <is>
-          <t>Çek Tahsilat Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="11" t="inlineStr">
-        <is>
-          <t>Çek Tahsilat</t>
-        </is>
-      </c>
-      <c r="B92" s="21" t="inlineStr">
-        <is>
-          <t>45USD</t>
-        </is>
-      </c>
-      <c r="C92" s="21" t="inlineStr">
-        <is>
-          <t>590.48TL / 0.77%</t>
-        </is>
-      </c>
-      <c r="D92" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E92" s="21" t="inlineStr">
-        <is>
-          <t>1.70%</t>
-        </is>
-      </c>
-      <c r="F92" s="21" t="inlineStr">
-        <is>
-          <t>714,29 TL</t>
-        </is>
-      </c>
-      <c r="G92" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H92" s="21" t="inlineStr">
-        <is>
-          <t>260 TL / -</t>
-        </is>
-      </c>
-      <c r="I92" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
         </is>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="11" t="inlineStr">
         <is>
+          <t>Çek İade Ücreti</t>
+        </is>
+      </c>
+      <c r="B93" s="21" t="inlineStr">
+        <is>
+          <t>171.43TL</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D93" s="21" t="inlineStr">
+        <is>
+          <t>390TL</t>
+        </is>
+      </c>
+      <c r="E93" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F93" s="21" t="inlineStr">
+        <is>
+          <t>380,95 TL</t>
+        </is>
+      </c>
+      <c r="G93" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H93" s="21" t="inlineStr">
+        <is>
+          <t>123,81 TL / -</t>
+        </is>
+      </c>
+      <c r="I93" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t>Çek Tahsilat Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>Çek Tahsilat</t>
+        </is>
+      </c>
+      <c r="B96" s="21" t="inlineStr">
+        <is>
+          <t>45USD</t>
+        </is>
+      </c>
+      <c r="C96" s="21" t="inlineStr">
+        <is>
+          <t>590.48TL / 0.77%</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E96" s="21" t="inlineStr">
+        <is>
+          <t>1.70%</t>
+        </is>
+      </c>
+      <c r="F96" s="21" t="inlineStr">
+        <is>
+          <t>714,29 TL</t>
+        </is>
+      </c>
+      <c r="G96" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H96" s="21" t="inlineStr">
+        <is>
+          <t>260 TL / -</t>
+        </is>
+      </c>
+      <c r="I96" s="21" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="11" t="inlineStr">
+        <is>
           <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
         </is>
       </c>
-      <c r="B93" s="21" t="inlineStr">
+      <c r="B97" s="21" t="inlineStr">
         <is>
           <t>257.15TL</t>
         </is>
       </c>
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D93" s="21" t="inlineStr">
+      <c r="C97" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D97" s="21" t="inlineStr">
         <is>
           <t>2940TL / 1%</t>
         </is>
       </c>
-      <c r="E93" s="21" t="inlineStr">
+      <c r="E97" s="21" t="inlineStr">
         <is>
           <t>390TL / 0.2%</t>
         </is>
       </c>
-      <c r="F93" s="21" t="inlineStr">
+      <c r="F97" s="21" t="inlineStr">
         <is>
           <t>1.666,67 TL</t>
         </is>
       </c>
-      <c r="G93" s="21" t="inlineStr">
+      <c r="G97" s="21" t="inlineStr">
         <is>
           <t>585,71 TL</t>
         </is>
       </c>
-      <c r="H93" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I93" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="11" t="inlineStr">
-        <is>
-          <t>Diğer Banka Çeki -</t>
-        </is>
-      </c>
-      <c r="B94" s="21" t="inlineStr">
-        <is>
-          <t>390.48TL</t>
-        </is>
-      </c>
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D94" s="21" t="inlineStr">
-        <is>
-          <t>350TL</t>
-        </is>
-      </c>
-      <c r="E94" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F94" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G94" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H94" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I94" s="19" t="inlineStr">
-        <is>
-          <t>576,19 TL / 0,6</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="A95" s="11" t="inlineStr">
-        <is>
-          <t>Aynı Banka Çeki -</t>
-        </is>
-      </c>
-      <c r="B95" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C95" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D95" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E95" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F95" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G95" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H95" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I95" s="19" t="inlineStr">
-        <is>
-          <t>427,62 TL / -</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="10" t="inlineStr">
-        <is>
-          <t>Çek Belgelendirme ve Düzeltme Ücreti</t>
+      <c r="H97" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I97" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="11" t="inlineStr">
         <is>
+          <t>Diğer Banka Çeki -</t>
+        </is>
+      </c>
+      <c r="B98" s="21" t="inlineStr">
+        <is>
+          <t>390.48TL</t>
+        </is>
+      </c>
+      <c r="C98" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D98" s="21" t="inlineStr">
+        <is>
+          <t>350TL</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F98" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G98" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H98" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I98" s="19" t="inlineStr">
+        <is>
+          <t>576,19 TL / 0,6</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="11" t="inlineStr">
+        <is>
+          <t>Aynı Banka Çeki -</t>
+        </is>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E99" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F99" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G99" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H99" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I99" s="19" t="inlineStr">
+        <is>
+          <t>427,62 TL / -</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>Çek Belgelendirme ve Düzeltme Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="11" t="inlineStr">
+        <is>
           <t>Karşılıksız Çek Belgelendirme -</t>
         </is>
       </c>
-      <c r="B98" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C98" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D98" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E98" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F98" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G98" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H98" s="18" t="inlineStr">
+      <c r="B102" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C102" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E102" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F102" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G102" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H102" s="18" t="inlineStr">
         <is>
           <t>371,43 TL / -</t>
         </is>
       </c>
-      <c r="I98" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="18" customHeight="1">
-      <c r="A100" s="10" t="inlineStr">
+      <c r="I102" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="10" t="inlineStr">
         <is>
           <t>Senet İade Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="20" customHeight="1">
-      <c r="A101" s="11" t="inlineStr">
-        <is>
-          <t>Senet İade Ücreti</t>
-        </is>
-      </c>
-      <c r="B101" s="21" t="inlineStr">
-        <is>
-          <t>495.24TL</t>
-        </is>
-      </c>
-      <c r="C101" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D101" s="21" t="inlineStr">
-        <is>
-          <t>780TL</t>
-        </is>
-      </c>
-      <c r="E101" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F101" s="21" t="inlineStr">
-        <is>
-          <t>571,43 TL</t>
-        </is>
-      </c>
-      <c r="G101" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H101" s="21" t="inlineStr">
-        <is>
-          <t>600 TL / -</t>
-        </is>
-      </c>
-      <c r="I101" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="10" t="inlineStr">
-        <is>
-          <t>Senet Protesto İşlemleri Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="20" customHeight="1">
-      <c r="A104" s="11" t="inlineStr">
-        <is>
-          <t>Senet Protesto Kaldırma -</t>
-        </is>
-      </c>
-      <c r="B104" s="21" t="inlineStr">
-        <is>
-          <t>533.34TL</t>
-        </is>
-      </c>
-      <c r="C104" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D104" s="21" t="inlineStr">
-        <is>
-          <t>780TL</t>
-        </is>
-      </c>
-      <c r="E104" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F104" s="21" t="inlineStr">
-        <is>
-          <t>619,05 TL</t>
-        </is>
-      </c>
-      <c r="G104" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H104" s="21" t="inlineStr">
-        <is>
-          <t>551,43 TL / -</t>
-        </is>
-      </c>
-      <c r="I104" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="11" t="inlineStr">
         <is>
-          <t>Senet Protesto -</t>
+          <t>Senet İade Ücreti</t>
         </is>
       </c>
       <c r="B105" s="21" t="inlineStr">
         <is>
-          <t>600.00TL</t>
+          <t>495.24TL</t>
         </is>
       </c>
       <c r="C105" s="13" t="inlineStr">
@@ -3577,7 +3664,7 @@
       </c>
       <c r="F105" s="21" t="inlineStr">
         <is>
-          <t>666,67 TL</t>
+          <t>571,43 TL</t>
         </is>
       </c>
       <c r="G105" s="17" t="inlineStr">
@@ -3599,29 +3686,29 @@
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>Senet Tahsile Alma Ücreti</t>
+          <t>Senet Protesto İşlemleri Ücreti</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>Muhabir Banka Senet Tahsili -</t>
-        </is>
-      </c>
-      <c r="B108" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>Senet Protesto Kaldırma -</t>
+        </is>
+      </c>
+      <c r="B108" s="21" t="inlineStr">
+        <is>
+          <t>533.34TL</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>600.00TL</t>
-        </is>
-      </c>
-      <c r="D108" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D108" s="21" t="inlineStr">
+        <is>
+          <t>780TL</t>
         </is>
       </c>
       <c r="E108" s="15" t="inlineStr">
@@ -3631,7 +3718,7 @@
       </c>
       <c r="F108" s="21" t="inlineStr">
         <is>
-          <t>666,67 TL</t>
+          <t>619,05 TL</t>
         </is>
       </c>
       <c r="G108" s="17" t="inlineStr">
@@ -3641,7 +3728,7 @@
       </c>
       <c r="H108" s="21" t="inlineStr">
         <is>
-          <t>600 TL / -</t>
+          <t>551,43 TL / -</t>
         </is>
       </c>
       <c r="I108" s="19" t="inlineStr">
@@ -3653,12 +3740,12 @@
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="11" t="inlineStr">
         <is>
-          <t>Aynı Banka Senet Tahsili -</t>
-        </is>
-      </c>
-      <c r="B109" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>Senet Protesto -</t>
+        </is>
+      </c>
+      <c r="B109" s="21" t="inlineStr">
+        <is>
+          <t>600.00TL</t>
         </is>
       </c>
       <c r="C109" s="13" t="inlineStr">
@@ -3666,9 +3753,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D109" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D109" s="21" t="inlineStr">
+        <is>
+          <t>780TL</t>
         </is>
       </c>
       <c r="E109" s="15" t="inlineStr">
@@ -3676,9 +3763,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F109" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F109" s="21" t="inlineStr">
+        <is>
+          <t>666,67 TL</t>
         </is>
       </c>
       <c r="G109" s="17" t="inlineStr">
@@ -3686,7 +3773,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H109" s="18" t="inlineStr">
+      <c r="H109" s="21" t="inlineStr">
         <is>
           <t>600 TL / -</t>
         </is>
@@ -3700,61 +3787,162 @@
     <row r="111" ht="18" customHeight="1">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>HGS</t>
+          <t>Senet Tahsile Alma Ücreti</t>
         </is>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="11" t="inlineStr">
         <is>
+          <t>Muhabir Banka Senet Tahsili -</t>
+        </is>
+      </c>
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C112" s="13" t="inlineStr">
+        <is>
+          <t>600.00TL</t>
+        </is>
+      </c>
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E112" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F112" s="21" t="inlineStr">
+        <is>
+          <t>666,67 TL</t>
+        </is>
+      </c>
+      <c r="G112" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H112" s="21" t="inlineStr">
+        <is>
+          <t>600 TL / -</t>
+        </is>
+      </c>
+      <c r="I112" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="11" t="inlineStr">
+        <is>
+          <t>Aynı Banka Senet Tahsili -</t>
+        </is>
+      </c>
+      <c r="B113" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C113" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E113" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F113" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G113" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H113" s="18" t="inlineStr">
+        <is>
+          <t>600 TL / -</t>
+        </is>
+      </c>
+      <c r="I113" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>HGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
           <t>HGS Kart Ücreti</t>
         </is>
       </c>
-      <c r="B112" s="21" t="inlineStr">
+      <c r="B116" s="21" t="inlineStr">
         <is>
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="C112" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D112" s="21" t="inlineStr">
+      <c r="C116" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D116" s="21" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="E112" s="15" t="inlineStr">
+      <c r="E116" s="15" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="F112" s="21" t="inlineStr">
+      <c r="F116" s="21" t="inlineStr">
         <is>
           <t>500 TL</t>
         </is>
       </c>
-      <c r="G112" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H112" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I112" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="22" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 14.08.2026 11:11</t>
+      <c r="G116" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H116" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I116" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="22" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 14.08.2026 11:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 15:13)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1333,14 +1333,14 @@
           <t>19,94 TL</t>
         </is>
       </c>
-      <c r="H18" s="21" t="inlineStr">
-        <is>
-          <t>13,33 TL / -</t>
-        </is>
-      </c>
-      <c r="I18" s="21" t="inlineStr">
-        <is>
-          <t>19,94 TL / -</t>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1380,14 +1380,14 @@
           <t>39,88 TL</t>
         </is>
       </c>
-      <c r="H19" s="21" t="inlineStr">
-        <is>
-          <t>27,62 TL / -</t>
-        </is>
-      </c>
-      <c r="I19" s="21" t="inlineStr">
-        <is>
-          <t>39,88 TL / -</t>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1427,14 +1427,14 @@
           <t>398,84 TL</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr">
-        <is>
-          <t>199,05 TL / -</t>
-        </is>
-      </c>
-      <c r="I20" s="21" t="inlineStr">
-        <is>
-          <t>398,84 TL / -</t>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
           <t>FAST - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
@@ -1528,9 +1528,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr">
-        <is>
-          <t>7,97 TL / -</t>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I24" s="19" t="inlineStr">
@@ -1592,7 +1592,7 @@
           <t>FAST - 8300-399000 TRY</t>
         </is>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
@@ -1622,9 +1622,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H26" s="21" t="inlineStr">
-        <is>
-          <t>15,96 TL / -</t>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I26" s="19" t="inlineStr">
@@ -1633,69 +1633,69 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>FAST</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G27" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H27" s="18" t="inlineStr">
-        <is>
-          <t>200 TL / 0,4</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Kiralık Kasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Yıllık Kasa Ücreti - büyük</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>30000.00TL</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="inlineStr">
+        <is>
+          <t>4140TL</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H29" s="21" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - büyük</t>
+          <t>Yıllık Kasa Ücreti - küçük</t>
         </is>
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>30000.00TL</t>
+          <t>22000.00TL</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
-          <t>4140TL</t>
+          <t>2610TL</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -1737,12 +1737,12 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - küçük</t>
+          <t>Yıllık Kasa Ücreti - orta</t>
         </is>
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>22000.00TL</t>
+          <t>25000.00TL</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
-          <t>2610TL</t>
+          <t>3390TL</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -1784,12 +1784,12 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - orta</t>
+          <t>Kasa Depozito - büyük</t>
         </is>
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>25000.00TL</t>
+          <t>28570.00TL</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1797,9 +1797,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D32" s="21" t="inlineStr">
-        <is>
-          <t>3390TL</t>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -1831,12 +1831,12 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - büyük</t>
+          <t>Kasa Depozito - orta</t>
         </is>
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>28570.00TL</t>
+          <t>23805.00TL</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1878,12 +1878,12 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - orta</t>
+          <t>Kasa Depozito - küçük</t>
         </is>
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>23805.00TL</t>
+          <t>20950.00TL</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1925,12 +1925,12 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - küçük</t>
-        </is>
-      </c>
-      <c r="B35" s="21" t="inlineStr">
-        <is>
-          <t>20950.00TL</t>
+          <t>Yıllık Kasa Ücreti - genel</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>1469.52TL</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1958,9 +1958,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H35" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H35" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
@@ -1972,12 +1972,12 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - genel</t>
+          <t>Kasa Depozito - genel</t>
         </is>
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>1469.52TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>9420TL</t>
         </is>
       </c>
       <c r="E36" s="15" t="inlineStr">
@@ -2019,7 +2019,7 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - genel</t>
+          <t>Kasa Depozito - 0-8300</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>9420TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E37" s="15" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>- / -</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
@@ -2063,69 +2063,69 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Yıllık Kasa Ücreti - 0-8300</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H38" s="18" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
+      <c r="I38" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Kıymetli Maden</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>Altın Transfer - 0-8300</t>
-        </is>
-      </c>
-      <c r="B40" s="21" t="inlineStr">
-        <is>
-          <t>50.00TL</t>
-        </is>
-      </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D40" s="21" t="inlineStr">
-        <is>
-          <t>3.25%</t>
-        </is>
-      </c>
-      <c r="E40" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F40" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G40" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H40" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I40" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 8300-399000</t>
+          <t>Altın Transfer - 0-8300</t>
         </is>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>100.00TL</t>
+          <t>50.00TL</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="D41" s="21" t="inlineStr">
         <is>
-          <t>170TL</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr">
@@ -2167,12 +2167,12 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer</t>
-        </is>
-      </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>Altın Transfer - 8300-399000</t>
+        </is>
+      </c>
+      <c r="B42" s="21" t="inlineStr">
+        <is>
+          <t>100.00TL</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -2180,9 +2180,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D42" s="14" t="inlineStr">
-        <is>
-          <t>10%</t>
+      <c r="D42" s="21" t="inlineStr">
+        <is>
+          <t>170TL</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr">
@@ -2214,7 +2214,7 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 1-10gr</t>
+          <t>Altın Transfer</t>
         </is>
       </c>
       <c r="B43" s="12" t="inlineStr">
@@ -2229,17 +2229,17 @@
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>57,5TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>60 TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G43" s="17" t="inlineStr">
@@ -2261,7 +2261,7 @@
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 11-100gr</t>
+          <t>Altın Transfer - 1-10gr</t>
         </is>
       </c>
       <c r="B44" s="12" t="inlineStr">
@@ -2281,12 +2281,12 @@
       </c>
       <c r="E44" s="15" t="inlineStr">
         <is>
-          <t>115TL</t>
+          <t>57,5TL</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>120 TL</t>
+          <t>60 TL</t>
         </is>
       </c>
       <c r="G44" s="17" t="inlineStr">
@@ -2308,454 +2308,454 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
+          <t>Altın Transfer - 11-100gr</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>115TL</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>120 TL</t>
+        </is>
+      </c>
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H45" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I45" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
           <t>Altın Transfer - 399000+</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D45" s="21" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D46" s="21" t="inlineStr">
         <is>
           <t>415TL</t>
         </is>
       </c>
-      <c r="E45" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F45" s="21" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F46" s="21" t="inlineStr">
         <is>
           <t>0.00018</t>
         </is>
       </c>
-      <c r="G45" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H45" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I45" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="G46" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H46" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I46" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="11" t="inlineStr">
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
-      <c r="B48" s="21" t="inlineStr">
+      <c r="B49" s="21" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
+      <c r="C49" s="13" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="D48" s="21" t="inlineStr">
+      <c r="D49" s="21" t="inlineStr">
         <is>
           <t>95TL</t>
         </is>
       </c>
-      <c r="E48" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F48" s="21" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F49" s="21" t="inlineStr">
         <is>
           <t>65 TL</t>
         </is>
       </c>
-      <c r="G48" s="17" t="inlineStr">
+      <c r="G49" s="17" t="inlineStr">
         <is>
           <t>95,24 TL</t>
         </is>
       </c>
-      <c r="H48" s="21" t="inlineStr">
-        <is>
-          <t>339 TL / -</t>
-        </is>
-      </c>
-      <c r="I48" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="H49" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I49" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri - Kart</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri</t>
         </is>
       </c>
-      <c r="B51" s="21" t="inlineStr">
+      <c r="B52" s="21" t="inlineStr">
         <is>
           <t>5.00TL / 3.50%</t>
         </is>
       </c>
-      <c r="C51" s="21" t="inlineStr">
+      <c r="C52" s="21" t="inlineStr">
         <is>
           <t>0.00TL</t>
         </is>
       </c>
-      <c r="D51" s="21" t="inlineStr">
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E51" s="21" t="inlineStr">
+      <c r="E52" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="F51" s="21" t="inlineStr">
+      <c r="F52" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="G51" s="21" t="inlineStr">
+      <c r="G52" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="H51" s="21" t="inlineStr">
-        <is>
-          <t>0,63 TL / -</t>
-        </is>
-      </c>
-      <c r="I51" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L51" s="20" t="inlineStr">
+      <c r="H52" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I52" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L52" s="20" t="inlineStr">
         <is>
           <t>Fatura ödemeleri üst tier için %3,5'a çıkabiliyor</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="L52" s="20" t="inlineStr">
+    <row r="53">
+      <c r="L53" s="20" t="inlineStr">
         <is>
           <t>Borcu Yoktur Yazısı almak için ücret alınabiliyor</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="10" t="inlineStr">
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
-      <c r="L53" s="20" t="inlineStr">
+      <c r="L54" s="20" t="inlineStr">
         <is>
           <t>Mevduat Araştırma Ücretleri zamlanabilir</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
-      <c r="B54" s="21" t="inlineStr">
+      <c r="B55" s="21" t="inlineStr">
         <is>
           <t>3.50TL / 3.50%</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D54" s="21" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F54" s="21" t="inlineStr">
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F55" s="21" t="inlineStr">
         <is>
           <t>2 TL / 3,5%</t>
         </is>
       </c>
-      <c r="G54" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H54" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I54" s="19" t="inlineStr">
-        <is>
-          <t>3 TL / -</t>
-        </is>
-      </c>
-      <c r="L54" s="20" t="inlineStr">
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I55" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L55" s="20" t="inlineStr">
         <is>
           <t>Güvenli Araç Alım Satım YKB 97,53 TRY</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="10" t="inlineStr">
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="11" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>275.00TL</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="E57" s="15" t="inlineStr">
+      <c r="E58" s="15" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="F57" s="16" t="inlineStr">
+      <c r="F58" s="16" t="inlineStr">
         <is>
           <t>275 TL</t>
         </is>
       </c>
-      <c r="G57" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H57" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
+      <c r="G58" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H58" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I58" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="10" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="11" t="inlineStr">
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D60" s="21" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D61" s="21" t="inlineStr">
         <is>
           <t>26TL</t>
         </is>
       </c>
-      <c r="E60" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F60" s="21" t="inlineStr">
+      <c r="E61" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="inlineStr">
         <is>
           <t>38,10 TL</t>
         </is>
       </c>
-      <c r="G60" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H60" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I60" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="10" t="inlineStr">
+      <c r="G61" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H61" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="10" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="11" t="inlineStr">
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="11" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D63" s="14" t="inlineStr">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E63" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F63" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G63" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H63" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="10" t="inlineStr">
+      <c r="E64" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G64" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H64" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I64" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>Telefon Ödemeleri Aracılık</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>Telefon - 0-8300 TRY</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C66" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D66" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E66" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F66" s="16" t="inlineStr">
-        <is>
-          <t>3,99 TL</t>
-        </is>
-      </c>
-      <c r="G66" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H66" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I66" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>Telefon - 8300-399000 TRY</t>
+          <t>Telefon - 0-8300 TRY</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>7,98 TL</t>
+          <t>3,99 TL</t>
         </is>
       </c>
       <c r="G67" s="17" t="inlineStr">
@@ -2802,7 +2802,7 @@
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>Telefon - 399000+ TRY</t>
+          <t>Telefon - 8300-399000 TRY</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="F68" s="16" t="inlineStr">
         <is>
-          <t>99,71 TL</t>
+          <t>7,98 TL</t>
         </is>
       </c>
       <c r="G68" s="17" t="inlineStr">
@@ -2849,189 +2849,189 @@
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="11" t="inlineStr">
         <is>
+          <t>Telefon - 399000+ TRY</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>99,71 TL</t>
+        </is>
+      </c>
+      <c r="G69" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H69" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I69" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
           <t>Telefon Ödemeleri</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C69" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D69" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E69" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F69" s="16" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F70" s="16" t="inlineStr">
         <is>
           <t>1 %</t>
         </is>
       </c>
-      <c r="G69" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H69" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I69" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="10" t="inlineStr">
+      <c r="G70" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H70" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I70" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="10" t="inlineStr">
         <is>
           <t>Vergi Tahsilat Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="11" t="inlineStr">
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="11" t="inlineStr">
         <is>
           <t>Vergi Tahsilat</t>
         </is>
       </c>
-      <c r="B72" s="12" t="inlineStr"/>
-      <c r="C72" s="13" t="inlineStr"/>
-      <c r="D72" s="14" t="inlineStr"/>
-      <c r="E72" s="15" t="inlineStr"/>
-      <c r="F72" s="16" t="inlineStr"/>
-      <c r="G72" s="17" t="inlineStr"/>
-      <c r="H72" s="18" t="inlineStr"/>
-      <c r="I72" s="19" t="inlineStr"/>
-    </row>
-    <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="10" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr"/>
+      <c r="C73" s="13" t="inlineStr"/>
+      <c r="D73" s="14" t="inlineStr"/>
+      <c r="E73" s="15" t="inlineStr"/>
+      <c r="F73" s="16" t="inlineStr"/>
+      <c r="G73" s="17" t="inlineStr"/>
+      <c r="H73" s="18" t="inlineStr"/>
+      <c r="I73" s="19" t="inlineStr"/>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="10" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="11" t="inlineStr">
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="11" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr">
+      <c r="B76" s="12" t="inlineStr">
         <is>
           <t>287.62TL</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D75" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E75" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F75" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G75" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H75" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I75" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="10" t="inlineStr">
+      <c r="C76" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D76" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F76" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G76" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H76" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I76" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="10" t="inlineStr">
         <is>
           <t>Mevduat Araştırma</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="11" t="inlineStr">
-        <is>
-          <t>Referans Mektubu -</t>
-        </is>
-      </c>
-      <c r="B78" s="21" t="inlineStr">
-        <is>
-          <t>4000.00TL</t>
-        </is>
-      </c>
-      <c r="C78" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D78" s="21" t="inlineStr">
-        <is>
-          <t>770TL</t>
-        </is>
-      </c>
-      <c r="E78" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F78" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G78" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H78" s="21" t="inlineStr">
-        <is>
-          <t>50 TL / -</t>
-        </is>
-      </c>
-      <c r="I78" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="11" t="inlineStr">
         <is>
-          <t>Hesap Özeti Verilmesi -</t>
-        </is>
-      </c>
-      <c r="B79" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>Referans Mektubu -</t>
+        </is>
+      </c>
+      <c r="B79" s="21" t="inlineStr">
+        <is>
+          <t>4000.00TL</t>
         </is>
       </c>
       <c r="C79" s="13" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="D79" s="21" t="inlineStr">
         <is>
-          <t>190TL</t>
+          <t>770TL</t>
         </is>
       </c>
       <c r="E79" s="15" t="inlineStr">
@@ -3049,9 +3049,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F79" s="21" t="inlineStr">
-        <is>
-          <t>12 TL</t>
+      <c r="F79" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G79" s="17" t="inlineStr">
@@ -3073,401 +3073,401 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="11" t="inlineStr">
         <is>
+          <t>Hesap Özeti Verilmesi -</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D80" s="21" t="inlineStr">
+        <is>
+          <t>190TL</t>
+        </is>
+      </c>
+      <c r="E80" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F80" s="21" t="inlineStr">
+        <is>
+          <t>12 TL</t>
+        </is>
+      </c>
+      <c r="G80" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I80" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
           <t>Borcu Yoktur Yazısı</t>
         </is>
       </c>
-      <c r="B80" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C80" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D80" s="14" t="inlineStr">
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E80" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F80" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G80" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H80" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I80" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="10" t="inlineStr">
+      <c r="E81" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G81" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I81" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="20" customHeight="1">
-      <c r="A83" s="11" t="inlineStr">
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="11" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
-      <c r="B83" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C83" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D83" s="21" t="inlineStr">
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C84" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
         <is>
           <t>0.41TL</t>
         </is>
       </c>
-      <c r="E83" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F83" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G83" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H83" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
-      <c r="I83" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="10" t="inlineStr">
+      <c r="E84" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F84" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G84" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H84" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I84" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="A86" s="11" t="inlineStr">
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="11" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
-      <c r="B86" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C86" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D86" s="21" t="inlineStr">
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D87" s="21" t="inlineStr">
         <is>
           <t>0.45EUR</t>
         </is>
       </c>
-      <c r="E86" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F86" s="21" t="inlineStr">
+      <c r="E87" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F87" s="21" t="inlineStr">
         <is>
           <t>0.27 TL</t>
         </is>
       </c>
-      <c r="G86" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H86" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I86" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="10" t="inlineStr">
+      <c r="G87" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H87" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I87" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="10" t="inlineStr">
         <is>
           <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="20" customHeight="1">
-      <c r="A89" s="11" t="inlineStr">
-        <is>
-          <t>Çek Düzenleme -</t>
-        </is>
-      </c>
-      <c r="B89" s="21" t="inlineStr">
-        <is>
-          <t>9.52TL / 0.10%</t>
-        </is>
-      </c>
-      <c r="C89" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D89" s="21" t="inlineStr">
-        <is>
-          <t>290TL / 1.10%</t>
-        </is>
-      </c>
-      <c r="E89" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F89" s="21" t="inlineStr">
-        <is>
-          <t>761,90 TL</t>
-        </is>
-      </c>
-      <c r="G89" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H89" s="21" t="inlineStr">
-        <is>
-          <t>104,76 TL / -</t>
-        </is>
-      </c>
-      <c r="I89" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
+          <t>Çek Düzenleme -</t>
+        </is>
+      </c>
+      <c r="B90" s="21" t="inlineStr">
+        <is>
+          <t>9.52TL / 0.10%</t>
+        </is>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D90" s="21" t="inlineStr">
+        <is>
+          <t>290TL / 1.10%</t>
+        </is>
+      </c>
+      <c r="E90" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F90" s="21" t="inlineStr">
+        <is>
+          <t>761,90 TL</t>
+        </is>
+      </c>
+      <c r="G90" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I90" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
           <t>Çek Defteri (Yaprak Başı) -</t>
         </is>
       </c>
-      <c r="B90" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C90" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D90" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E90" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F90" s="16" t="inlineStr">
+      <c r="B91" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C91" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E91" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F91" s="16" t="inlineStr">
         <is>
           <t>2.380,95 TL</t>
         </is>
       </c>
-      <c r="G90" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H90" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I90" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="10" t="inlineStr">
+      <c r="G91" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H91" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I91" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="10" t="inlineStr">
         <is>
           <t>Çek İade Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="20" customHeight="1">
-      <c r="A93" s="11" t="inlineStr">
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="11" t="inlineStr">
         <is>
           <t>Çek İade Ücreti</t>
         </is>
       </c>
-      <c r="B93" s="21" t="inlineStr">
+      <c r="B94" s="21" t="inlineStr">
         <is>
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D93" s="21" t="inlineStr">
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D94" s="21" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E93" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F93" s="21" t="inlineStr">
+      <c r="E94" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F94" s="21" t="inlineStr">
         <is>
           <t>380,95 TL</t>
         </is>
       </c>
-      <c r="G93" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H93" s="21" t="inlineStr">
-        <is>
-          <t>123,81 TL / -</t>
-        </is>
-      </c>
-      <c r="I93" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="10" t="inlineStr">
+      <c r="G94" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H94" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I94" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="10" t="inlineStr">
         <is>
           <t>Çek Tahsilat Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="11" t="inlineStr">
-        <is>
-          <t>Çek Tahsilat</t>
-        </is>
-      </c>
-      <c r="B96" s="21" t="inlineStr">
-        <is>
-          <t>45USD</t>
-        </is>
-      </c>
-      <c r="C96" s="21" t="inlineStr">
-        <is>
-          <t>590.48TL / 0.77%</t>
-        </is>
-      </c>
-      <c r="D96" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E96" s="21" t="inlineStr">
-        <is>
-          <t>1.70%</t>
-        </is>
-      </c>
-      <c r="F96" s="21" t="inlineStr">
-        <is>
-          <t>714,29 TL</t>
-        </is>
-      </c>
-      <c r="G96" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H96" s="21" t="inlineStr">
-        <is>
-          <t>260 TL / -</t>
-        </is>
-      </c>
-      <c r="I96" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
         </is>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="11" t="inlineStr">
         <is>
-          <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
+          <t>Çek Tahsilat</t>
         </is>
       </c>
       <c r="B97" s="21" t="inlineStr">
         <is>
-          <t>257.15TL</t>
-        </is>
-      </c>
-      <c r="C97" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D97" s="21" t="inlineStr">
-        <is>
-          <t>2940TL / 1%</t>
+          <t>45USD</t>
+        </is>
+      </c>
+      <c r="C97" s="21" t="inlineStr">
+        <is>
+          <t>590.48TL / 0.77%</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E97" s="21" t="inlineStr">
         <is>
-          <t>390TL / 0.2%</t>
+          <t>1.70%</t>
         </is>
       </c>
       <c r="F97" s="21" t="inlineStr">
         <is>
-          <t>1.666,67 TL</t>
-        </is>
-      </c>
-      <c r="G97" s="21" t="inlineStr">
-        <is>
-          <t>585,71 TL</t>
+          <t>714,29 TL</t>
+        </is>
+      </c>
+      <c r="G97" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H97" s="18" t="inlineStr">
@@ -3484,12 +3484,12 @@
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>Diğer Banka Çeki -</t>
+          <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
         </is>
       </c>
       <c r="B98" s="21" t="inlineStr">
         <is>
-          <t>390.48TL</t>
+          <t>257.15TL</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -3499,22 +3499,22 @@
       </c>
       <c r="D98" s="21" t="inlineStr">
         <is>
-          <t>350TL</t>
-        </is>
-      </c>
-      <c r="E98" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F98" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G98" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>2940TL / 1%</t>
+        </is>
+      </c>
+      <c r="E98" s="21" t="inlineStr">
+        <is>
+          <t>390TL / 0.2%</t>
+        </is>
+      </c>
+      <c r="F98" s="21" t="inlineStr">
+        <is>
+          <t>1.666,67 TL</t>
+        </is>
+      </c>
+      <c r="G98" s="21" t="inlineStr">
+        <is>
+          <t>585,71 TL</t>
         </is>
       </c>
       <c r="H98" s="18" t="inlineStr">
@@ -3524,19 +3524,19 @@
       </c>
       <c r="I98" s="19" t="inlineStr">
         <is>
-          <t>576,19 TL / 0,6</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="11" t="inlineStr">
         <is>
-          <t>Aynı Banka Çeki -</t>
-        </is>
-      </c>
-      <c r="B99" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>Diğer Banka Çeki -</t>
+        </is>
+      </c>
+      <c r="B99" s="21" t="inlineStr">
+        <is>
+          <t>390.48TL</t>
         </is>
       </c>
       <c r="C99" s="13" t="inlineStr">
@@ -3544,9 +3544,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D99" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D99" s="21" t="inlineStr">
+        <is>
+          <t>350TL</t>
         </is>
       </c>
       <c r="E99" s="15" t="inlineStr">
@@ -3571,26 +3571,26 @@
       </c>
       <c r="I99" s="19" t="inlineStr">
         <is>
-          <t>427,62 TL / -</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>Çek Belgelendirme ve Düzeltme Ücreti</t>
+          <t>Senet İade Ücreti</t>
         </is>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>Karşılıksız Çek Belgelendirme -</t>
-        </is>
-      </c>
-      <c r="B102" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>Senet İade Ücreti</t>
+        </is>
+      </c>
+      <c r="B102" s="21" t="inlineStr">
+        <is>
+          <t>495.24TL</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -3598,9 +3598,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D102" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D102" s="21" t="inlineStr">
+        <is>
+          <t>780TL</t>
         </is>
       </c>
       <c r="E102" s="15" t="inlineStr">
@@ -3608,9 +3608,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F102" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F102" s="21" t="inlineStr">
+        <is>
+          <t>571,43 TL</t>
         </is>
       </c>
       <c r="G102" s="17" t="inlineStr">
@@ -3618,9 +3618,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H102" s="18" t="inlineStr">
-        <is>
-          <t>371,43 TL / -</t>
+      <c r="H102" s="21" t="inlineStr">
+        <is>
+          <t>123,81 TL / -</t>
         </is>
       </c>
       <c r="I102" s="19" t="inlineStr">
@@ -3632,19 +3632,19 @@
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Senet İade Ücreti</t>
+          <t>Senet Protesto İşlemleri Ücreti</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="11" t="inlineStr">
         <is>
-          <t>Senet İade Ücreti</t>
+          <t>Senet Protesto Kaldırma -</t>
         </is>
       </c>
       <c r="B105" s="21" t="inlineStr">
         <is>
-          <t>495.24TL</t>
+          <t>533.34TL</t>
         </is>
       </c>
       <c r="C105" s="13" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="F105" s="21" t="inlineStr">
         <is>
-          <t>571,43 TL</t>
+          <t>619,05 TL</t>
         </is>
       </c>
       <c r="G105" s="17" t="inlineStr">
@@ -3674,88 +3674,88 @@
       </c>
       <c r="H105" s="21" t="inlineStr">
         <is>
+          <t>551,43 TL / -</t>
+        </is>
+      </c>
+      <c r="I105" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="11" t="inlineStr">
+        <is>
+          <t>Senet Protesto -</t>
+        </is>
+      </c>
+      <c r="B106" s="21" t="inlineStr">
+        <is>
+          <t>600.00TL</t>
+        </is>
+      </c>
+      <c r="C106" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D106" s="21" t="inlineStr">
+        <is>
+          <t>780TL</t>
+        </is>
+      </c>
+      <c r="E106" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F106" s="21" t="inlineStr">
+        <is>
+          <t>666,67 TL</t>
+        </is>
+      </c>
+      <c r="G106" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H106" s="21" t="inlineStr">
+        <is>
           <t>600 TL / -</t>
         </is>
       </c>
-      <c r="I105" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="10" t="inlineStr">
-        <is>
-          <t>Senet Protesto İşlemleri Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="11" t="inlineStr">
-        <is>
-          <t>Senet Protesto Kaldırma -</t>
-        </is>
-      </c>
-      <c r="B108" s="21" t="inlineStr">
-        <is>
-          <t>533.34TL</t>
-        </is>
-      </c>
-      <c r="C108" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D108" s="21" t="inlineStr">
-        <is>
-          <t>780TL</t>
-        </is>
-      </c>
-      <c r="E108" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F108" s="21" t="inlineStr">
-        <is>
-          <t>619,05 TL</t>
-        </is>
-      </c>
-      <c r="G108" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H108" s="21" t="inlineStr">
-        <is>
-          <t>551,43 TL / -</t>
-        </is>
-      </c>
-      <c r="I108" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I106" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="10" t="inlineStr">
+        <is>
+          <t>Senet Tahsile Alma Ücreti</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="11" t="inlineStr">
         <is>
-          <t>Senet Protesto -</t>
-        </is>
-      </c>
-      <c r="B109" s="21" t="inlineStr">
+          <t>Muhabir Banka Senet Tahsili -</t>
+        </is>
+      </c>
+      <c r="B109" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C109" s="21" t="inlineStr">
         <is>
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="C109" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D109" s="21" t="inlineStr">
-        <is>
-          <t>780TL</t>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E109" s="15" t="inlineStr">
@@ -3775,78 +3775,78 @@
       </c>
       <c r="H109" s="21" t="inlineStr">
         <is>
+          <t>104,76 TL / -</t>
+        </is>
+      </c>
+      <c r="I109" s="21" t="inlineStr">
+        <is>
+          <t>576,19 TL / 0,6</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="11" t="inlineStr">
+        <is>
+          <t>Aynı Banka Senet Tahsili -</t>
+        </is>
+      </c>
+      <c r="B110" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C110" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E110" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F110" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G110" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H110" s="18" t="inlineStr">
+        <is>
           <t>600 TL / -</t>
         </is>
       </c>
-      <c r="I109" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="18" customHeight="1">
-      <c r="A111" s="10" t="inlineStr">
-        <is>
-          <t>Senet Tahsile Alma Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="A112" s="11" t="inlineStr">
-        <is>
-          <t>Muhabir Banka Senet Tahsili -</t>
-        </is>
-      </c>
-      <c r="B112" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C112" s="13" t="inlineStr">
-        <is>
-          <t>600.00TL</t>
-        </is>
-      </c>
-      <c r="D112" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E112" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F112" s="21" t="inlineStr">
-        <is>
-          <t>666,67 TL</t>
-        </is>
-      </c>
-      <c r="G112" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H112" s="21" t="inlineStr">
-        <is>
-          <t>600 TL / -</t>
-        </is>
-      </c>
-      <c r="I112" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I110" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>HGS</t>
         </is>
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="11" t="inlineStr">
         <is>
-          <t>Aynı Banka Senet Tahsili -</t>
-        </is>
-      </c>
-      <c r="B113" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>HGS Kart Ücreti</t>
+        </is>
+      </c>
+      <c r="B113" s="21" t="inlineStr">
+        <is>
+          <t>550.00TL</t>
         </is>
       </c>
       <c r="C113" s="13" t="inlineStr">
@@ -3854,19 +3854,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D113" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D113" s="21" t="inlineStr">
+        <is>
+          <t>550TL</t>
         </is>
       </c>
       <c r="E113" s="15" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F113" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>550TL</t>
+        </is>
+      </c>
+      <c r="F113" s="21" t="inlineStr">
+        <is>
+          <t>500 TL</t>
         </is>
       </c>
       <c r="G113" s="17" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="H113" s="18" t="inlineStr">
         <is>
-          <t>600 TL / -</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I113" s="19" t="inlineStr">
@@ -3885,64 +3885,10 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="10" t="inlineStr">
-        <is>
-          <t>HGS</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="11" t="inlineStr">
-        <is>
-          <t>HGS Kart Ücreti</t>
-        </is>
-      </c>
-      <c r="B116" s="21" t="inlineStr">
-        <is>
-          <t>550.00TL</t>
-        </is>
-      </c>
-      <c r="C116" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D116" s="21" t="inlineStr">
-        <is>
-          <t>550TL</t>
-        </is>
-      </c>
-      <c r="E116" s="15" t="inlineStr">
-        <is>
-          <t>550TL</t>
-        </is>
-      </c>
-      <c r="F116" s="21" t="inlineStr">
-        <is>
-          <t>500 TL</t>
-        </is>
-      </c>
-      <c r="G116" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H116" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I116" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="22" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 14.08.2026 14:56</t>
+    <row r="115">
+      <c r="A115" s="22" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 14.08.2026 15:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 15:31)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1333,14 +1333,14 @@
           <t>19,94 TL</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I18" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>13,33 TL / -</t>
+        </is>
+      </c>
+      <c r="I18" s="21" t="inlineStr">
+        <is>
+          <t>19,94 TL / -</t>
         </is>
       </c>
     </row>
@@ -1380,14 +1380,14 @@
           <t>39,88 TL</t>
         </is>
       </c>
-      <c r="H19" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>27,62 TL / -</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="inlineStr">
+        <is>
+          <t>39,88 TL / -</t>
         </is>
       </c>
     </row>
@@ -1427,14 +1427,14 @@
           <t>398,84 TL</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I20" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H20" s="21" t="inlineStr">
+        <is>
+          <t>199,05 TL / -</t>
+        </is>
+      </c>
+      <c r="I20" s="21" t="inlineStr">
+        <is>
+          <t>398,84 TL / -</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
           <t>FAST - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
@@ -1528,9 +1528,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>7,97 TL / -</t>
         </is>
       </c>
       <c r="I24" s="19" t="inlineStr">
@@ -1592,7 +1592,7 @@
           <t>FAST - 8300-399000 TRY</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
@@ -1622,9 +1622,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H26" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H26" s="21" t="inlineStr">
+        <is>
+          <t>15,96 TL / -</t>
         </is>
       </c>
       <c r="I26" s="19" t="inlineStr">
@@ -1633,69 +1633,69 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="inlineStr">
+        <is>
+          <t>200 TL / 0,4</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Kiralık Kasa</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>Yıllık Kasa Ücreti - büyük</t>
-        </is>
-      </c>
-      <c r="B29" s="21" t="inlineStr">
-        <is>
-          <t>30000.00TL</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D29" s="21" t="inlineStr">
-        <is>
-          <t>4140TL</t>
-        </is>
-      </c>
-      <c r="E29" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H29" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - küçük</t>
+          <t>Yıllık Kasa Ücreti - büyük</t>
         </is>
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>22000.00TL</t>
+          <t>30000.00TL</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
-          <t>2610TL</t>
+          <t>4140TL</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
@@ -1737,12 +1737,12 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - orta</t>
+          <t>Yıllık Kasa Ücreti - küçük</t>
         </is>
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>25000.00TL</t>
+          <t>22000.00TL</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
-          <t>3390TL</t>
+          <t>2610TL</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
@@ -1784,12 +1784,12 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - büyük</t>
+          <t>Yıllık Kasa Ücreti - orta</t>
         </is>
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>28570.00TL</t>
+          <t>25000.00TL</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -1797,9 +1797,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>3390TL</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -1831,12 +1831,12 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - orta</t>
+          <t>Kasa Depozito - büyük</t>
         </is>
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>23805.00TL</t>
+          <t>28570.00TL</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -1878,12 +1878,12 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - küçük</t>
+          <t>Kasa Depozito - orta</t>
         </is>
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>20950.00TL</t>
+          <t>23805.00TL</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1925,12 +1925,12 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - genel</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>1469.52TL</t>
+          <t>Kasa Depozito - küçük</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>20950.00TL</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -1958,9 +1958,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H35" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="H35" s="21" t="inlineStr">
+        <is>
+          <t>- / -</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
@@ -1972,12 +1972,12 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - genel</t>
+          <t>Yıllık Kasa Ücreti - genel</t>
         </is>
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1469.52TL</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>9420TL</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E36" s="15" t="inlineStr">
@@ -2019,7 +2019,7 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>Kasa Depozito - 0-8300</t>
+          <t>Kasa Depozito - genel</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>9420TL</t>
         </is>
       </c>
       <c r="E37" s="15" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>- / -</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
@@ -2063,69 +2063,69 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>Yıllık Kasa Ücreti - 0-8300</t>
-        </is>
-      </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E38" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F38" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G38" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H38" s="18" t="inlineStr">
-        <is>
-          <t>- / -</t>
-        </is>
-      </c>
-      <c r="I38" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Kıymetli Maden</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Altın Transfer - 0-8300</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>50.00TL</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>3.25%</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H40" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I40" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 0-8300</t>
+          <t>Altın Transfer - 8300-399000</t>
         </is>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>50.00TL</t>
+          <t>100.00TL</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="D41" s="21" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>170TL</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr">
@@ -2167,12 +2167,12 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 8300-399000</t>
-        </is>
-      </c>
-      <c r="B42" s="21" t="inlineStr">
-        <is>
-          <t>100.00TL</t>
+          <t>Altın Transfer</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -2180,9 +2180,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D42" s="21" t="inlineStr">
-        <is>
-          <t>170TL</t>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>10%</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr">
@@ -2214,7 +2214,7 @@
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer</t>
+          <t>Altın Transfer - 1-10gr</t>
         </is>
       </c>
       <c r="B43" s="12" t="inlineStr">
@@ -2229,17 +2229,17 @@
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>57,5TL</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>60 TL</t>
         </is>
       </c>
       <c r="G43" s="17" t="inlineStr">
@@ -2261,7 +2261,7 @@
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 1-10gr</t>
+          <t>Altın Transfer - 11-100gr</t>
         </is>
       </c>
       <c r="B44" s="12" t="inlineStr">
@@ -2281,12 +2281,12 @@
       </c>
       <c r="E44" s="15" t="inlineStr">
         <is>
-          <t>57,5TL</t>
+          <t>115TL</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>60 TL</t>
+          <t>120 TL</t>
         </is>
       </c>
       <c r="G44" s="17" t="inlineStr">
@@ -2308,7 +2308,7 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>Altın Transfer - 11-100gr</t>
+          <t>Altın Transfer - 399000+</t>
         </is>
       </c>
       <c r="B45" s="12" t="inlineStr">
@@ -2321,19 +2321,19 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="D45" s="21" t="inlineStr">
+        <is>
+          <t>415TL</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>115TL</t>
-        </is>
-      </c>
-      <c r="F45" s="16" t="inlineStr">
-        <is>
-          <t>120 TL</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F45" s="21" t="inlineStr">
+        <is>
+          <t>0.00018</t>
         </is>
       </c>
       <c r="G45" s="17" t="inlineStr">
@@ -2352,410 +2352,410 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
-        <is>
-          <t>Altın Transfer - 399000+</t>
-        </is>
-      </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D46" s="21" t="inlineStr">
-        <is>
-          <t>415TL</t>
-        </is>
-      </c>
-      <c r="E46" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F46" s="21" t="inlineStr">
-        <is>
-          <t>0.00018</t>
-        </is>
-      </c>
-      <c r="G46" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H46" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I46" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="10" t="inlineStr">
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>Üçüncü Kişi ve Kuruluşlardan Temin Edilecek Rapor Ücretleri - Kredi Risk Raporu</t>
         </is>
       </c>
-      <c r="B49" s="21" t="inlineStr">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="D49" s="21" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>95TL</t>
         </is>
       </c>
-      <c r="E49" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F49" s="21" t="inlineStr">
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F48" s="21" t="inlineStr">
         <is>
           <t>65 TL</t>
         </is>
       </c>
-      <c r="G49" s="17" t="inlineStr">
+      <c r="G48" s="17" t="inlineStr">
         <is>
           <t>95,24 TL</t>
         </is>
       </c>
-      <c r="H49" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
+      <c r="H48" s="21" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
+      <c r="I48" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri - Kart</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Fatura Ödemeleri</t>
         </is>
       </c>
-      <c r="B52" s="21" t="inlineStr">
+      <c r="B51" s="21" t="inlineStr">
         <is>
           <t>5.00TL / 3.50%</t>
         </is>
       </c>
-      <c r="C52" s="21" t="inlineStr">
+      <c r="C51" s="21" t="inlineStr">
         <is>
           <t>0.00TL</t>
         </is>
       </c>
-      <c r="D52" s="21" t="inlineStr">
+      <c r="D51" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E52" s="21" t="inlineStr">
+      <c r="E51" s="21" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="F52" s="21" t="inlineStr">
+      <c r="F51" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="G52" s="21" t="inlineStr">
+      <c r="G51" s="21" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="H52" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I52" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="H51" s="21" t="inlineStr">
+        <is>
+          <t>0,63 TL / -</t>
+        </is>
+      </c>
+      <c r="I51" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L51" s="20" t="inlineStr">
+        <is>
+          <t>Fatura ödemeleri üst tier için %3,5'a çıkabiliyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
       <c r="L52" s="20" t="inlineStr">
         <is>
-          <t>Fatura ödemeleri üst tier için %3,5'a çıkabiliyor</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
+          <t>Borcu Yoktur Yazısı almak için ücret alınabiliyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>SGK Prim Ödemeleri</t>
+        </is>
+      </c>
       <c r="L53" s="20" t="inlineStr">
         <is>
-          <t>Borcu Yoktur Yazısı almak için ücret alınabiliyor</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="10" t="inlineStr">
+          <t>Mevduat Araştırma Ücretleri zamlanabilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>SGK Prim Ödemeleri</t>
         </is>
       </c>
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>3.50TL / 3.50%</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>0TL</t>
+        </is>
+      </c>
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F54" s="21" t="inlineStr">
+        <is>
+          <t>2 TL / 3,5%</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I54" s="19" t="inlineStr">
+        <is>
+          <t>3 TL / -</t>
+        </is>
+      </c>
       <c r="L54" s="20" t="inlineStr">
         <is>
-          <t>Mevduat Araştırma Ücretleri zamlanabilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>SGK Prim Ödemeleri</t>
-        </is>
-      </c>
-      <c r="B55" s="21" t="inlineStr">
-        <is>
-          <t>3.50TL / 3.50%</t>
-        </is>
-      </c>
-      <c r="C55" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="inlineStr">
-        <is>
-          <t>0TL</t>
-        </is>
-      </c>
-      <c r="E55" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F55" s="21" t="inlineStr">
-        <is>
-          <t>2 TL / 3,5%</t>
-        </is>
-      </c>
-      <c r="G55" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H55" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L55" s="20" t="inlineStr">
-        <is>
           <t>Güvenli Araç Alım Satım YKB 97,53 TRY</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="10" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>275.00TL</t>
         </is>
       </c>
-      <c r="C58" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D58" s="14" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="E58" s="15" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>275TL</t>
         </is>
       </c>
-      <c r="F58" s="16" t="inlineStr">
+      <c r="F57" s="16" t="inlineStr">
         <is>
           <t>275 TL</t>
         </is>
       </c>
-      <c r="G58" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H58" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I58" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="10" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="11" t="inlineStr">
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>Şans Oyunu Ödemeleri Aracılık</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D61" s="21" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
         <is>
           <t>26TL</t>
         </is>
       </c>
-      <c r="E61" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="inlineStr">
+      <c r="E60" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F60" s="21" t="inlineStr">
         <is>
           <t>38,10 TL</t>
         </is>
       </c>
-      <c r="G61" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H61" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="G60" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I60" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="10" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="11" t="inlineStr">
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D64" s="14" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E64" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F64" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G64" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H64" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I64" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="10" t="inlineStr">
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="10" t="inlineStr">
         <is>
           <t>Telefon Ödemeleri Aracılık</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>Telefon - 0-8300 TRY</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>3,99 TL</t>
+        </is>
+      </c>
+      <c r="G66" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I66" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>Telefon - 0-8300 TRY</t>
+          <t>Telefon - 8300-399000 TRY</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>3,99 TL</t>
+          <t>7,98 TL</t>
         </is>
       </c>
       <c r="G67" s="17" t="inlineStr">
@@ -2802,7 +2802,7 @@
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>Telefon - 8300-399000 TRY</t>
+          <t>Telefon - 399000+ TRY</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="F68" s="16" t="inlineStr">
         <is>
-          <t>7,98 TL</t>
+          <t>99,71 TL</t>
         </is>
       </c>
       <c r="G68" s="17" t="inlineStr">
@@ -2849,7 +2849,7 @@
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>Telefon - 399000+ TRY</t>
+          <t>Telefon Ödemeleri</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>99,71 TL</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="G69" s="17" t="inlineStr">
@@ -2893,145 +2893,145 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="11" t="inlineStr">
-        <is>
-          <t>Telefon Ödemeleri</t>
-        </is>
-      </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D70" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E70" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F70" s="16" t="inlineStr">
-        <is>
-          <t>1 %</t>
-        </is>
-      </c>
-      <c r="G70" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H70" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I70" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="10" t="inlineStr">
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="10" t="inlineStr">
         <is>
           <t>Vergi Tahsilat Aracılık</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="11" t="inlineStr">
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="11" t="inlineStr">
         <is>
           <t>Vergi Tahsilat</t>
         </is>
       </c>
-      <c r="B73" s="12" t="inlineStr"/>
-      <c r="C73" s="13" t="inlineStr"/>
-      <c r="D73" s="14" t="inlineStr"/>
-      <c r="E73" s="15" t="inlineStr"/>
-      <c r="F73" s="16" t="inlineStr"/>
-      <c r="G73" s="17" t="inlineStr"/>
-      <c r="H73" s="18" t="inlineStr"/>
-      <c r="I73" s="19" t="inlineStr"/>
-    </row>
-    <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="10" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr"/>
+      <c r="C72" s="13" t="inlineStr"/>
+      <c r="D72" s="14" t="inlineStr"/>
+      <c r="E72" s="15" t="inlineStr"/>
+      <c r="F72" s="16" t="inlineStr"/>
+      <c r="G72" s="17" t="inlineStr"/>
+      <c r="H72" s="18" t="inlineStr"/>
+      <c r="I72" s="19" t="inlineStr"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="10" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="11" t="inlineStr">
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="11" t="inlineStr">
         <is>
           <t>Arşiv Araştırma Ücreti</t>
         </is>
       </c>
-      <c r="B76" s="12" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>287.62TL</t>
         </is>
       </c>
-      <c r="C76" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D76" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E76" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F76" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G76" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H76" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I76" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="10" t="inlineStr">
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G75" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H75" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I75" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="10" t="inlineStr">
         <is>
           <t>Mevduat Araştırma</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>Referans Mektubu -</t>
+        </is>
+      </c>
+      <c r="B78" s="21" t="inlineStr">
+        <is>
+          <t>4000.00TL</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D78" s="21" t="inlineStr">
+        <is>
+          <t>770TL</t>
+        </is>
+      </c>
+      <c r="E78" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G78" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H78" s="21" t="inlineStr">
+        <is>
+          <t>50 TL / -</t>
+        </is>
+      </c>
+      <c r="I78" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="11" t="inlineStr">
         <is>
-          <t>Referans Mektubu -</t>
-        </is>
-      </c>
-      <c r="B79" s="21" t="inlineStr">
-        <is>
-          <t>4000.00TL</t>
+          <t>Hesap Özeti Verilmesi -</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C79" s="13" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="D79" s="21" t="inlineStr">
         <is>
-          <t>770TL</t>
+          <t>190TL</t>
         </is>
       </c>
       <c r="E79" s="15" t="inlineStr">
@@ -3049,9 +3049,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F79" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="F79" s="21" t="inlineStr">
+        <is>
+          <t>12 TL</t>
         </is>
       </c>
       <c r="G79" s="17" t="inlineStr">
@@ -3073,7 +3073,7 @@
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>Hesap Özeti Verilmesi -</t>
+          <t>Borcu Yoktur Yazısı</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -3086,9 +3086,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D80" s="21" t="inlineStr">
-        <is>
-          <t>190TL</t>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>390TL</t>
         </is>
       </c>
       <c r="E80" s="15" t="inlineStr">
@@ -3096,9 +3096,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F80" s="21" t="inlineStr">
-        <is>
-          <t>12 TL</t>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G80" s="17" t="inlineStr">
@@ -3117,177 +3117,177 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="11" t="inlineStr">
-        <is>
-          <t>Borcu Yoktur Yazısı</t>
-        </is>
-      </c>
-      <c r="B81" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D81" s="14" t="inlineStr">
-        <is>
-          <t>390TL</t>
-        </is>
-      </c>
-      <c r="E81" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F81" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G81" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H81" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I81" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="10" t="inlineStr">
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="20" customHeight="1">
-      <c r="A84" s="11" t="inlineStr">
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="11" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
-      <c r="B84" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C84" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D84" s="14" t="inlineStr">
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C83" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D83" s="21" t="inlineStr">
         <is>
           <t>0.41TL</t>
         </is>
       </c>
-      <c r="E84" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F84" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G84" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H84" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I84" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="10" t="inlineStr">
+      <c r="E83" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F83" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G83" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H83" s="21" t="inlineStr">
+        <is>
+          <t>- / -</t>
+        </is>
+      </c>
+      <c r="I83" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="11" t="inlineStr">
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="11" t="inlineStr">
         <is>
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
-      <c r="B87" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C87" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D87" s="21" t="inlineStr">
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C86" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D86" s="21" t="inlineStr">
         <is>
           <t>0.45EUR</t>
         </is>
       </c>
-      <c r="E87" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F87" s="21" t="inlineStr">
+      <c r="E86" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F86" s="21" t="inlineStr">
         <is>
           <t>0.27 TL</t>
         </is>
       </c>
-      <c r="G87" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H87" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I87" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="10" t="inlineStr">
+      <c r="G86" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I86" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="10" t="inlineStr">
         <is>
           <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="11" t="inlineStr">
+        <is>
+          <t>Çek Düzenleme -</t>
+        </is>
+      </c>
+      <c r="B89" s="21" t="inlineStr">
+        <is>
+          <t>9.52TL / 0.10%</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D89" s="21" t="inlineStr">
+        <is>
+          <t>290TL / 1.10%</t>
+        </is>
+      </c>
+      <c r="E89" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F89" s="21" t="inlineStr">
+        <is>
+          <t>761,90 TL</t>
+        </is>
+      </c>
+      <c r="G89" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H89" s="21" t="inlineStr">
+        <is>
+          <t>104,76 TL / -</t>
+        </is>
+      </c>
+      <c r="I89" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>Çek Düzenleme -</t>
-        </is>
-      </c>
-      <c r="B90" s="21" t="inlineStr">
-        <is>
-          <t>9.52TL / 0.10%</t>
+          <t>Çek Defteri (Yaprak Başı) -</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
@@ -3295,9 +3295,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D90" s="21" t="inlineStr">
-        <is>
-          <t>290TL / 1.10%</t>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E90" s="15" t="inlineStr">
@@ -3305,9 +3305,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F90" s="21" t="inlineStr">
-        <is>
-          <t>761,90 TL</t>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>2.380,95 TL</t>
         </is>
       </c>
       <c r="G90" s="17" t="inlineStr">
@@ -3326,148 +3326,148 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="A91" s="11" t="inlineStr">
-        <is>
-          <t>Çek Defteri (Yaprak Başı) -</t>
-        </is>
-      </c>
-      <c r="B91" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C91" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D91" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E91" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F91" s="16" t="inlineStr">
-        <is>
-          <t>2.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G91" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H91" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I91" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="10" t="inlineStr">
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="10" t="inlineStr">
         <is>
           <t>Çek İade Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="11" t="inlineStr">
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="11" t="inlineStr">
         <is>
           <t>Çek İade Ücreti</t>
         </is>
       </c>
-      <c r="B94" s="21" t="inlineStr">
+      <c r="B93" s="21" t="inlineStr">
         <is>
           <t>171.43TL</t>
         </is>
       </c>
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D94" s="21" t="inlineStr">
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D93" s="21" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
-      <c r="E94" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F94" s="21" t="inlineStr">
+      <c r="E93" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F93" s="21" t="inlineStr">
         <is>
           <t>380,95 TL</t>
         </is>
       </c>
-      <c r="G94" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H94" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I94" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="18" customHeight="1">
-      <c r="A96" s="10" t="inlineStr">
+      <c r="G93" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H93" s="21" t="inlineStr">
+        <is>
+          <t>123,81 TL / -</t>
+        </is>
+      </c>
+      <c r="I93" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="10" t="inlineStr">
         <is>
           <t>Çek Tahsilat Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>Çek Tahsilat</t>
+        </is>
+      </c>
+      <c r="B96" s="21" t="inlineStr">
+        <is>
+          <t>45USD</t>
+        </is>
+      </c>
+      <c r="C96" s="21" t="inlineStr">
+        <is>
+          <t>590.48TL / 0.77%</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E96" s="21" t="inlineStr">
+        <is>
+          <t>1.70%</t>
+        </is>
+      </c>
+      <c r="F96" s="21" t="inlineStr">
+        <is>
+          <t>714,29 TL</t>
+        </is>
+      </c>
+      <c r="G96" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H96" s="21" t="inlineStr">
+        <is>
+          <t>260 TL / -</t>
+        </is>
+      </c>
+      <c r="I96" s="21" t="inlineStr">
+        <is>
+          <t>- / -</t>
         </is>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="11" t="inlineStr">
         <is>
-          <t>Çek Tahsilat</t>
+          <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
         </is>
       </c>
       <c r="B97" s="21" t="inlineStr">
         <is>
-          <t>45USD</t>
-        </is>
-      </c>
-      <c r="C97" s="21" t="inlineStr">
-        <is>
-          <t>590.48TL / 0.77%</t>
-        </is>
-      </c>
-      <c r="D97" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>257.15TL</t>
+        </is>
+      </c>
+      <c r="C97" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D97" s="21" t="inlineStr">
+        <is>
+          <t>2940TL / 1%</t>
         </is>
       </c>
       <c r="E97" s="21" t="inlineStr">
         <is>
-          <t>1.70%</t>
+          <t>390TL / 0.2%</t>
         </is>
       </c>
       <c r="F97" s="21" t="inlineStr">
         <is>
-          <t>714,29 TL</t>
-        </is>
-      </c>
-      <c r="G97" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>1.666,67 TL</t>
+        </is>
+      </c>
+      <c r="G97" s="21" t="inlineStr">
+        <is>
+          <t>585,71 TL</t>
         </is>
       </c>
       <c r="H97" s="18" t="inlineStr">
@@ -3484,12 +3484,12 @@
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>Döviz Çekleri Tahsilatı (Diğer Banka) -</t>
+          <t>Diğer Banka Çeki -</t>
         </is>
       </c>
       <c r="B98" s="21" t="inlineStr">
         <is>
-          <t>257.15TL</t>
+          <t>390.48TL</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -3499,22 +3499,22 @@
       </c>
       <c r="D98" s="21" t="inlineStr">
         <is>
-          <t>2940TL / 1%</t>
-        </is>
-      </c>
-      <c r="E98" s="21" t="inlineStr">
-        <is>
-          <t>390TL / 0.2%</t>
-        </is>
-      </c>
-      <c r="F98" s="21" t="inlineStr">
-        <is>
-          <t>1.666,67 TL</t>
-        </is>
-      </c>
-      <c r="G98" s="21" t="inlineStr">
-        <is>
-          <t>585,71 TL</t>
+          <t>350TL</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F98" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G98" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H98" s="18" t="inlineStr">
@@ -3524,19 +3524,19 @@
       </c>
       <c r="I98" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>576,19 TL / 0,6</t>
         </is>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="11" t="inlineStr">
         <is>
-          <t>Diğer Banka Çeki -</t>
-        </is>
-      </c>
-      <c r="B99" s="21" t="inlineStr">
-        <is>
-          <t>390.48TL</t>
+          <t>Aynı Banka Çeki -</t>
+        </is>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C99" s="13" t="inlineStr">
@@ -3544,9 +3544,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D99" s="21" t="inlineStr">
-        <is>
-          <t>350TL</t>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E99" s="15" t="inlineStr">
@@ -3571,26 +3571,26 @@
       </c>
       <c r="I99" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>427,62 TL / -</t>
         </is>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>Senet İade Ücreti</t>
+          <t>Çek Belgelendirme ve Düzeltme Ücreti</t>
         </is>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>Senet İade Ücreti</t>
-        </is>
-      </c>
-      <c r="B102" s="21" t="inlineStr">
-        <is>
-          <t>495.24TL</t>
+          <t>Karşılıksız Çek Belgelendirme -</t>
+        </is>
+      </c>
+      <c r="B102" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -3598,9 +3598,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D102" s="21" t="inlineStr">
-        <is>
-          <t>780TL</t>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E102" s="15" t="inlineStr">
@@ -3608,9 +3608,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F102" s="21" t="inlineStr">
-        <is>
-          <t>571,43 TL</t>
+      <c r="F102" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G102" s="17" t="inlineStr">
@@ -3618,9 +3618,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H102" s="21" t="inlineStr">
-        <is>
-          <t>123,81 TL / -</t>
+      <c r="H102" s="18" t="inlineStr">
+        <is>
+          <t>371,43 TL / -</t>
         </is>
       </c>
       <c r="I102" s="19" t="inlineStr">
@@ -3632,263 +3632,317 @@
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Senet Protesto İşlemleri Ücreti</t>
+          <t>Senet İade Ücreti</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="11" t="inlineStr">
         <is>
+          <t>Senet İade Ücreti</t>
+        </is>
+      </c>
+      <c r="B105" s="21" t="inlineStr">
+        <is>
+          <t>495.24TL</t>
+        </is>
+      </c>
+      <c r="C105" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D105" s="21" t="inlineStr">
+        <is>
+          <t>780TL</t>
+        </is>
+      </c>
+      <c r="E105" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F105" s="21" t="inlineStr">
+        <is>
+          <t>571,43 TL</t>
+        </is>
+      </c>
+      <c r="G105" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H105" s="21" t="inlineStr">
+        <is>
+          <t>600 TL / -</t>
+        </is>
+      </c>
+      <c r="I105" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>Senet Protesto İşlemleri Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="11" t="inlineStr">
+        <is>
           <t>Senet Protesto Kaldırma -</t>
         </is>
       </c>
-      <c r="B105" s="21" t="inlineStr">
+      <c r="B108" s="21" t="inlineStr">
         <is>
           <t>533.34TL</t>
         </is>
       </c>
-      <c r="C105" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D105" s="21" t="inlineStr">
+      <c r="C108" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D108" s="21" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
-      <c r="E105" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F105" s="21" t="inlineStr">
+      <c r="E108" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F108" s="21" t="inlineStr">
         <is>
           <t>619,05 TL</t>
         </is>
       </c>
-      <c r="G105" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H105" s="21" t="inlineStr">
+      <c r="G108" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H108" s="21" t="inlineStr">
         <is>
           <t>551,43 TL / -</t>
         </is>
       </c>
-      <c r="I105" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="20" customHeight="1">
-      <c r="A106" s="11" t="inlineStr">
-        <is>
-          <t>Senet Protesto -</t>
-        </is>
-      </c>
-      <c r="B106" s="21" t="inlineStr">
-        <is>
-          <t>600.00TL</t>
-        </is>
-      </c>
-      <c r="C106" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D106" s="21" t="inlineStr">
-        <is>
-          <t>780TL</t>
-        </is>
-      </c>
-      <c r="E106" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F106" s="21" t="inlineStr">
-        <is>
-          <t>666,67 TL</t>
-        </is>
-      </c>
-      <c r="G106" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H106" s="21" t="inlineStr">
-        <is>
-          <t>600 TL / -</t>
-        </is>
-      </c>
-      <c r="I106" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="10" t="inlineStr">
-        <is>
-          <t>Senet Tahsile Alma Ücreti</t>
+      <c r="I108" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="11" t="inlineStr">
         <is>
+          <t>Senet Protesto -</t>
+        </is>
+      </c>
+      <c r="B109" s="21" t="inlineStr">
+        <is>
+          <t>600.00TL</t>
+        </is>
+      </c>
+      <c r="C109" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D109" s="21" t="inlineStr">
+        <is>
+          <t>780TL</t>
+        </is>
+      </c>
+      <c r="E109" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F109" s="21" t="inlineStr">
+        <is>
+          <t>666,67 TL</t>
+        </is>
+      </c>
+      <c r="G109" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H109" s="21" t="inlineStr">
+        <is>
+          <t>600 TL / -</t>
+        </is>
+      </c>
+      <c r="I109" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>Senet Tahsile Alma Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="11" t="inlineStr">
+        <is>
           <t>Muhabir Banka Senet Tahsili -</t>
         </is>
       </c>
-      <c r="B109" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C109" s="21" t="inlineStr">
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C112" s="13" t="inlineStr">
         <is>
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="D109" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E109" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F109" s="21" t="inlineStr">
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E112" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F112" s="21" t="inlineStr">
         <is>
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="G109" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H109" s="21" t="inlineStr">
-        <is>
-          <t>104,76 TL / -</t>
-        </is>
-      </c>
-      <c r="I109" s="21" t="inlineStr">
-        <is>
-          <t>576,19 TL / 0,6</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="20" customHeight="1">
-      <c r="A110" s="11" t="inlineStr">
-        <is>
-          <t>Aynı Banka Senet Tahsili -</t>
-        </is>
-      </c>
-      <c r="B110" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C110" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D110" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E110" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F110" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G110" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H110" s="18" t="inlineStr">
+      <c r="G112" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H112" s="21" t="inlineStr">
         <is>
           <t>600 TL / -</t>
         </is>
       </c>
-      <c r="I110" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="10" t="inlineStr">
-        <is>
-          <t>HGS</t>
+      <c r="I112" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="11" t="inlineStr">
         <is>
+          <t>Aynı Banka Senet Tahsili -</t>
+        </is>
+      </c>
+      <c r="B113" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C113" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E113" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F113" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G113" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H113" s="18" t="inlineStr">
+        <is>
+          <t>600 TL / -</t>
+        </is>
+      </c>
+      <c r="I113" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>HGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
           <t>HGS Kart Ücreti</t>
         </is>
       </c>
-      <c r="B113" s="21" t="inlineStr">
+      <c r="B116" s="21" t="inlineStr">
         <is>
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="C113" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D113" s="21" t="inlineStr">
+      <c r="C116" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D116" s="21" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="E113" s="15" t="inlineStr">
+      <c r="E116" s="15" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="F113" s="21" t="inlineStr">
+      <c r="F116" s="21" t="inlineStr">
         <is>
           <t>500 TL</t>
         </is>
       </c>
-      <c r="G113" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H113" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I113" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="22" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 14.08.2026 15:13</t>
+      <c r="G116" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H116" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I116" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="22" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 14.08.2026 15:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 15:52)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1333,14 +1333,14 @@
           <t>19,94 TL</t>
         </is>
       </c>
-      <c r="H18" s="21" t="inlineStr">
-        <is>
-          <t>13,33 TL / -</t>
-        </is>
-      </c>
-      <c r="I18" s="21" t="inlineStr">
-        <is>
-          <t>19,94 TL / -</t>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1380,14 +1380,14 @@
           <t>39,88 TL</t>
         </is>
       </c>
-      <c r="H19" s="21" t="inlineStr">
-        <is>
-          <t>27,62 TL / -</t>
-        </is>
-      </c>
-      <c r="I19" s="21" t="inlineStr">
-        <is>
-          <t>39,88 TL / -</t>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1427,14 +1427,14 @@
           <t>398,84 TL</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr">
-        <is>
-          <t>199,05 TL / -</t>
-        </is>
-      </c>
-      <c r="I20" s="21" t="inlineStr">
-        <is>
-          <t>398,84 TL / -</t>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
           <t>FAST - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
@@ -1528,9 +1528,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr">
-        <is>
-          <t>7,97 TL / -</t>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I24" s="19" t="inlineStr">
@@ -1592,7 +1592,7 @@
           <t>FAST - 8300-399000 TRY</t>
         </is>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
@@ -1622,9 +1622,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H26" s="21" t="inlineStr">
-        <is>
-          <t>15,96 TL / -</t>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I26" s="19" t="inlineStr">
@@ -1639,46 +1639,14 @@
           <t>FAST</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G27" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H27" s="18" t="inlineStr">
-        <is>
-          <t>200 TL / 0,4</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B27" s="12" t="inlineStr"/>
+      <c r="C27" s="13" t="inlineStr"/>
+      <c r="D27" s="14" t="inlineStr"/>
+      <c r="E27" s="15" t="inlineStr"/>
+      <c r="F27" s="16" t="inlineStr"/>
+      <c r="G27" s="17" t="inlineStr"/>
+      <c r="H27" s="18" t="inlineStr"/>
+      <c r="I27" s="19" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -1723,9 +1691,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H30" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H30" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I30" s="19" t="inlineStr">
@@ -1770,9 +1738,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H31" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H31" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
@@ -1817,9 +1785,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H32" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H32" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I32" s="19" t="inlineStr">
@@ -1834,7 +1802,7 @@
           <t>Kasa Depozito - büyük</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>28570.00TL</t>
         </is>
@@ -1864,9 +1832,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H33" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H33" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
@@ -1881,7 +1849,7 @@
           <t>Kasa Depozito - orta</t>
         </is>
       </c>
-      <c r="B34" s="21" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>23805.00TL</t>
         </is>
@@ -1911,9 +1879,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H34" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H34" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I34" s="19" t="inlineStr">
@@ -1928,7 +1896,7 @@
           <t>Kasa Depozito - küçük</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>20950.00TL</t>
         </is>
@@ -1958,9 +1926,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H35" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H35" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
@@ -2395,9 +2363,9 @@
           <t>95,24 TL</t>
         </is>
       </c>
-      <c r="H48" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H48" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I48" s="19" t="inlineStr">
@@ -2449,9 +2417,9 @@
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="H51" s="21" t="inlineStr">
-        <is>
-          <t>0,63 TL / -</t>
+      <c r="H51" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
@@ -2527,7 +2495,7 @@
       </c>
       <c r="I54" s="19" t="inlineStr">
         <is>
-          <t>3 TL / -</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L54" s="20" t="inlineStr">
@@ -3012,9 +2980,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H78" s="21" t="inlineStr">
-        <is>
-          <t>50 TL / -</t>
+      <c r="H78" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I78" s="19" t="inlineStr">
@@ -3140,7 +3108,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D83" s="21" t="inlineStr">
+      <c r="D83" s="14" t="inlineStr">
         <is>
           <t>0.41TL</t>
         </is>
@@ -3160,9 +3128,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H83" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H83" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I83" s="19" t="inlineStr">
@@ -3268,9 +3236,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H89" s="21" t="inlineStr">
-        <is>
-          <t>104,76 TL / -</t>
+      <c r="H89" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I89" s="19" t="inlineStr">
@@ -3369,9 +3337,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H93" s="21" t="inlineStr">
-        <is>
-          <t>123,81 TL / -</t>
+      <c r="H93" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I93" s="19" t="inlineStr">
@@ -3423,14 +3391,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H96" s="21" t="inlineStr">
-        <is>
-          <t>260 TL / -</t>
-        </is>
-      </c>
-      <c r="I96" s="21" t="inlineStr">
-        <is>
-          <t>- / -</t>
+      <c r="H96" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I96" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -3524,181 +3492,149 @@
       </c>
       <c r="I98" s="19" t="inlineStr">
         <is>
-          <t>576,19 TL / 0,6</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="11" t="inlineStr">
-        <is>
-          <t>Aynı Banka Çeki -</t>
-        </is>
-      </c>
-      <c r="B99" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C99" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D99" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E99" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F99" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G99" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H99" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I99" s="19" t="inlineStr">
-        <is>
-          <t>427,62 TL / -</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="10" t="inlineStr">
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="10" t="inlineStr">
         <is>
           <t>Çek Belgelendirme ve Düzeltme Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="20" customHeight="1">
-      <c r="A102" s="11" t="inlineStr">
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="11" t="inlineStr">
         <is>
           <t>Karşılıksız Çek Belgelendirme -</t>
         </is>
       </c>
-      <c r="B102" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C102" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D102" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E102" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F102" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G102" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H102" s="18" t="inlineStr">
-        <is>
-          <t>371,43 TL / -</t>
-        </is>
-      </c>
-      <c r="I102" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="10" t="inlineStr">
+      <c r="B101" s="12" t="inlineStr"/>
+      <c r="C101" s="13" t="inlineStr"/>
+      <c r="D101" s="14" t="inlineStr"/>
+      <c r="E101" s="15" t="inlineStr"/>
+      <c r="F101" s="16" t="inlineStr"/>
+      <c r="G101" s="17" t="inlineStr"/>
+      <c r="H101" s="18" t="inlineStr"/>
+      <c r="I101" s="19" t="inlineStr"/>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="10" t="inlineStr">
         <is>
           <t>Senet İade Ücreti</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="20" customHeight="1">
-      <c r="A105" s="11" t="inlineStr">
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="11" t="inlineStr">
         <is>
           <t>Senet İade Ücreti</t>
         </is>
       </c>
-      <c r="B105" s="21" t="inlineStr">
+      <c r="B104" s="21" t="inlineStr">
         <is>
           <t>495.24TL</t>
         </is>
       </c>
-      <c r="C105" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D105" s="21" t="inlineStr">
+      <c r="C104" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D104" s="21" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
-      <c r="E105" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F105" s="21" t="inlineStr">
+      <c r="E104" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F104" s="21" t="inlineStr">
         <is>
           <t>571,43 TL</t>
         </is>
       </c>
-      <c r="G105" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H105" s="21" t="inlineStr">
-        <is>
-          <t>600 TL / -</t>
-        </is>
-      </c>
-      <c r="I105" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="10" t="inlineStr">
+      <c r="G104" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I104" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="10" t="inlineStr">
         <is>
           <t>Senet Protesto İşlemleri Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="11" t="inlineStr">
+        <is>
+          <t>Senet Protesto Kaldırma -</t>
+        </is>
+      </c>
+      <c r="B107" s="21" t="inlineStr">
+        <is>
+          <t>533.34TL</t>
+        </is>
+      </c>
+      <c r="C107" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D107" s="21" t="inlineStr">
+        <is>
+          <t>780TL</t>
+        </is>
+      </c>
+      <c r="E107" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F107" s="21" t="inlineStr">
+        <is>
+          <t>619,05 TL</t>
+        </is>
+      </c>
+      <c r="G107" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H107" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I107" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>Senet Protesto Kaldırma -</t>
+          <t>Senet Protesto -</t>
         </is>
       </c>
       <c r="B108" s="21" t="inlineStr">
         <is>
-          <t>533.34TL</t>
+          <t>600.00TL</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
@@ -3718,7 +3654,7 @@
       </c>
       <c r="F108" s="21" t="inlineStr">
         <is>
-          <t>619,05 TL</t>
+          <t>666,67 TL</t>
         </is>
       </c>
       <c r="G108" s="17" t="inlineStr">
@@ -3726,9 +3662,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H108" s="21" t="inlineStr">
-        <is>
-          <t>551,43 TL / -</t>
+      <c r="H108" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I108" s="19" t="inlineStr">
@@ -3737,212 +3673,133 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="20" customHeight="1">
-      <c r="A109" s="11" t="inlineStr">
-        <is>
-          <t>Senet Protesto -</t>
-        </is>
-      </c>
-      <c r="B109" s="21" t="inlineStr">
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t>Senet Tahsile Alma Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="11" t="inlineStr">
+        <is>
+          <t>Muhabir Banka Senet Tahsili -</t>
+        </is>
+      </c>
+      <c r="B111" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C111" s="13" t="inlineStr">
         <is>
           <t>600.00TL</t>
         </is>
       </c>
-      <c r="C109" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D109" s="21" t="inlineStr">
-        <is>
-          <t>780TL</t>
-        </is>
-      </c>
-      <c r="E109" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F109" s="21" t="inlineStr">
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E111" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F111" s="16" t="inlineStr">
         <is>
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="G109" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H109" s="21" t="inlineStr">
-        <is>
-          <t>600 TL / -</t>
-        </is>
-      </c>
-      <c r="I109" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="18" customHeight="1">
-      <c r="A111" s="10" t="inlineStr">
-        <is>
-          <t>Senet Tahsile Alma Ücreti</t>
+      <c r="G111" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H111" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I111" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>Muhabir Banka Senet Tahsili -</t>
-        </is>
-      </c>
-      <c r="B112" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C112" s="13" t="inlineStr">
-        <is>
-          <t>600.00TL</t>
-        </is>
-      </c>
-      <c r="D112" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E112" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F112" s="21" t="inlineStr">
-        <is>
-          <t>666,67 TL</t>
-        </is>
-      </c>
-      <c r="G112" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H112" s="21" t="inlineStr">
-        <is>
-          <t>600 TL / -</t>
-        </is>
-      </c>
-      <c r="I112" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="11" t="inlineStr">
-        <is>
           <t>Aynı Banka Senet Tahsili -</t>
         </is>
       </c>
-      <c r="B113" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C113" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D113" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E113" s="15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F113" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G113" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H113" s="18" t="inlineStr">
-        <is>
-          <t>600 TL / -</t>
-        </is>
-      </c>
-      <c r="I113" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="10" t="inlineStr">
+      <c r="B112" s="12" t="inlineStr"/>
+      <c r="C112" s="13" t="inlineStr"/>
+      <c r="D112" s="14" t="inlineStr"/>
+      <c r="E112" s="15" t="inlineStr"/>
+      <c r="F112" s="16" t="inlineStr"/>
+      <c r="G112" s="17" t="inlineStr"/>
+      <c r="H112" s="18" t="inlineStr"/>
+      <c r="I112" s="19" t="inlineStr"/>
+    </row>
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="10" t="inlineStr">
         <is>
           <t>HGS</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="11" t="inlineStr">
+    <row r="115" ht="20" customHeight="1">
+      <c r="A115" s="11" t="inlineStr">
         <is>
           <t>HGS Kart Ücreti</t>
         </is>
       </c>
-      <c r="B116" s="21" t="inlineStr">
+      <c r="B115" s="21" t="inlineStr">
         <is>
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="C116" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D116" s="21" t="inlineStr">
+      <c r="C115" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D115" s="21" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="E116" s="15" t="inlineStr">
+      <c r="E115" s="15" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="F116" s="21" t="inlineStr">
+      <c r="F115" s="21" t="inlineStr">
         <is>
           <t>500 TL</t>
         </is>
       </c>
-      <c r="G116" s="17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H116" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I116" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="22" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 14.08.2026 15:31</t>
+      <c r="G115" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H115" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I115" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="22" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 14.08.2026 15:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 17:03)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -45,7 +45,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
       <sz val="10"/>
     </font>
     <font>
@@ -62,12 +62,12 @@
       <sz val="10"/>
     </font>
     <font>
+      <b val="1"/>
       <color rgb="00FF0000"/>
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -75,7 +75,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -124,12 +124,6 @@
         <bgColor rgb="00F4B183"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -157,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -186,7 +180,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,9 +196,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -660,12 +651,12 @@
       </c>
       <c r="D4" s="12" t="inlineStr"/>
       <c r="E4" s="13" t="inlineStr"/>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>4.25 %</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr"/>
+      <c r="G4" s="15" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
@@ -673,7 +664,7 @@
           <t>Düzenli EFT - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
@@ -689,12 +680,12 @@
           <t>7,97TL</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>7,97 TL</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr"/>
+      <c r="G5" s="15" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -702,7 +693,7 @@
           <t>Düzenli EFT - 8300-399000 TRY</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
@@ -718,12 +709,12 @@
           <t>15,96TL</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>15,96 TL</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="15" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -731,7 +722,7 @@
           <t>Düzenli EFT - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>199.41TL</t>
         </is>
@@ -747,12 +738,12 @@
           <t>199,41TL</t>
         </is>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>199,41 TL</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr"/>
+      <c r="G7" s="15" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -770,7 +761,7 @@
           <t>39.87TL</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>27,84TL</t>
         </is>
@@ -780,12 +771,12 @@
           <t>39,87TL</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>309.523,82 TL</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>39,87 TL</t>
         </is>
@@ -807,7 +798,7 @@
           <t>79.76TL</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>55,69TL</t>
         </is>
@@ -817,12 +808,12 @@
           <t>79,76TL</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>619.047,62 TL</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>79,76 TL</t>
         </is>
@@ -844,7 +835,7 @@
           <t>797.68TL</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>398,83TL</t>
         </is>
@@ -854,12 +845,12 @@
           <t>797,68TL</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>398,83 TL</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>797,68 TL</t>
         </is>
@@ -871,7 +862,7 @@
           <t>Düzenli EFT</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>1.00TL / 1.00%</t>
         </is>
@@ -879,8 +870,8 @@
       <c r="C11" s="11" t="inlineStr"/>
       <c r="D11" s="12" t="inlineStr"/>
       <c r="E11" s="13" t="inlineStr"/>
-      <c r="F11" s="16" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
+      <c r="F11" s="14" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -895,7 +886,7 @@
           <t>Düzenli Havale - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>3.99TL</t>
         </is>
@@ -911,12 +902,12 @@
           <t>3,99TL</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>3,99 TL</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>3,99 TL</t>
         </is>
@@ -928,7 +919,7 @@
           <t>Düzenli Havale - 8300-399000 TRY</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>7.98TL</t>
         </is>
@@ -944,12 +935,12 @@
           <t>7,98TL</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>7,98 TL</t>
         </is>
       </c>
-      <c r="G15" s="14" t="inlineStr">
+      <c r="G15" s="15" t="inlineStr">
         <is>
           <t>7,98 TL</t>
         </is>
@@ -961,7 +952,7 @@
           <t>Düzenli Havale - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>99.71TL</t>
         </is>
@@ -977,12 +968,12 @@
           <t>99,71TL</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>99,71 TL</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
         <is>
           <t>99,71 TL</t>
         </is>
@@ -999,27 +990,27 @@
           <t>1050.00TL</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>2485.72TL</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>3,99TL</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>19,94TL</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>152.380,96 TL</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="15" t="inlineStr">
         <is>
           <t>19,94 TL</t>
         </is>
@@ -1036,27 +1027,27 @@
           <t>1500.00TL</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>2923.81TL</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>7,98TL</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>39,88TL</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>309.523,81 TL</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="15" t="inlineStr">
         <is>
           <t>39,88 TL</t>
         </is>
@@ -1073,27 +1064,27 @@
           <t>1900.00TL / 0.70%</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>3676.20TL / 0.70%</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>99,71TL</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>398,84TL</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr">
         <is>
           <t>199,42</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="15" t="inlineStr">
         <is>
           <t>398,84 TL</t>
         </is>
@@ -1105,28 +1096,28 @@
           <t>Havale Gönderimi</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr"/>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr"/>
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>1038.10TL / 0.58%</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>150TL</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>125TL</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>1.300 TL / 0,6 %</t>
         </is>
       </c>
-      <c r="G20" s="14" t="inlineStr"/>
+      <c r="G20" s="15" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -1141,7 +1132,7 @@
           <t>FAST - 0-8300 TRY</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>7.97TL</t>
         </is>
@@ -1149,8 +1140,8 @@
       <c r="C23" s="11" t="inlineStr"/>
       <c r="D23" s="12" t="inlineStr"/>
       <c r="E23" s="13" t="inlineStr"/>
-      <c r="F23" s="16" t="inlineStr"/>
-      <c r="G23" s="14" t="inlineStr"/>
+      <c r="F23" s="14" t="inlineStr"/>
+      <c r="G23" s="15" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
@@ -1158,7 +1149,7 @@
           <t>FAST - 399000+ TRY</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>380.95TL / 0.48%</t>
         </is>
@@ -1166,8 +1157,8 @@
       <c r="C24" s="11" t="inlineStr"/>
       <c r="D24" s="12" t="inlineStr"/>
       <c r="E24" s="13" t="inlineStr"/>
-      <c r="F24" s="16" t="inlineStr"/>
-      <c r="G24" s="14" t="inlineStr"/>
+      <c r="F24" s="14" t="inlineStr"/>
+      <c r="G24" s="15" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -1175,7 +1166,7 @@
           <t>FAST - 8300-399000 TRY</t>
         </is>
       </c>
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>15.96TL</t>
         </is>
@@ -1183,8 +1174,8 @@
       <c r="C25" s="11" t="inlineStr"/>
       <c r="D25" s="12" t="inlineStr"/>
       <c r="E25" s="13" t="inlineStr"/>
-      <c r="F25" s="16" t="inlineStr"/>
-      <c r="G25" s="14" t="inlineStr"/>
+      <c r="F25" s="14" t="inlineStr"/>
+      <c r="G25" s="15" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
@@ -1205,7 +1196,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr"/>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>2355TL</t>
         </is>
@@ -1215,8 +1206,8 @@
           <t>3270TL / 0,7%</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr"/>
-      <c r="G28" s="14" t="inlineStr"/>
+      <c r="F28" s="14" t="inlineStr"/>
+      <c r="G28" s="15" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
@@ -1224,16 +1215,16 @@
           <t>Uluslararası Transfer - 0-8300</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr"/>
       <c r="C29" s="11" t="inlineStr"/>
       <c r="D29" s="12" t="inlineStr"/>
       <c r="E29" s="13" t="inlineStr"/>
-      <c r="F29" s="16" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>919.047,62 TL</t>
         </is>
       </c>
-      <c r="G29" s="14" t="inlineStr"/>
+      <c r="G29" s="15" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
@@ -1254,14 +1245,14 @@
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr"/>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>3.25%</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr"/>
-      <c r="F32" s="16" t="inlineStr"/>
-      <c r="G32" s="14" t="inlineStr"/>
+      <c r="F32" s="14" t="inlineStr"/>
+      <c r="G32" s="15" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
@@ -1275,14 +1266,14 @@
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr"/>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>170TL</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr"/>
-      <c r="F33" s="16" t="inlineStr"/>
-      <c r="G33" s="14" t="inlineStr"/>
+      <c r="F33" s="14" t="inlineStr"/>
+      <c r="G33" s="15" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
@@ -1290,7 +1281,7 @@
           <t>Altın Transfer</t>
         </is>
       </c>
-      <c r="B34" s="15" t="inlineStr"/>
+      <c r="B34" s="10" t="inlineStr"/>
       <c r="C34" s="11" t="inlineStr"/>
       <c r="D34" s="12" t="inlineStr">
         <is>
@@ -1298,8 +1289,8 @@
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr"/>
-      <c r="F34" s="16" t="inlineStr"/>
-      <c r="G34" s="14" t="inlineStr"/>
+      <c r="F34" s="14" t="inlineStr"/>
+      <c r="G34" s="15" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
@@ -1307,7 +1298,7 @@
           <t>Altın Transfer - 1-10gr</t>
         </is>
       </c>
-      <c r="B35" s="15" t="inlineStr"/>
+      <c r="B35" s="10" t="inlineStr"/>
       <c r="C35" s="11" t="inlineStr"/>
       <c r="D35" s="12" t="inlineStr"/>
       <c r="E35" s="13" t="inlineStr">
@@ -1315,12 +1306,12 @@
           <t>57,5TL</t>
         </is>
       </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>60 TL</t>
         </is>
       </c>
-      <c r="G35" s="14" t="inlineStr"/>
+      <c r="G35" s="15" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
@@ -1328,7 +1319,7 @@
           <t>Altın Transfer - 11-100gr</t>
         </is>
       </c>
-      <c r="B36" s="15" t="inlineStr"/>
+      <c r="B36" s="10" t="inlineStr"/>
       <c r="C36" s="11" t="inlineStr"/>
       <c r="D36" s="12" t="inlineStr"/>
       <c r="E36" s="13" t="inlineStr">
@@ -1336,12 +1327,12 @@
           <t>115TL</t>
         </is>
       </c>
-      <c r="F36" s="16" t="inlineStr">
+      <c r="F36" s="14" t="inlineStr">
         <is>
           <t>120 TL</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr"/>
+      <c r="G36" s="15" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
@@ -1349,20 +1340,20 @@
           <t>Altın Transfer - 399000+</t>
         </is>
       </c>
-      <c r="B37" s="15" t="inlineStr"/>
+      <c r="B37" s="10" t="inlineStr"/>
       <c r="C37" s="11" t="inlineStr"/>
-      <c r="D37" s="10" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>415TL</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr"/>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F37" s="14" t="inlineStr">
         <is>
           <t>0.00018</t>
         </is>
       </c>
-      <c r="G37" s="14" t="inlineStr"/>
+      <c r="G37" s="15" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
@@ -1383,14 +1374,14 @@
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr"/>
-      <c r="D40" s="10" t="inlineStr">
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>4140TL</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr"/>
-      <c r="F40" s="16" t="inlineStr"/>
-      <c r="G40" s="14" t="inlineStr"/>
+      <c r="F40" s="14" t="inlineStr"/>
+      <c r="G40" s="15" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
@@ -1404,14 +1395,14 @@
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr"/>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>2610TL</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr"/>
-      <c r="F41" s="16" t="inlineStr"/>
-      <c r="G41" s="14" t="inlineStr"/>
+      <c r="F41" s="14" t="inlineStr"/>
+      <c r="G41" s="15" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
@@ -1425,14 +1416,14 @@
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr"/>
-      <c r="D42" s="10" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>3390TL</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr"/>
-      <c r="F42" s="16" t="inlineStr"/>
-      <c r="G42" s="14" t="inlineStr"/>
+      <c r="F42" s="14" t="inlineStr"/>
+      <c r="G42" s="15" t="inlineStr"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
@@ -1440,7 +1431,7 @@
           <t>Kasa Depozito - büyük</t>
         </is>
       </c>
-      <c r="B43" s="15" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>28570.00TL</t>
         </is>
@@ -1448,8 +1439,8 @@
       <c r="C43" s="11" t="inlineStr"/>
       <c r="D43" s="12" t="inlineStr"/>
       <c r="E43" s="13" t="inlineStr"/>
-      <c r="F43" s="16" t="inlineStr"/>
-      <c r="G43" s="14" t="inlineStr"/>
+      <c r="F43" s="14" t="inlineStr"/>
+      <c r="G43" s="15" t="inlineStr"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
@@ -1457,7 +1448,7 @@
           <t>Kasa Depozito - orta</t>
         </is>
       </c>
-      <c r="B44" s="15" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>23805.00TL</t>
         </is>
@@ -1465,8 +1456,8 @@
       <c r="C44" s="11" t="inlineStr"/>
       <c r="D44" s="12" t="inlineStr"/>
       <c r="E44" s="13" t="inlineStr"/>
-      <c r="F44" s="16" t="inlineStr"/>
-      <c r="G44" s="14" t="inlineStr"/>
+      <c r="F44" s="14" t="inlineStr"/>
+      <c r="G44" s="15" t="inlineStr"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
@@ -1474,7 +1465,7 @@
           <t>Kasa Depozito - küçük</t>
         </is>
       </c>
-      <c r="B45" s="15" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>20950.00TL</t>
         </is>
@@ -1482,8 +1473,8 @@
       <c r="C45" s="11" t="inlineStr"/>
       <c r="D45" s="12" t="inlineStr"/>
       <c r="E45" s="13" t="inlineStr"/>
-      <c r="F45" s="16" t="inlineStr"/>
-      <c r="G45" s="14" t="inlineStr"/>
+      <c r="F45" s="14" t="inlineStr"/>
+      <c r="G45" s="15" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
@@ -1491,7 +1482,7 @@
           <t>Yıllık Kasa Ücreti - genel</t>
         </is>
       </c>
-      <c r="B46" s="15" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>1469.52TL</t>
         </is>
@@ -1499,8 +1490,8 @@
       <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="12" t="inlineStr"/>
       <c r="E46" s="13" t="inlineStr"/>
-      <c r="F46" s="16" t="inlineStr"/>
-      <c r="G46" s="14" t="inlineStr"/>
+      <c r="F46" s="14" t="inlineStr"/>
+      <c r="G46" s="15" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
@@ -1508,7 +1499,7 @@
           <t>Kasa Depozito - genel</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr"/>
+      <c r="B47" s="10" t="inlineStr"/>
       <c r="C47" s="11" t="inlineStr"/>
       <c r="D47" s="12" t="inlineStr">
         <is>
@@ -1516,8 +1507,8 @@
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr"/>
-      <c r="F47" s="16" t="inlineStr"/>
-      <c r="G47" s="14" t="inlineStr"/>
+      <c r="F47" s="14" t="inlineStr"/>
+      <c r="G47" s="15" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
@@ -1532,7 +1523,7 @@
           <t>HGS Etiket Bedeli</t>
         </is>
       </c>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>275.00TL</t>
         </is>
@@ -1548,12 +1539,12 @@
           <t>275TL</t>
         </is>
       </c>
-      <c r="F50" s="16" t="inlineStr">
+      <c r="F50" s="14" t="inlineStr">
         <is>
           <t>275 TL</t>
         </is>
       </c>
-      <c r="G50" s="14" t="inlineStr"/>
+      <c r="G50" s="15" t="inlineStr"/>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="8" t="inlineStr">
@@ -1574,18 +1565,18 @@
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr"/>
-      <c r="D53" s="10" t="inlineStr">
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>290TL / 1.10%</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr"/>
-      <c r="F53" s="10" t="inlineStr">
+      <c r="F53" s="14" t="inlineStr">
         <is>
           <t>761,90 TL</t>
         </is>
       </c>
-      <c r="G53" s="14" t="inlineStr"/>
+      <c r="G53" s="15" t="inlineStr"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
@@ -1593,16 +1584,16 @@
           <t>Çek Defteri (Yaprak Başı) -</t>
         </is>
       </c>
-      <c r="B54" s="15" t="inlineStr"/>
+      <c r="B54" s="10" t="inlineStr"/>
       <c r="C54" s="11" t="inlineStr"/>
       <c r="D54" s="12" t="inlineStr"/>
       <c r="E54" s="13" t="inlineStr"/>
-      <c r="F54" s="16" t="inlineStr">
+      <c r="F54" s="14" t="inlineStr">
         <is>
           <t>2.380,95 TL</t>
         </is>
       </c>
-      <c r="G54" s="14" t="inlineStr"/>
+      <c r="G54" s="15" t="inlineStr"/>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="8" t="inlineStr">
@@ -1623,18 +1614,18 @@
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr"/>
-      <c r="D57" s="10" t="inlineStr">
+      <c r="D57" s="12" t="inlineStr">
         <is>
           <t>390TL</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr"/>
-      <c r="F57" s="10" t="inlineStr">
+      <c r="F57" s="14" t="inlineStr">
         <is>
           <t>380,95 TL</t>
         </is>
       </c>
-      <c r="G57" s="14" t="inlineStr"/>
+      <c r="G57" s="15" t="inlineStr"/>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="8" t="inlineStr">
@@ -1654,27 +1645,27 @@
           <t>11.99%</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
         <is>
           <t>95.24TL</t>
         </is>
       </c>
-      <c r="D60" s="10" t="inlineStr">
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E60" s="10" t="inlineStr">
+      <c r="E60" s="13" t="inlineStr">
         <is>
           <t>780TL / 0.6%</t>
         </is>
       </c>
-      <c r="F60" s="10" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>41.904,77 TL</t>
         </is>
       </c>
-      <c r="G60" s="10" t="inlineStr">
+      <c r="G60" s="15" t="inlineStr">
         <is>
           <t>95,24 TL</t>
         </is>
@@ -1686,20 +1677,20 @@
           <t>Aynı Banka Çeki -</t>
         </is>
       </c>
-      <c r="B61" s="15" t="inlineStr"/>
-      <c r="C61" s="10" t="inlineStr">
+      <c r="B61" s="10" t="inlineStr"/>
+      <c r="C61" s="11" t="inlineStr">
         <is>
           <t>438.10TL</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr"/>
-      <c r="E61" s="10" t="inlineStr">
+      <c r="E61" s="13" t="inlineStr">
         <is>
           <t>390TL / 0.2%</t>
         </is>
       </c>
-      <c r="F61" s="16" t="inlineStr"/>
-      <c r="G61" s="14" t="inlineStr"/>
+      <c r="F61" s="14" t="inlineStr"/>
+      <c r="G61" s="15" t="inlineStr"/>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
@@ -1717,14 +1708,14 @@
           <t>590.48TL / 0.77%</t>
         </is>
       </c>
-      <c r="D62" s="10" t="inlineStr">
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>350TL</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr"/>
-      <c r="F62" s="16" t="inlineStr"/>
-      <c r="G62" s="14" t="inlineStr"/>
+      <c r="F62" s="14" t="inlineStr"/>
+      <c r="G62" s="15" t="inlineStr"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="8" t="inlineStr">
@@ -1745,18 +1736,18 @@
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr"/>
-      <c r="D65" s="10" t="inlineStr">
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr"/>
-      <c r="F65" s="10" t="inlineStr">
+      <c r="F65" s="14" t="inlineStr">
         <is>
           <t>55.333,33 TL</t>
         </is>
       </c>
-      <c r="G65" s="14" t="inlineStr"/>
+      <c r="G65" s="15" t="inlineStr"/>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="8" t="inlineStr">
@@ -1777,18 +1768,18 @@
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr"/>
-      <c r="D68" s="10" t="inlineStr">
+      <c r="D68" s="12" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr"/>
-      <c r="F68" s="10" t="inlineStr">
+      <c r="F68" s="14" t="inlineStr">
         <is>
           <t>619,05 TL</t>
         </is>
       </c>
-      <c r="G68" s="14" t="inlineStr"/>
+      <c r="G68" s="15" t="inlineStr"/>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
@@ -1802,18 +1793,18 @@
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr"/>
-      <c r="D69" s="10" t="inlineStr">
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>780TL</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr"/>
-      <c r="F69" s="10" t="inlineStr">
+      <c r="F69" s="14" t="inlineStr">
         <is>
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="G69" s="14" t="inlineStr"/>
+      <c r="G69" s="15" t="inlineStr"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="8" t="inlineStr">
@@ -1828,7 +1819,7 @@
           <t>Senet Tahsile Alma -</t>
         </is>
       </c>
-      <c r="B72" s="15" t="inlineStr"/>
+      <c r="B72" s="10" t="inlineStr"/>
       <c r="C72" s="11" t="inlineStr">
         <is>
           <t>600.00TL</t>
@@ -1836,12 +1827,12 @@
       </c>
       <c r="D72" s="12" t="inlineStr"/>
       <c r="E72" s="13" t="inlineStr"/>
-      <c r="F72" s="16" t="inlineStr">
+      <c r="F72" s="14" t="inlineStr">
         <is>
           <t>666,67 TL</t>
         </is>
       </c>
-      <c r="G72" s="14" t="inlineStr"/>
+      <c r="G72" s="15" t="inlineStr"/>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="8" t="inlineStr">
@@ -1861,27 +1852,27 @@
           <t>5.00TL / 3.50%</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
+      <c r="C75" s="11" t="inlineStr">
         <is>
           <t>0.00TL</t>
         </is>
       </c>
-      <c r="D75" s="10" t="inlineStr">
+      <c r="D75" s="12" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="E75" s="10" t="inlineStr">
+      <c r="E75" s="13" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
-      <c r="F75" s="10" t="inlineStr">
+      <c r="F75" s="14" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
       </c>
-      <c r="G75" s="10" t="inlineStr">
+      <c r="G75" s="15" t="inlineStr">
         <is>
           <t>0.5 TL</t>
         </is>
@@ -1906,18 +1897,18 @@
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr"/>
-      <c r="D78" s="10" t="inlineStr">
+      <c r="D78" s="12" t="inlineStr">
         <is>
           <t>0TL</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr"/>
-      <c r="F78" s="10" t="inlineStr">
+      <c r="F78" s="14" t="inlineStr">
         <is>
           <t>2 TL / 3,5%</t>
         </is>
       </c>
-      <c r="G78" s="14" t="inlineStr"/>
+      <c r="G78" s="15" t="inlineStr"/>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="8" t="inlineStr">
@@ -1932,12 +1923,12 @@
           <t>Vergi Tahsilat</t>
         </is>
       </c>
-      <c r="B81" s="15" t="inlineStr"/>
+      <c r="B81" s="10" t="inlineStr"/>
       <c r="C81" s="11" t="inlineStr"/>
       <c r="D81" s="12" t="inlineStr"/>
       <c r="E81" s="13" t="inlineStr"/>
-      <c r="F81" s="16" t="inlineStr"/>
-      <c r="G81" s="14" t="inlineStr"/>
+      <c r="F81" s="14" t="inlineStr"/>
+      <c r="G81" s="15" t="inlineStr"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="8" t="inlineStr">
@@ -1952,20 +1943,20 @@
           <t>Şans Oyunu Ödemeleri</t>
         </is>
       </c>
-      <c r="B84" s="15" t="inlineStr"/>
+      <c r="B84" s="10" t="inlineStr"/>
       <c r="C84" s="11" t="inlineStr"/>
-      <c r="D84" s="10" t="inlineStr">
+      <c r="D84" s="12" t="inlineStr">
         <is>
           <t>26TL</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr"/>
-      <c r="F84" s="10" t="inlineStr">
+      <c r="F84" s="14" t="inlineStr">
         <is>
           <t>38,10 TL</t>
         </is>
       </c>
-      <c r="G84" s="14" t="inlineStr"/>
+      <c r="G84" s="15" t="inlineStr"/>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="8" t="inlineStr">
@@ -1980,16 +1971,16 @@
           <t>Telefon Ödemeleri</t>
         </is>
       </c>
-      <c r="B87" s="15" t="inlineStr"/>
+      <c r="B87" s="10" t="inlineStr"/>
       <c r="C87" s="11" t="inlineStr"/>
       <c r="D87" s="12" t="inlineStr"/>
       <c r="E87" s="13" t="inlineStr"/>
-      <c r="F87" s="16" t="inlineStr">
+      <c r="F87" s="14" t="inlineStr">
         <is>
           <t>1 %</t>
         </is>
       </c>
-      <c r="G87" s="14" t="inlineStr"/>
+      <c r="G87" s="15" t="inlineStr"/>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="8" t="inlineStr">
@@ -2004,7 +1995,7 @@
           <t>Özel Okul Ödeme</t>
         </is>
       </c>
-      <c r="B90" s="15" t="inlineStr"/>
+      <c r="B90" s="10" t="inlineStr"/>
       <c r="C90" s="11" t="inlineStr"/>
       <c r="D90" s="12" t="inlineStr">
         <is>
@@ -2012,8 +2003,8 @@
         </is>
       </c>
       <c r="E90" s="13" t="inlineStr"/>
-      <c r="F90" s="16" t="inlineStr"/>
-      <c r="G90" s="14" t="inlineStr"/>
+      <c r="F90" s="14" t="inlineStr"/>
+      <c r="G90" s="15" t="inlineStr"/>
     </row>
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="8" t="inlineStr">
@@ -2028,7 +2019,7 @@
           <t>Bakiye Sorma - Yurtiçi - ATM</t>
         </is>
       </c>
-      <c r="B93" s="15" t="inlineStr"/>
+      <c r="B93" s="10" t="inlineStr"/>
       <c r="C93" s="11" t="inlineStr"/>
       <c r="D93" s="12" t="inlineStr">
         <is>
@@ -2036,8 +2027,8 @@
         </is>
       </c>
       <c r="E93" s="13" t="inlineStr"/>
-      <c r="F93" s="16" t="inlineStr"/>
-      <c r="G93" s="14" t="inlineStr"/>
+      <c r="F93" s="14" t="inlineStr"/>
+      <c r="G93" s="15" t="inlineStr"/>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="8" t="inlineStr">
@@ -2052,20 +2043,20 @@
           <t>Bakiye Sorma - Yurtdışı - ATM</t>
         </is>
       </c>
-      <c r="B96" s="15" t="inlineStr"/>
+      <c r="B96" s="10" t="inlineStr"/>
       <c r="C96" s="11" t="inlineStr"/>
-      <c r="D96" s="10" t="inlineStr">
+      <c r="D96" s="12" t="inlineStr">
         <is>
           <t>0.45EUR</t>
         </is>
       </c>
       <c r="E96" s="13" t="inlineStr"/>
-      <c r="F96" s="10" t="inlineStr">
+      <c r="F96" s="14" t="inlineStr">
         <is>
           <t>0.27 TL</t>
         </is>
       </c>
-      <c r="G96" s="14" t="inlineStr"/>
+      <c r="G96" s="15" t="inlineStr"/>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="8" t="inlineStr">
@@ -2080,20 +2071,20 @@
           <t>Kredi Risk Raporu</t>
         </is>
       </c>
-      <c r="B99" s="15" t="inlineStr"/>
+      <c r="B99" s="10" t="inlineStr"/>
       <c r="C99" s="11" t="inlineStr"/>
-      <c r="D99" s="10" t="inlineStr">
+      <c r="D99" s="12" t="inlineStr">
         <is>
           <t>95TL</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr"/>
-      <c r="F99" s="10" t="inlineStr">
+      <c r="F99" s="14" t="inlineStr">
         <is>
           <t>65 TL</t>
         </is>
       </c>
-      <c r="G99" s="14" t="inlineStr"/>
+      <c r="G99" s="15" t="inlineStr"/>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="8" t="inlineStr">
@@ -2114,14 +2105,14 @@
         </is>
       </c>
       <c r="C102" s="11" t="inlineStr"/>
-      <c r="D102" s="10" t="inlineStr">
+      <c r="D102" s="12" t="inlineStr">
         <is>
           <t>770TL</t>
         </is>
       </c>
       <c r="E102" s="13" t="inlineStr"/>
-      <c r="F102" s="16" t="inlineStr"/>
-      <c r="G102" s="14" t="inlineStr"/>
+      <c r="F102" s="14" t="inlineStr"/>
+      <c r="G102" s="15" t="inlineStr"/>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="8" t="inlineStr">
@@ -2136,7 +2127,7 @@
           <t>Arşiv Araştırma</t>
         </is>
       </c>
-      <c r="B105" s="15" t="inlineStr">
+      <c r="B105" s="10" t="inlineStr">
         <is>
           <t>287.62TL</t>
         </is>
@@ -2144,8 +2135,8 @@
       <c r="C105" s="11" t="inlineStr"/>
       <c r="D105" s="12" t="inlineStr"/>
       <c r="E105" s="13" t="inlineStr"/>
-      <c r="F105" s="16" t="inlineStr"/>
-      <c r="G105" s="14" t="inlineStr"/>
+      <c r="F105" s="14" t="inlineStr"/>
+      <c r="G105" s="15" t="inlineStr"/>
     </row>
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="8" t="inlineStr">
@@ -2160,20 +2151,20 @@
           <t>Hesap Özeti</t>
         </is>
       </c>
-      <c r="B108" s="15" t="inlineStr"/>
+      <c r="B108" s="10" t="inlineStr"/>
       <c r="C108" s="11" t="inlineStr"/>
-      <c r="D108" s="10" t="inlineStr">
+      <c r="D108" s="12" t="inlineStr">
         <is>
           <t>190TL</t>
         </is>
       </c>
       <c r="E108" s="13" t="inlineStr"/>
-      <c r="F108" s="10" t="inlineStr">
+      <c r="F108" s="14" t="inlineStr">
         <is>
           <t>12 TL</t>
         </is>
       </c>
-      <c r="G108" s="14" t="inlineStr"/>
+      <c r="G108" s="15" t="inlineStr"/>
     </row>
     <row r="110" ht="18" customHeight="1">
       <c r="A110" s="8" t="inlineStr">
@@ -2194,7 +2185,7 @@
         </is>
       </c>
       <c r="C111" s="11" t="inlineStr"/>
-      <c r="D111" s="10" t="inlineStr">
+      <c r="D111" s="12" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
@@ -2204,17 +2195,17 @@
           <t>550TL</t>
         </is>
       </c>
-      <c r="F111" s="10" t="inlineStr">
+      <c r="F111" s="14" t="inlineStr">
         <is>
           <t>500 TL</t>
         </is>
       </c>
-      <c r="G111" s="14" t="inlineStr"/>
+      <c r="G111" s="15" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="17" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 14.08.2026 16:24</t>
+      <c r="A113" s="16" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 14.08.2026 17:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 17:20)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -653,7 +653,7 @@
       <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>4.25 %</t>
+          <t xml:space="preserve">4.25 </t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>1.00TL / 1.00%</t>
+          <t>1.00TL / 1.00</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr"/>
@@ -873,268 +873,302 @@
       <c r="F11" s="14" t="inlineStr"/>
       <c r="G11" s="15" t="inlineStr"/>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Havale Gönderimi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Düzenli Havale - 0-8300 TRY</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>3.99TL</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr"/>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>3,99TL</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>3,99TL</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>3,99 TL</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>3,99 TL</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Düzenli Havale - 0-8300 TRY</t>
+          <t>Düzenli Havale - 8300-399000 TRY</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>3.99TL</t>
+          <t>7.98TL</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr"/>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>3,99TL</t>
+          <t>7,98TL</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>3,99TL</t>
+          <t>7,98TL</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>3,99 TL</t>
+          <t>7,98 TL</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>3,99 TL</t>
+          <t>7,98 TL</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Düzenli Havale - 8300-399000 TRY</t>
+          <t>Düzenli Havale - 399000+ TRY</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>7.98TL</t>
+          <t>99.71TL</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr"/>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>7,98TL</t>
+          <t>99,71TL</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>7,98TL</t>
+          <t>99,71TL</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>7,98 TL</t>
+          <t>99,71 TL</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>7,98 TL</t>
+          <t>99,71 TL</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Düzenli Havale - 399000+ TRY</t>
+          <t>Havale - 0-8300 TRY</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>99.71TL</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr"/>
+          <t>1050.00TL</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>2485.72TL</t>
+        </is>
+      </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>99,71TL</t>
+          <t>3,99TL</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>99,71TL</t>
+          <t>19,94TL</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>99,71 TL</t>
+          <t>152.380,96 TL</t>
         </is>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>99,71 TL</t>
+          <t>19,94 TL</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Havale - 0-8300 TRY</t>
+          <t>Havale - 8300-399000 TRY</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>1050.00TL</t>
+          <t>1500.00TL</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>2485.72TL</t>
+          <t>2923.81TL</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>3,99TL</t>
+          <t>7,98TL</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>19,94TL</t>
+          <t>39,88TL</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>152.380,96 TL</t>
+          <t>309.523,81 TL</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>19,94 TL</t>
+          <t>39,88 TL</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Havale - 8300-399000 TRY</t>
+          <t>Havale - 399000+ TRY</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>1500.00TL</t>
+          <t>1900.00TL / 0.70</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>2923.81TL</t>
+          <t>3676.20TL / 0.70</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>7,98TL</t>
+          <t>99,71TL</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>39,88TL</t>
+          <t>398,84TL</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>309.523,81 TL</t>
+          <t>199,42</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>39,88 TL</t>
+          <t>398,84 TL</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Havale - 399000+ TRY</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>1900.00TL / 0.70%</t>
-        </is>
-      </c>
+          <t>Havale Gönderimi</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr"/>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>3676.20TL / 0.70%</t>
+          <t>1038.10TL / 0.58</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>99,71TL</t>
+          <t>150TL</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>398,84TL</t>
+          <t>125TL</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>199,42</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>398,84 TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>Havale Gönderimi</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr"/>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>1038.10TL / 0.58%</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>150TL</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>125TL</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>1.300 TL / 0,6 %</t>
-        </is>
-      </c>
-      <c r="G20" s="15" t="inlineStr"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+          <t xml:space="preserve">1.300 TL / 0,6 </t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>FAST</t>
         </is>
       </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>FAST - 0-8300 TRY</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>7.97TL</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr"/>
+      <c r="D21" s="12" t="inlineStr"/>
+      <c r="E21" s="13" t="inlineStr"/>
+      <c r="F21" s="14" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>FAST - 399000+ TRY</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>380.95TL / 0.48</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr"/>
+      <c r="D22" s="12" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr"/>
+      <c r="F22" s="14" t="inlineStr"/>
+      <c r="G22" s="15" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>FAST - 0-8300 TRY</t>
+          <t>FAST - 8300-399000 TRY</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>7.97TL</t>
+          <t>15.96TL</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr"/>
@@ -1143,242 +1177,301 @@
       <c r="F23" s="14" t="inlineStr"/>
       <c r="G23" s="15" t="inlineStr"/>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>FAST - 399000+ TRY</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>380.95TL / 0.48%</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr"/>
-      <c r="D24" s="12" t="inlineStr"/>
-      <c r="E24" s="13" t="inlineStr"/>
-      <c r="F24" s="14" t="inlineStr"/>
-      <c r="G24" s="15" t="inlineStr"/>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Uluslararası Transfer</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>FAST - 8300-399000 TRY</t>
+          <t>Uluslararası Transfer</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>15.96TL</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr"/>
-      <c r="D25" s="12" t="inlineStr"/>
-      <c r="E25" s="13" t="inlineStr"/>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>2355TL</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>3270TL / 0,7</t>
+        </is>
+      </c>
       <c r="F25" s="14" t="inlineStr"/>
       <c r="G25" s="15" t="inlineStr"/>
     </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Uluslararası Transfer - 0-8300</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr"/>
+      <c r="C26" s="11" t="inlineStr"/>
+      <c r="D26" s="12" t="inlineStr"/>
+      <c r="E26" s="13" t="inlineStr"/>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>919.047,62 TL</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr"/>
+    </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Uluslararası Transfer</t>
+          <t>Kıymetli Maden</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Uluslararası Transfer</t>
+          <t>Altın Transfer - 0-8300</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>50.00TL</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr"/>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>2355TL</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>3270TL / 0,7%</t>
-        </is>
-      </c>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr"/>
       <c r="F28" s="14" t="inlineStr"/>
       <c r="G28" s="15" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Uluslararası Transfer - 0-8300</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr"/>
+          <t>Altın Transfer - 8300-399000</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>100.00TL</t>
+        </is>
+      </c>
       <c r="C29" s="11" t="inlineStr"/>
-      <c r="D29" s="12" t="inlineStr"/>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>170TL</t>
+        </is>
+      </c>
       <c r="E29" s="13" t="inlineStr"/>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>919.047,62 TL</t>
-        </is>
-      </c>
+      <c r="F29" s="14" t="inlineStr"/>
       <c r="G29" s="15" t="inlineStr"/>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Kıymetli Maden</t>
-        </is>
-      </c>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Altın Transfer</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr"/>
+      <c r="C30" s="11" t="inlineStr"/>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr"/>
+      <c r="F30" s="14" t="inlineStr"/>
+      <c r="G30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Altın Transfer - 1-10gr</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr"/>
+      <c r="C31" s="11" t="inlineStr"/>
+      <c r="D31" s="12" t="inlineStr"/>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>57,5TL</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>60 TL</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Altın Transfer - 0-8300</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>50.00TL</t>
-        </is>
-      </c>
+          <t>Altın Transfer - 11-100gr</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr"/>
       <c r="C32" s="11" t="inlineStr"/>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>3.25%</t>
-        </is>
-      </c>
-      <c r="E32" s="13" t="inlineStr"/>
-      <c r="F32" s="14" t="inlineStr"/>
+      <c r="D32" s="12" t="inlineStr"/>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>115TL</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>120 TL</t>
+        </is>
+      </c>
       <c r="G32" s="15" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Altın Transfer - 8300-399000</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>100.00TL</t>
-        </is>
-      </c>
+          <t>Altın Transfer - 399000+</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr"/>
       <c r="C33" s="11" t="inlineStr"/>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>170TL</t>
+          <t>415TL</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr"/>
-      <c r="F33" s="14" t="inlineStr"/>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>0.00018</t>
+        </is>
+      </c>
       <c r="G33" s="15" t="inlineStr"/>
     </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Altın Transfer</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="inlineStr"/>
-      <c r="C34" s="11" t="inlineStr"/>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="E34" s="13" t="inlineStr"/>
-      <c r="F34" s="14" t="inlineStr"/>
-      <c r="G34" s="15" t="inlineStr"/>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Kiralık Kasa</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Altın Transfer - 1-10gr</t>
-        </is>
-      </c>
-      <c r="B35" s="10" t="inlineStr"/>
+          <t>Yıllık Kasa Ücreti - büyük</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>30000.00TL</t>
+        </is>
+      </c>
       <c r="C35" s="11" t="inlineStr"/>
-      <c r="D35" s="12" t="inlineStr"/>
-      <c r="E35" s="13" t="inlineStr">
-        <is>
-          <t>57,5TL</t>
-        </is>
-      </c>
-      <c r="F35" s="14" t="inlineStr">
-        <is>
-          <t>60 TL</t>
-        </is>
-      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>4140TL</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr"/>
+      <c r="F35" s="14" t="inlineStr"/>
       <c r="G35" s="15" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Altın Transfer - 11-100gr</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr"/>
+          <t>Yıllık Kasa Ücreti - küçük</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>22000.00TL</t>
+        </is>
+      </c>
       <c r="C36" s="11" t="inlineStr"/>
-      <c r="D36" s="12" t="inlineStr"/>
-      <c r="E36" s="13" t="inlineStr">
-        <is>
-          <t>115TL</t>
-        </is>
-      </c>
-      <c r="F36" s="14" t="inlineStr">
-        <is>
-          <t>120 TL</t>
-        </is>
-      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>2610TL</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr"/>
+      <c r="F36" s="14" t="inlineStr"/>
       <c r="G36" s="15" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>Altın Transfer - 399000+</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr"/>
+          <t>Yıllık Kasa Ücreti - orta</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>25000.00TL</t>
+        </is>
+      </c>
       <c r="C37" s="11" t="inlineStr"/>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>415TL</t>
+          <t>3390TL</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr"/>
-      <c r="F37" s="14" t="inlineStr">
-        <is>
-          <t>0.00018</t>
-        </is>
-      </c>
+      <c r="F37" s="14" t="inlineStr"/>
       <c r="G37" s="15" t="inlineStr"/>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>Kiralık Kasa</t>
-        </is>
-      </c>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Kasa Depozito - büyük</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>28570.00TL</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr"/>
+      <c r="D38" s="12" t="inlineStr"/>
+      <c r="E38" s="13" t="inlineStr"/>
+      <c r="F38" s="14" t="inlineStr"/>
+      <c r="G38" s="15" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Kasa Depozito - orta</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>23805.00TL</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr"/>
+      <c r="D39" s="12" t="inlineStr"/>
+      <c r="E39" s="13" t="inlineStr"/>
+      <c r="F39" s="14" t="inlineStr"/>
+      <c r="G39" s="15" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - büyük</t>
+          <t>Kasa Depozito - küçük</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>30000.00TL</t>
+          <t>20950.00TL</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr"/>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t>4140TL</t>
-        </is>
-      </c>
+      <c r="D40" s="12" t="inlineStr"/>
       <c r="E40" s="13" t="inlineStr"/>
       <c r="F40" s="14" t="inlineStr"/>
       <c r="G40" s="15" t="inlineStr"/>
@@ -1386,20 +1479,16 @@
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - küçük</t>
+          <t>Yıllık Kasa Ücreti - genel</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>22000.00TL</t>
+          <t>1469.52TL</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr"/>
-      <c r="D41" s="12" t="inlineStr">
-        <is>
-          <t>2610TL</t>
-        </is>
-      </c>
+      <c r="D41" s="12" t="inlineStr"/>
       <c r="E41" s="13" t="inlineStr"/>
       <c r="F41" s="14" t="inlineStr"/>
       <c r="G41" s="15" t="inlineStr"/>
@@ -1407,805 +1496,716 @@
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - orta</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>25000.00TL</t>
-        </is>
-      </c>
+          <t>Kasa Depozito - genel</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr"/>
       <c r="C42" s="11" t="inlineStr"/>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>3390TL</t>
+          <t>9420TL</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr"/>
       <c r="F42" s="14" t="inlineStr"/>
       <c r="G42" s="15" t="inlineStr"/>
     </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
-        <is>
-          <t>Kasa Depozito - büyük</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>28570.00TL</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr"/>
-      <c r="D43" s="12" t="inlineStr"/>
-      <c r="E43" s="13" t="inlineStr"/>
-      <c r="F43" s="14" t="inlineStr"/>
-      <c r="G43" s="15" t="inlineStr"/>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>HGS Etiket Bedeli</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>Kasa Depozito - orta</t>
+          <t>HGS Etiket Bedeli</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>23805.00TL</t>
+          <t>275.00TL</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr"/>
-      <c r="D44" s="12" t="inlineStr"/>
-      <c r="E44" s="13" t="inlineStr"/>
-      <c r="F44" s="14" t="inlineStr"/>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>275TL</t>
+        </is>
+      </c>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>275TL</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>275 TL</t>
+        </is>
+      </c>
       <c r="G44" s="15" t="inlineStr"/>
     </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>Kasa Depozito - küçük</t>
-        </is>
-      </c>
-      <c r="B45" s="10" t="inlineStr">
-        <is>
-          <t>20950.00TL</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr"/>
-      <c r="D45" s="12" t="inlineStr"/>
-      <c r="E45" s="13" t="inlineStr"/>
-      <c r="F45" s="14" t="inlineStr"/>
-      <c r="G45" s="15" t="inlineStr"/>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>Yıllık Kasa Ücreti - genel</t>
+          <t>Çek Düzenleme -</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>1469.52TL</t>
+          <t>9.52TL / 0.10</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr"/>
-      <c r="D46" s="12" t="inlineStr"/>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>290TL / 1.10</t>
+        </is>
+      </c>
       <c r="E46" s="13" t="inlineStr"/>
-      <c r="F46" s="14" t="inlineStr"/>
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>761,90 TL</t>
+        </is>
+      </c>
       <c r="G46" s="15" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>Kasa Depozito - genel</t>
+          <t>Çek Defteri (Yaprak Başı) -</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr"/>
       <c r="C47" s="11" t="inlineStr"/>
-      <c r="D47" s="12" t="inlineStr">
-        <is>
-          <t>9420TL</t>
-        </is>
-      </c>
+      <c r="D47" s="12" t="inlineStr"/>
       <c r="E47" s="13" t="inlineStr"/>
-      <c r="F47" s="14" t="inlineStr"/>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>2.380,95 TL</t>
+        </is>
+      </c>
       <c r="G47" s="15" t="inlineStr"/>
     </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>HGS Etiket Bedeli</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>HGS Etiket Bedeli</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>275.00TL</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr"/>
-      <c r="D50" s="12" t="inlineStr">
-        <is>
-          <t>275TL</t>
-        </is>
-      </c>
-      <c r="E50" s="13" t="inlineStr">
-        <is>
-          <t>275TL</t>
-        </is>
-      </c>
-      <c r="F50" s="14" t="inlineStr">
-        <is>
-          <t>275 TL</t>
-        </is>
-      </c>
-      <c r="G50" s="15" t="inlineStr"/>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t>Çek Defteri ve Çek Düzenleme Ücreti</t>
-        </is>
-      </c>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Çek İade Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>Çek İade Ücreti</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>171.43TL</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr"/>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>390TL</t>
+        </is>
+      </c>
+      <c r="E49" s="13" t="inlineStr"/>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>380,95 TL</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="inlineStr"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>Çek Tahsilat Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>Çek Tahsilat</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>11.99</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>95.24TL</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>0TL</t>
+        </is>
+      </c>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>780TL / 0.6</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>41.904,77 TL</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>95,24 TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>Aynı Banka Çeki -</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr"/>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>438.10TL</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr"/>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>390TL / 0.2</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr"/>
+      <c r="G52" s="15" t="inlineStr"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>Çek Düzenleme -</t>
+          <t>Diğer Banka Çeki -</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>9.52TL / 0.10%</t>
-        </is>
-      </c>
-      <c r="C53" s="11" t="inlineStr"/>
+          <t>390.48TL</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>590.48TL / 0.77</t>
+        </is>
+      </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>290TL / 1.10%</t>
+          <t>350TL</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr"/>
-      <c r="F53" s="14" t="inlineStr">
-        <is>
-          <t>761,90 TL</t>
-        </is>
-      </c>
+      <c r="F53" s="14" t="inlineStr"/>
       <c r="G53" s="15" t="inlineStr"/>
     </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>Çek Defteri (Yaprak Başı) -</t>
-        </is>
-      </c>
-      <c r="B54" s="10" t="inlineStr"/>
-      <c r="C54" s="11" t="inlineStr"/>
-      <c r="D54" s="12" t="inlineStr"/>
-      <c r="E54" s="13" t="inlineStr"/>
-      <c r="F54" s="14" t="inlineStr">
-        <is>
-          <t>2.380,95 TL</t>
-        </is>
-      </c>
-      <c r="G54" s="15" t="inlineStr"/>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>Senet İade Ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>Senet İade Ücreti</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>495.24TL</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr"/>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>780TL</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr"/>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>55.333,33 TL</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr"/>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>Çek İade Ücreti</t>
+          <t>Senet Protesto İşlemleri Ücreti</t>
         </is>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>Çek İade Ücreti</t>
+          <t>Senet Protesto Kaldırma -</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>171.43TL</t>
+          <t>533.34TL</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr"/>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>390TL</t>
+          <t>780TL</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr"/>
       <c r="F57" s="14" t="inlineStr">
         <is>
-          <t>380,95 TL</t>
+          <t>619,05 TL</t>
         </is>
       </c>
       <c r="G57" s="15" t="inlineStr"/>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>Senet Protesto -</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>600.00TL</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr"/>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>780TL</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="inlineStr"/>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
+          <t>666,67 TL</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="inlineStr"/>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>Çek Tahsilat Ücreti</t>
+          <t>Senet Tahsile Alma Ücreti</t>
         </is>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>Çek Tahsilat</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>11.99%</t>
-        </is>
-      </c>
+          <t>Senet Tahsile Alma -</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr"/>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>95.24TL</t>
-        </is>
-      </c>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>0TL</t>
-        </is>
-      </c>
-      <c r="E60" s="13" t="inlineStr">
-        <is>
-          <t>780TL / 0.6%</t>
-        </is>
-      </c>
+          <t>600.00TL</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr"/>
+      <c r="E60" s="13" t="inlineStr"/>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>41.904,77 TL</t>
-        </is>
-      </c>
-      <c r="G60" s="15" t="inlineStr">
-        <is>
-          <t>95,24 TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="9" t="inlineStr">
-        <is>
-          <t>Aynı Banka Çeki -</t>
-        </is>
-      </c>
-      <c r="B61" s="10" t="inlineStr"/>
-      <c r="C61" s="11" t="inlineStr">
-        <is>
-          <t>438.10TL</t>
-        </is>
-      </c>
-      <c r="D61" s="12" t="inlineStr"/>
-      <c r="E61" s="13" t="inlineStr">
-        <is>
-          <t>390TL / 0.2%</t>
-        </is>
-      </c>
-      <c r="F61" s="14" t="inlineStr"/>
-      <c r="G61" s="15" t="inlineStr"/>
+          <t>666,67 TL</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="inlineStr"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>Fatura Ödemeleri</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>Diğer Banka Çeki -</t>
+          <t>Fatura Ödemeleri</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>390.48TL</t>
+          <t>5.00TL / 3.50</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>590.48TL / 0.77%</t>
+          <t>0.00TL</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>350TL</t>
-        </is>
-      </c>
-      <c r="E62" s="13" t="inlineStr"/>
-      <c r="F62" s="14" t="inlineStr"/>
-      <c r="G62" s="15" t="inlineStr"/>
-    </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="8" t="inlineStr">
-        <is>
-          <t>Senet İade Ücreti</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="9" t="inlineStr">
-        <is>
-          <t>Senet İade Ücreti</t>
-        </is>
-      </c>
-      <c r="B65" s="10" t="inlineStr">
-        <is>
-          <t>495.24TL</t>
-        </is>
-      </c>
-      <c r="C65" s="11" t="inlineStr"/>
-      <c r="D65" s="12" t="inlineStr">
-        <is>
-          <t>780TL</t>
-        </is>
-      </c>
-      <c r="E65" s="13" t="inlineStr"/>
-      <c r="F65" s="14" t="inlineStr">
-        <is>
-          <t>55.333,33 TL</t>
-        </is>
-      </c>
-      <c r="G65" s="15" t="inlineStr"/>
+          <t>0TL</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>0TL</t>
+        </is>
+      </c>
+      <c r="F62" s="14" t="inlineStr">
+        <is>
+          <t>0.5 TL</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>0.5 TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>SGK Prim Ödemeleri</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>SGK Prim Ödemeleri</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>3.50TL / 3.50</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr"/>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>0TL</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr"/>
+      <c r="F64" s="14" t="inlineStr">
+        <is>
+          <t>2 TL / 3,5</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr"/>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>Vergi Tahsilat</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>Vergi Tahsilat</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="inlineStr"/>
+      <c r="C66" s="11" t="inlineStr"/>
+      <c r="D66" s="12" t="inlineStr"/>
+      <c r="E66" s="13" t="inlineStr"/>
+      <c r="F66" s="14" t="inlineStr"/>
+      <c r="G66" s="15" t="inlineStr"/>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>Senet Protesto İşlemleri Ücreti</t>
+          <t>Şans Oyunu Ödemeleri</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>Senet Protesto Kaldırma -</t>
-        </is>
-      </c>
-      <c r="B68" s="10" t="inlineStr">
-        <is>
-          <t>533.34TL</t>
-        </is>
-      </c>
+          <t>Şans Oyunu Ödemeleri</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr"/>
       <c r="C68" s="11" t="inlineStr"/>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>780TL</t>
+          <t>26TL</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr"/>
       <c r="F68" s="14" t="inlineStr">
         <is>
-          <t>619,05 TL</t>
+          <t>38,10 TL</t>
         </is>
       </c>
       <c r="G68" s="15" t="inlineStr"/>
     </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="9" t="inlineStr">
-        <is>
-          <t>Senet Protesto -</t>
-        </is>
-      </c>
-      <c r="B69" s="10" t="inlineStr">
-        <is>
-          <t>600.00TL</t>
-        </is>
-      </c>
-      <c r="C69" s="11" t="inlineStr"/>
-      <c r="D69" s="12" t="inlineStr">
-        <is>
-          <t>780TL</t>
-        </is>
-      </c>
-      <c r="E69" s="13" t="inlineStr"/>
-      <c r="F69" s="14" t="inlineStr">
-        <is>
-          <t>666,67 TL</t>
-        </is>
-      </c>
-      <c r="G69" s="15" t="inlineStr"/>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>Telefon Ödemeleri</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>Telefon Ödemeleri</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr"/>
+      <c r="C70" s="11" t="inlineStr"/>
+      <c r="D70" s="12" t="inlineStr"/>
+      <c r="E70" s="13" t="inlineStr"/>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 </t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="inlineStr"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>Senet Tahsile Alma Ücreti</t>
+          <t>Özel Okul Ödeme</t>
         </is>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>Senet Tahsile Alma -</t>
+          <t>Özel Okul Ödeme</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr"/>
-      <c r="C72" s="11" t="inlineStr">
-        <is>
-          <t>600.00TL</t>
-        </is>
-      </c>
-      <c r="D72" s="12" t="inlineStr"/>
+      <c r="C72" s="11" t="inlineStr"/>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t>390TL</t>
+        </is>
+      </c>
       <c r="E72" s="13" t="inlineStr"/>
-      <c r="F72" s="14" t="inlineStr">
-        <is>
-          <t>666,67 TL</t>
-        </is>
-      </c>
+      <c r="F72" s="14" t="inlineStr"/>
       <c r="G72" s="15" t="inlineStr"/>
     </row>
-    <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>Fatura Ödemeleri</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="9" t="inlineStr">
-        <is>
-          <t>Fatura Ödemeleri</t>
-        </is>
-      </c>
-      <c r="B75" s="10" t="inlineStr">
-        <is>
-          <t>5.00TL / 3.50%</t>
-        </is>
-      </c>
-      <c r="C75" s="11" t="inlineStr">
-        <is>
-          <t>0.00TL</t>
-        </is>
-      </c>
-      <c r="D75" s="12" t="inlineStr">
-        <is>
-          <t>0TL</t>
-        </is>
-      </c>
-      <c r="E75" s="13" t="inlineStr">
-        <is>
-          <t>0TL</t>
-        </is>
-      </c>
-      <c r="F75" s="14" t="inlineStr">
-        <is>
-          <t>0.5 TL</t>
-        </is>
-      </c>
-      <c r="G75" s="15" t="inlineStr">
-        <is>
-          <t>0.5 TL</t>
-        </is>
-      </c>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>Bakiye Sorma - Yurtiçi - ATM</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>Bakiye Sorma - Yurtiçi - ATM</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr"/>
+      <c r="C74" s="11" t="inlineStr"/>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t>0.41TL</t>
+        </is>
+      </c>
+      <c r="E74" s="13" t="inlineStr"/>
+      <c r="F74" s="14" t="inlineStr"/>
+      <c r="G74" s="15" t="inlineStr"/>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>Bakiye Sorma - Yurtdışı - ATM</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>Bakiye Sorma - Yurtdışı - ATM</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr"/>
+      <c r="C76" s="11" t="inlineStr"/>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>0.45EUR</t>
+        </is>
+      </c>
+      <c r="E76" s="13" t="inlineStr"/>
+      <c r="F76" s="14" t="inlineStr">
+        <is>
+          <t>0.27 TL</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr"/>
     </row>
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>SGK Prim Ödemeleri</t>
+          <t>Kredi Risk Raporu</t>
         </is>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>SGK Prim Ödemeleri</t>
-        </is>
-      </c>
-      <c r="B78" s="10" t="inlineStr">
-        <is>
-          <t>3.50TL / 3.50%</t>
-        </is>
-      </c>
+          <t>Kredi Risk Raporu</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="inlineStr"/>
       <c r="C78" s="11" t="inlineStr"/>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>0TL</t>
+          <t>95TL</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr"/>
       <c r="F78" s="14" t="inlineStr">
         <is>
-          <t>2 TL / 3,5%</t>
+          <t>65 TL</t>
         </is>
       </c>
       <c r="G78" s="15" t="inlineStr"/>
     </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="8" t="inlineStr">
-        <is>
-          <t>Vergi Tahsilat</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="9" t="inlineStr">
-        <is>
-          <t>Vergi Tahsilat</t>
-        </is>
-      </c>
-      <c r="B81" s="10" t="inlineStr"/>
-      <c r="C81" s="11" t="inlineStr"/>
-      <c r="D81" s="12" t="inlineStr"/>
-      <c r="E81" s="13" t="inlineStr"/>
-      <c r="F81" s="14" t="inlineStr"/>
-      <c r="G81" s="15" t="inlineStr"/>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>Referans Mektubu</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>Referans Mektubu</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>4000.00TL</t>
+        </is>
+      </c>
+      <c r="C80" s="11" t="inlineStr"/>
+      <c r="D80" s="12" t="inlineStr">
+        <is>
+          <t>770TL</t>
+        </is>
+      </c>
+      <c r="E80" s="13" t="inlineStr"/>
+      <c r="F80" s="14" t="inlineStr"/>
+      <c r="G80" s="15" t="inlineStr"/>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>Arşiv Araştırma</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>Arşiv Araştırma</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>287.62TL</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="inlineStr"/>
+      <c r="D82" s="12" t="inlineStr"/>
+      <c r="E82" s="13" t="inlineStr"/>
+      <c r="F82" s="14" t="inlineStr"/>
+      <c r="G82" s="15" t="inlineStr"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>Şans Oyunu Ödemeleri</t>
+          <t>Hesap Özeti</t>
         </is>
       </c>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>Şans Oyunu Ödemeleri</t>
+          <t>Hesap Özeti</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr"/>
       <c r="C84" s="11" t="inlineStr"/>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>26TL</t>
+          <t>190TL</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr"/>
       <c r="F84" s="14" t="inlineStr">
         <is>
-          <t>38,10 TL</t>
+          <t>12 TL</t>
         </is>
       </c>
       <c r="G84" s="15" t="inlineStr"/>
     </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="8" t="inlineStr">
-        <is>
-          <t>Telefon Ödemeleri</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="9" t="inlineStr">
-        <is>
-          <t>Telefon Ödemeleri</t>
-        </is>
-      </c>
-      <c r="B87" s="10" t="inlineStr"/>
-      <c r="C87" s="11" t="inlineStr"/>
-      <c r="D87" s="12" t="inlineStr"/>
-      <c r="E87" s="13" t="inlineStr"/>
-      <c r="F87" s="14" t="inlineStr">
-        <is>
-          <t>1 %</t>
-        </is>
-      </c>
-      <c r="G87" s="15" t="inlineStr"/>
-    </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="8" t="inlineStr">
-        <is>
-          <t>Özel Okul Ödeme</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="20" customHeight="1">
-      <c r="A90" s="9" t="inlineStr">
-        <is>
-          <t>Özel Okul Ödeme</t>
-        </is>
-      </c>
-      <c r="B90" s="10" t="inlineStr"/>
-      <c r="C90" s="11" t="inlineStr"/>
-      <c r="D90" s="12" t="inlineStr">
-        <is>
-          <t>390TL</t>
-        </is>
-      </c>
-      <c r="E90" s="13" t="inlineStr"/>
-      <c r="F90" s="14" t="inlineStr"/>
-      <c r="G90" s="15" t="inlineStr"/>
-    </row>
-    <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="8" t="inlineStr">
-        <is>
-          <t>Bakiye Sorma - Yurtiçi - ATM</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="20" customHeight="1">
-      <c r="A93" s="9" t="inlineStr">
-        <is>
-          <t>Bakiye Sorma - Yurtiçi - ATM</t>
-        </is>
-      </c>
-      <c r="B93" s="10" t="inlineStr"/>
-      <c r="C93" s="11" t="inlineStr"/>
-      <c r="D93" s="12" t="inlineStr">
-        <is>
-          <t>0.41TL</t>
-        </is>
-      </c>
-      <c r="E93" s="13" t="inlineStr"/>
-      <c r="F93" s="14" t="inlineStr"/>
-      <c r="G93" s="15" t="inlineStr"/>
-    </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="8" t="inlineStr">
-        <is>
-          <t>Bakiye Sorma - Yurtdışı - ATM</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="9" t="inlineStr">
-        <is>
-          <t>Bakiye Sorma - Yurtdışı - ATM</t>
-        </is>
-      </c>
-      <c r="B96" s="10" t="inlineStr"/>
-      <c r="C96" s="11" t="inlineStr"/>
-      <c r="D96" s="12" t="inlineStr">
-        <is>
-          <t>0.45EUR</t>
-        </is>
-      </c>
-      <c r="E96" s="13" t="inlineStr"/>
-      <c r="F96" s="14" t="inlineStr">
-        <is>
-          <t>0.27 TL</t>
-        </is>
-      </c>
-      <c r="G96" s="15" t="inlineStr"/>
-    </row>
-    <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="8" t="inlineStr">
-        <is>
-          <t>Kredi Risk Raporu</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="9" t="inlineStr">
-        <is>
-          <t>Kredi Risk Raporu</t>
-        </is>
-      </c>
-      <c r="B99" s="10" t="inlineStr"/>
-      <c r="C99" s="11" t="inlineStr"/>
-      <c r="D99" s="12" t="inlineStr">
-        <is>
-          <t>95TL</t>
-        </is>
-      </c>
-      <c r="E99" s="13" t="inlineStr"/>
-      <c r="F99" s="14" t="inlineStr">
-        <is>
-          <t>65 TL</t>
-        </is>
-      </c>
-      <c r="G99" s="15" t="inlineStr"/>
-    </row>
-    <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="8" t="inlineStr">
-        <is>
-          <t>Referans Mektubu</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="20" customHeight="1">
-      <c r="A102" s="9" t="inlineStr">
-        <is>
-          <t>Referans Mektubu</t>
-        </is>
-      </c>
-      <c r="B102" s="10" t="inlineStr">
-        <is>
-          <t>4000.00TL</t>
-        </is>
-      </c>
-      <c r="C102" s="11" t="inlineStr"/>
-      <c r="D102" s="12" t="inlineStr">
-        <is>
-          <t>770TL</t>
-        </is>
-      </c>
-      <c r="E102" s="13" t="inlineStr"/>
-      <c r="F102" s="14" t="inlineStr"/>
-      <c r="G102" s="15" t="inlineStr"/>
-    </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="8" t="inlineStr">
-        <is>
-          <t>Arşiv Araştırma</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="20" customHeight="1">
-      <c r="A105" s="9" t="inlineStr">
-        <is>
-          <t>Arşiv Araştırma</t>
-        </is>
-      </c>
-      <c r="B105" s="10" t="inlineStr">
-        <is>
-          <t>287.62TL</t>
-        </is>
-      </c>
-      <c r="C105" s="11" t="inlineStr"/>
-      <c r="D105" s="12" t="inlineStr"/>
-      <c r="E105" s="13" t="inlineStr"/>
-      <c r="F105" s="14" t="inlineStr"/>
-      <c r="G105" s="15" t="inlineStr"/>
-    </row>
-    <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="8" t="inlineStr">
-        <is>
-          <t>Hesap Özeti</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="9" t="inlineStr">
-        <is>
-          <t>Hesap Özeti</t>
-        </is>
-      </c>
-      <c r="B108" s="10" t="inlineStr"/>
-      <c r="C108" s="11" t="inlineStr"/>
-      <c r="D108" s="12" t="inlineStr">
-        <is>
-          <t>190TL</t>
-        </is>
-      </c>
-      <c r="E108" s="13" t="inlineStr"/>
-      <c r="F108" s="14" t="inlineStr">
-        <is>
-          <t>12 TL</t>
-        </is>
-      </c>
-      <c r="G108" s="15" t="inlineStr"/>
-    </row>
-    <row r="110" ht="18" customHeight="1">
-      <c r="A110" s="8" t="inlineStr">
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="8" t="inlineStr">
         <is>
           <t>HGS</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="20" customHeight="1">
-      <c r="A111" s="9" t="inlineStr">
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
         <is>
           <t>HGS Kart Ücreti</t>
         </is>
       </c>
-      <c r="B111" s="10" t="inlineStr">
+      <c r="B86" s="10" t="inlineStr">
         <is>
           <t>550.00TL</t>
         </is>
       </c>
-      <c r="C111" s="11" t="inlineStr"/>
-      <c r="D111" s="12" t="inlineStr">
+      <c r="C86" s="11" t="inlineStr"/>
+      <c r="D86" s="12" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="E111" s="13" t="inlineStr">
+      <c r="E86" s="13" t="inlineStr">
         <is>
           <t>550TL</t>
         </is>
       </c>
-      <c r="F111" s="14" t="inlineStr">
+      <c r="F86" s="14" t="inlineStr">
         <is>
           <t>500 TL</t>
         </is>
       </c>
-      <c r="G111" s="15" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="16" t="inlineStr">
-        <is>
-          <t>Son güncelleme: 14.08.2026 17:03</t>
+      <c r="G86" s="15" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="16" t="inlineStr">
+        <is>
+          <t>Son güncelleme: 14.08.2026 17:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (14.08.2026 17:38)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -653,7 +653,7 @@
       <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.25 </t>
+          <t>3,99 TL</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>1.00TL / 1.00</t>
+          <t>1.00TL</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr"/>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>1900.00TL / 0.70</t>
+          <t>1900.00TL</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>3676.20TL / 0.70</t>
+          <t>3676.20TL</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -1099,7 +1099,7 @@
       <c r="B19" s="10" t="inlineStr"/>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>1038.10TL / 0.58</t>
+          <t>1038.10TL</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.300 TL / 0,6 </t>
+          <t>1.300 TL</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr"/>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>380.95TL / 0.48</t>
+          <t>380.95TL</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr"/>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>15.00TL</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr"/>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>3270TL / 0,7</t>
+          <t>3270TL</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr"/>
@@ -1245,11 +1245,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr"/>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>3.25</t>
-        </is>
-      </c>
+      <c r="D28" s="12" t="inlineStr"/>
       <c r="E28" s="13" t="inlineStr"/>
       <c r="F28" s="14" t="inlineStr"/>
       <c r="G28" s="15" t="inlineStr"/>
@@ -1285,7 +1281,7 @@
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0TL</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr"/>
@@ -1348,11 +1344,7 @@
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr"/>
-      <c r="F33" s="14" t="inlineStr">
-        <is>
-          <t>0.00018</t>
-        </is>
-      </c>
+      <c r="F33" s="14" t="inlineStr"/>
       <c r="G33" s="15" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -1561,13 +1553,13 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>9.52TL / 0.10</t>
+          <t>9.52TL</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>290TL / 1.10</t>
+          <t>290TL</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr"/>
@@ -1642,7 +1634,7 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>11.99</t>
+          <t>0.45EUR</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
@@ -1657,7 +1649,7 @@
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>780TL / 0.6</t>
+          <t>780TL</t>
         </is>
       </c>
       <c r="F51" s="14" t="inlineStr">
@@ -1686,7 +1678,7 @@
       <c r="D52" s="12" t="inlineStr"/>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>390TL / 0.2</t>
+          <t>390TL</t>
         </is>
       </c>
       <c r="F52" s="14" t="inlineStr"/>
@@ -1705,7 +1697,7 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>590.48TL / 0.77</t>
+          <t>590.48TL</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
@@ -1849,7 +1841,7 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>5.00TL / 3.50</t>
+          <t>5.00TL</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
@@ -1893,7 +1885,7 @@
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>3.50TL / 3.50</t>
+          <t>3.50TL</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr"/>
@@ -1905,7 +1897,7 @@
       <c r="E64" s="13" t="inlineStr"/>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>2 TL / 3,5</t>
+          <t>2 TL</t>
         </is>
       </c>
       <c r="G64" s="15" t="inlineStr"/>
@@ -1977,7 +1969,7 @@
       <c r="E70" s="13" t="inlineStr"/>
       <c r="F70" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 </t>
+          <t>99,71 TL</t>
         </is>
       </c>
       <c r="G70" s="15" t="inlineStr"/>
@@ -2205,7 +2197,7 @@
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
         <is>
-          <t>Son güncelleme: 14.08.2026 17:20</t>
+          <t>Son güncelleme: 14.08.2026 17:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Komisyon karşılaştırma güncellendi (17.08.2026 09:20)
</commit_message>
<xml_diff>
--- a/komisyon_karsilastirma.xlsx
+++ b/komisyon_karsilastirma.xlsx
@@ -653,7 +653,7 @@
       <c r="E4" s="13" t="inlineStr"/>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>3,99 TL</t>
+          <t>4.25 %</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr"/>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>15.00TL</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr"/>
@@ -1245,7 +1245,11 @@
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr"/>
-      <c r="D28" s="12" t="inlineStr"/>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>3.25%</t>
+        </is>
+      </c>
       <c r="E28" s="13" t="inlineStr"/>
       <c r="F28" s="14" t="inlineStr"/>
       <c r="G28" s="15" t="inlineStr"/>
@@ -1281,7 +1285,7 @@
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>0TL</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr"/>
@@ -1344,7 +1348,11 @@
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr"/>
-      <c r="F33" s="14" t="inlineStr"/>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>0.00018</t>
+        </is>
+      </c>
       <c r="G33" s="15" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -1634,7 +1642,7 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>0.45EUR</t>
+          <t>11.99%</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
@@ -1969,7 +1977,7 @@
       <c r="E70" s="13" t="inlineStr"/>
       <c r="F70" s="14" t="inlineStr">
         <is>
-          <t>99,71 TL</t>
+          <t>1 %</t>
         </is>
       </c>
       <c r="G70" s="15" t="inlineStr"/>
@@ -2197,7 +2205,7 @@
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
         <is>
-          <t>Son güncelleme: 16.08.2026 09:11</t>
+          <t>Son güncelleme: 17.08.2026 09:20</t>
         </is>
       </c>
     </row>

</xml_diff>